<commit_message>
learning pysystemtrade. Extracted Forecast Weights, Instrument Weights, IDM, FDM
</commit_message>
<xml_diff>
--- a/perplexity_examples/etf_turnover_analysis.xlsx
+++ b/perplexity_examples/etf_turnover_analysis.xlsx
@@ -607,31 +607,31 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>36.21304347685363</v>
+        <v>36.21314297445958</v>
       </c>
       <c r="C2">
-        <v>6.958818585934964</v>
+        <v>6.958799466197416</v>
       </c>
       <c r="D2">
-        <v>0.9941169408478521</v>
+        <v>0.9941142094567736</v>
       </c>
       <c r="E2">
-        <v>376.5270198442755</v>
+        <v>376.528993055139</v>
       </c>
       <c r="F2">
-        <v>214700.1242081307</v>
+        <v>214701.8392612503</v>
       </c>
       <c r="G2">
         <v>1984</v>
       </c>
       <c r="H2">
-        <v>0.3621304347685363</v>
+        <v>0.3621314297445958</v>
       </c>
       <c r="I2">
         <v>-123.5074635009766</v>
       </c>
       <c r="J2">
-        <v>0.2932053047674103</v>
+        <v>0.2932061103673564</v>
       </c>
       <c r="K2" t="s">
         <v>43</v>
@@ -645,31 +645,31 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>35.73981517165323</v>
+        <v>35.73983427744304</v>
       </c>
       <c r="C3">
-        <v>7.050959799027499</v>
+        <v>7.05095602972754</v>
       </c>
       <c r="D3">
-        <v>1.007279971289643</v>
+        <v>1.00727943281822</v>
       </c>
       <c r="E3">
-        <v>4706.164473320398</v>
+        <v>4706.176142795722</v>
       </c>
       <c r="F3">
-        <v>2648442.362798742</v>
+        <v>2648450.345723546</v>
       </c>
       <c r="G3">
         <v>1984</v>
       </c>
       <c r="H3">
-        <v>0.3573981517165323</v>
+        <v>0.3573983427744304</v>
       </c>
       <c r="I3">
         <v>93.64753532409668</v>
       </c>
       <c r="J3">
-        <v>0.3816418130809784</v>
+        <v>0.3816420170990526</v>
       </c>
       <c r="K3" t="s">
         <v>43</v>
@@ -683,31 +683,31 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>35.28804328874659</v>
+        <v>35.28818078629894</v>
       </c>
       <c r="C4">
-        <v>7.141229054215177</v>
+        <v>7.14120122899172</v>
       </c>
       <c r="D4">
-        <v>1.020175579173597</v>
+        <v>1.020171604141674</v>
       </c>
       <c r="E4">
-        <v>997.2061034251823</v>
+        <v>997.211981073113</v>
       </c>
       <c r="F4">
-        <v>554094.2306080378</v>
+        <v>554099.6555080692</v>
       </c>
       <c r="G4">
         <v>1984</v>
       </c>
       <c r="H4">
-        <v>0.3528804328874658</v>
+        <v>0.3528818078629894</v>
       </c>
       <c r="I4">
         <v>-92.20262858581543</v>
       </c>
       <c r="J4">
-        <v>0.3827227469540423</v>
+        <v>0.3827242382081905</v>
       </c>
       <c r="K4" t="s">
         <v>43</v>
@@ -721,31 +721,31 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>34.28462471972859</v>
+        <v>34.28474383414597</v>
       </c>
       <c r="C5">
-        <v>7.350233583131224</v>
+        <v>7.350208046443679</v>
       </c>
       <c r="D5">
-        <v>1.050033369018746</v>
+        <v>1.050029720920526</v>
       </c>
       <c r="E5">
-        <v>985.7363264701763</v>
+        <v>985.7482380290448</v>
       </c>
       <c r="F5">
-        <v>532146.590879822</v>
+        <v>532154.8701457183</v>
       </c>
       <c r="G5">
         <v>1984</v>
       </c>
       <c r="H5">
-        <v>0.3428462471972859</v>
+        <v>0.3428474383414597</v>
       </c>
       <c r="I5">
         <v>-198.7971412353516</v>
       </c>
       <c r="J5">
-        <v>0.1724603508213419</v>
+        <v>0.1724609499970476</v>
       </c>
       <c r="K5" t="s">
         <v>43</v>
@@ -759,31 +759,31 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>34.0091585140582</v>
+        <v>34.00927271614375</v>
       </c>
       <c r="C6">
-        <v>7.409768750844923</v>
+        <v>7.409743869070713</v>
       </c>
       <c r="D6">
-        <v>1.058538392977846</v>
+        <v>1.058534838438673</v>
       </c>
       <c r="E6">
-        <v>2744.180033764393</v>
+        <v>2744.198336791616</v>
       </c>
       <c r="F6">
-        <v>1469533.900465581</v>
+        <v>1469548.636605541</v>
       </c>
       <c r="G6">
         <v>1984</v>
       </c>
       <c r="H6">
-        <v>0.340091585140582</v>
+        <v>0.3400927271614375</v>
       </c>
       <c r="I6">
         <v>-282.6376909179788</v>
       </c>
       <c r="J6">
-        <v>0.1203277538943935</v>
+        <v>0.120328157952625</v>
       </c>
       <c r="K6" t="s">
         <v>43</v>
@@ -797,31 +797,31 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>33.25800745346309</v>
+        <v>33.25811346615763</v>
       </c>
       <c r="C7">
-        <v>7.577122602808238</v>
+        <v>7.57709845016997</v>
       </c>
       <c r="D7">
-        <v>1.082446086115463</v>
+        <v>1.082442635738567</v>
       </c>
       <c r="E7">
-        <v>7622.156744288965</v>
+        <v>7622.283821387688</v>
       </c>
       <c r="F7">
-        <v>3991583.5531194</v>
+        <v>3991662.824783263</v>
       </c>
       <c r="G7">
         <v>1984</v>
       </c>
       <c r="H7">
-        <v>0.3325800745346309</v>
+        <v>0.3325811346615763</v>
       </c>
       <c r="I7">
         <v>-288.3928489685059</v>
       </c>
       <c r="J7">
-        <v>0.1153218866987061</v>
+        <v>0.1153222542969143</v>
       </c>
       <c r="K7" t="s">
         <v>43</v>
@@ -835,31 +835,31 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>32.51060693467581</v>
+        <v>32.5107725123483</v>
       </c>
       <c r="C8">
-        <v>7.751316378262284</v>
+        <v>7.751276900734516</v>
       </c>
       <c r="D8">
-        <v>1.107330911180326</v>
+        <v>1.107325271533502</v>
       </c>
       <c r="E8">
-        <v>1504.346321302096</v>
+        <v>1504.363153432152</v>
       </c>
       <c r="F8">
-        <v>770094.5119033994</v>
+        <v>770107.0506529219</v>
       </c>
       <c r="G8">
         <v>1984</v>
       </c>
       <c r="H8">
-        <v>0.3251060693467581</v>
+        <v>0.325107725123483</v>
       </c>
       <c r="I8">
         <v>699.8680000000001</v>
       </c>
       <c r="J8">
-        <v>0.04645248380362555</v>
+        <v>0.04645272038777068</v>
       </c>
       <c r="K8" t="s">
         <v>43</v>
@@ -873,31 +873,31 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>32.23994760388378</v>
+        <v>32.24172325795473</v>
       </c>
       <c r="C9">
-        <v>7.816389874332265</v>
+        <v>7.815959400923961</v>
       </c>
       <c r="D9">
-        <v>1.116627124904609</v>
+        <v>1.116565628703423</v>
       </c>
       <c r="E9">
-        <v>36411.03619253603</v>
+        <v>36411.52575049087</v>
       </c>
       <c r="F9">
-        <v>18484107.61679482</v>
+        <v>18485374.18974669</v>
       </c>
       <c r="G9">
         <v>1984</v>
       </c>
       <c r="H9">
-        <v>0.3223994760388378</v>
+        <v>0.3224172325795473</v>
       </c>
       <c r="I9">
         <v>-201.9405915985107</v>
       </c>
       <c r="J9">
-        <v>0.1596506544260394</v>
+        <v>0.1596594473787434</v>
       </c>
       <c r="K9" t="s">
         <v>43</v>
@@ -911,31 +911,31 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>32.17431964099017</v>
+        <v>32.17454412208342</v>
       </c>
       <c r="C10">
-        <v>7.832333451394923</v>
+        <v>7.832278805375101</v>
       </c>
       <c r="D10">
-        <v>1.118904778770703</v>
+        <v>1.118896972196443</v>
       </c>
       <c r="E10">
-        <v>457.8378238348814</v>
+        <v>457.8427425093408</v>
       </c>
       <c r="F10">
-        <v>213593.9970730829</v>
+        <v>213597.7820377157</v>
       </c>
       <c r="G10">
         <v>1827</v>
       </c>
       <c r="H10">
-        <v>0.3217431964099017</v>
+        <v>0.3217454412208342</v>
       </c>
       <c r="I10">
         <v>19.60169787597656</v>
       </c>
       <c r="J10">
-        <v>1.641404731598397</v>
+        <v>1.641416183723344</v>
       </c>
       <c r="K10" t="s">
         <v>43</v>
@@ -949,31 +949,31 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>31.15324841695801</v>
+        <v>31.15333849933335</v>
       </c>
       <c r="C11">
-        <v>8.089044090272971</v>
+        <v>8.089020700153613</v>
       </c>
       <c r="D11">
-        <v>1.155577727181853</v>
+        <v>1.15557438573623</v>
       </c>
       <c r="E11">
-        <v>2047.355469544509</v>
+        <v>2047.373673141135</v>
       </c>
       <c r="F11">
-        <v>1004309.830987516</v>
+        <v>1004321.664657101</v>
       </c>
       <c r="G11">
         <v>1984</v>
       </c>
       <c r="H11">
-        <v>0.3115324841695801</v>
+        <v>0.3115333849933336</v>
       </c>
       <c r="I11">
         <v>475.9476782226562</v>
       </c>
       <c r="J11">
-        <v>0.06545519569145583</v>
+        <v>0.06545538496094797</v>
       </c>
       <c r="K11" t="s">
         <v>43</v>
@@ -987,31 +987,31 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.6279309184528</v>
+        <v>30.62816309239676</v>
       </c>
       <c r="C12">
-        <v>8.227784001176989</v>
+        <v>8.227721631224998</v>
       </c>
       <c r="D12">
-        <v>1.175397714453856</v>
+        <v>1.175388804460714</v>
       </c>
       <c r="E12">
-        <v>1922.310374030212</v>
+        <v>1922.328235984836</v>
       </c>
       <c r="F12">
-        <v>927069.495633421</v>
+        <v>927085.1375719371</v>
       </c>
       <c r="G12">
         <v>1984</v>
       </c>
       <c r="H12">
-        <v>0.3062793091845281</v>
+        <v>0.3062816309239677</v>
       </c>
       <c r="I12">
         <v>-23.32112231445312</v>
       </c>
       <c r="J12">
-        <v>1.31331290602045</v>
+        <v>1.313322861542352</v>
       </c>
       <c r="K12" t="s">
         <v>43</v>
@@ -1025,31 +1025,31 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.03201167048208</v>
+        <v>30.03209660063617</v>
       </c>
       <c r="C13">
-        <v>8.391046286376023</v>
+        <v>8.391022556668982</v>
       </c>
       <c r="D13">
-        <v>1.198720898053718</v>
+        <v>1.198717508095569</v>
       </c>
       <c r="E13">
-        <v>1919.039028591655</v>
+        <v>1919.059339413511</v>
       </c>
       <c r="F13">
-        <v>907484.7886151266</v>
+        <v>907496.9596811212</v>
       </c>
       <c r="G13">
         <v>1984</v>
       </c>
       <c r="H13">
-        <v>0.3003201167048208</v>
+        <v>0.3003209660063617</v>
       </c>
       <c r="I13">
         <v>-79.87465667724609</v>
       </c>
       <c r="J13">
-        <v>0.3759892426434341</v>
+        <v>0.3759903059363186</v>
       </c>
       <c r="K13" t="s">
         <v>43</v>
@@ -1063,31 +1063,31 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.86684914392284</v>
+        <v>29.86701921753074</v>
       </c>
       <c r="C14">
-        <v>8.437448449471804</v>
+        <v>8.437400403589191</v>
       </c>
       <c r="D14">
-        <v>1.205349778495972</v>
+        <v>1.205342914798456</v>
       </c>
       <c r="E14">
-        <v>375.4769335385265</v>
+        <v>375.4805258440902</v>
       </c>
       <c r="F14">
-        <v>176580.9274217424</v>
+        <v>176583.6223578482</v>
       </c>
       <c r="G14">
         <v>1984</v>
       </c>
       <c r="H14">
-        <v>0.2986684914392284</v>
+        <v>0.2986701921753074</v>
       </c>
       <c r="I14">
         <v>-31.90471960449219</v>
       </c>
       <c r="J14">
-        <v>0.9361263635652697</v>
+        <v>0.9361316942376596</v>
       </c>
       <c r="K14" t="s">
         <v>43</v>
@@ -1101,25 +1101,25 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.72917195190471</v>
+        <v>29.72922449361318</v>
       </c>
       <c r="C15">
-        <v>8.476522669641819</v>
+        <v>8.476507688726892</v>
       </c>
       <c r="D15">
-        <v>1.210931809948831</v>
+        <v>1.210929669818128</v>
       </c>
       <c r="E15">
-        <v>3512.869473557264</v>
+        <v>3512.913313264904</v>
       </c>
       <c r="F15">
-        <v>1644432.111412525</v>
+        <v>1644455.539817803</v>
       </c>
       <c r="G15">
         <v>1984</v>
       </c>
       <c r="H15">
-        <v>0.2972917195190471</v>
+        <v>0.2972922449361318</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -1139,31 +1139,31 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.26773228693315</v>
+        <v>28.26797135488714</v>
       </c>
       <c r="C16">
-        <v>8.914758263664746</v>
+        <v>8.914682869750139</v>
       </c>
       <c r="D16">
-        <v>1.273536894809249</v>
+        <v>1.27352612425002</v>
       </c>
       <c r="E16">
-        <v>4114.07545950133</v>
+        <v>4114.092036692101</v>
       </c>
       <c r="F16">
-        <v>1831193.952822947</v>
+        <v>1831216.818378174</v>
       </c>
       <c r="G16">
         <v>1984</v>
       </c>
       <c r="H16">
-        <v>0.2826773228693314</v>
+        <v>0.2826797135488714</v>
       </c>
       <c r="I16">
         <v>88.7705174560388</v>
       </c>
       <c r="J16">
-        <v>0.3184360426977569</v>
+        <v>0.3184387357985841</v>
       </c>
       <c r="K16" t="s">
         <v>43</v>
@@ -1177,31 +1177,31 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.47356228574118</v>
+        <v>27.47384700758074</v>
       </c>
       <c r="C17">
-        <v>9.172454499312904</v>
+        <v>9.172359441707115</v>
       </c>
       <c r="D17">
-        <v>1.310350642758986</v>
+        <v>1.310337063101016</v>
       </c>
       <c r="E17">
-        <v>1607.663722048145</v>
+        <v>1607.683194958874</v>
       </c>
       <c r="F17">
-        <v>695474.657253944</v>
+        <v>695490.2888552226</v>
       </c>
       <c r="G17">
         <v>1984</v>
       </c>
       <c r="H17">
-        <v>0.2747356228574118</v>
+        <v>0.2747384700758074</v>
       </c>
       <c r="I17">
         <v>-86.12577548219299</v>
       </c>
       <c r="J17">
-        <v>0.3189934968007516</v>
+        <v>0.3189968026849421</v>
       </c>
       <c r="K17" t="s">
         <v>43</v>
@@ -1215,31 +1215,31 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>26.17225582665544</v>
+        <v>26.17281989001769</v>
       </c>
       <c r="C18">
-        <v>9.628516611982205</v>
+        <v>9.628309103067368</v>
       </c>
       <c r="D18">
-        <v>1.375502373140315</v>
+        <v>1.375472729009624</v>
       </c>
       <c r="E18">
-        <v>2321.132121617712</v>
+        <v>2321.120693690204</v>
       </c>
       <c r="F18">
-        <v>956559.834680805</v>
+        <v>956575.7407630963</v>
       </c>
       <c r="G18">
         <v>1984</v>
       </c>
       <c r="H18">
-        <v>0.2617225582665544</v>
+        <v>0.2617281989001769</v>
       </c>
       <c r="I18">
         <v>228.6002487182617</v>
       </c>
       <c r="J18">
-        <v>0.1144891835131441</v>
+        <v>0.1144916509792357</v>
       </c>
       <c r="K18" t="s">
         <v>43</v>
@@ -1253,31 +1253,31 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>25.68819034269129</v>
+        <v>25.6883257658199</v>
       </c>
       <c r="C19">
-        <v>9.809955338940336</v>
+        <v>9.809903623042006</v>
       </c>
       <c r="D19">
-        <v>1.401422191277191</v>
+        <v>1.401414803291715</v>
       </c>
       <c r="E19">
-        <v>326.5731636744792</v>
+        <v>326.5749147811169</v>
       </c>
       <c r="F19">
-        <v>132094.6190566765</v>
+        <v>132096.0237374518</v>
       </c>
       <c r="G19">
         <v>1984</v>
       </c>
       <c r="H19">
-        <v>0.2568819034269129</v>
+        <v>0.256883257658199</v>
       </c>
       <c r="I19">
         <v>5.388</v>
       </c>
       <c r="J19">
-        <v>4.767667101464605</v>
+        <v>4.767692235675558</v>
       </c>
       <c r="K19" t="s">
         <v>43</v>
@@ -1291,25 +1291,25 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>25.51839895727322</v>
+        <v>25.51859381286541</v>
       </c>
       <c r="C20">
-        <v>9.875227690496441</v>
+        <v>9.875152284956711</v>
       </c>
       <c r="D20">
-        <v>1.410746812928063</v>
+        <v>1.410736040708102</v>
       </c>
       <c r="E20">
-        <v>4524.739744456628</v>
+        <v>4524.742566357086</v>
       </c>
       <c r="F20">
-        <v>1818101.604207297</v>
+        <v>1818116.620910785</v>
       </c>
       <c r="G20">
         <v>1984</v>
       </c>
       <c r="H20">
-        <v>0.2551839895727322</v>
+        <v>0.2551859381286541</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1329,31 +1329,31 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>24.350146537716</v>
+        <v>24.34935314196738</v>
       </c>
       <c r="C21">
-        <v>10.34901369524313</v>
+        <v>10.34935090598628</v>
       </c>
       <c r="D21">
-        <v>1.478430527891876</v>
+        <v>1.478478700855183</v>
       </c>
       <c r="E21">
-        <v>2851.572983342905</v>
+        <v>2851.630828696694</v>
       </c>
       <c r="F21">
-        <v>1093344.924560835</v>
+        <v>1093331.478568718</v>
       </c>
       <c r="G21">
         <v>1984</v>
       </c>
       <c r="H21">
-        <v>0.24350146537716</v>
+        <v>0.2434935314196738</v>
       </c>
       <c r="I21">
         <v>-70.15822219843648</v>
       </c>
       <c r="J21">
-        <v>0.3470747372823061</v>
+        <v>0.3470634286184923</v>
       </c>
       <c r="K21" t="s">
         <v>43</v>
@@ -1367,31 +1367,31 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>24.21587574727746</v>
+        <v>24.21616657915808</v>
       </c>
       <c r="C22">
-        <v>10.40639630917878</v>
+        <v>10.40627133019834</v>
       </c>
       <c r="D22">
-        <v>1.486628044168397</v>
+        <v>1.486610190028334</v>
       </c>
       <c r="E22">
-        <v>4010.839605886661</v>
+        <v>4010.859435164335</v>
       </c>
       <c r="F22">
-        <v>1529348.977620689</v>
+        <v>1529374.906124876</v>
       </c>
       <c r="G22">
         <v>1984</v>
       </c>
       <c r="H22">
-        <v>0.2421587574727746</v>
+        <v>0.2421616657915809</v>
       </c>
       <c r="I22">
         <v>-128.6229438781738</v>
       </c>
       <c r="J22">
-        <v>0.1882702651419152</v>
+        <v>0.1882725262616801</v>
       </c>
       <c r="K22" t="s">
         <v>43</v>
@@ -1405,31 +1405,31 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>23.53767811103409</v>
+        <v>23.53697886600697</v>
       </c>
       <c r="C23">
-        <v>10.7062386872334</v>
+        <v>10.70655675202005</v>
       </c>
       <c r="D23">
-        <v>1.529462669604772</v>
+        <v>1.529508107431435</v>
       </c>
       <c r="E23">
-        <v>1733.488241581939</v>
+        <v>1733.483412139244</v>
       </c>
       <c r="F23">
-        <v>642474.1259317657</v>
+        <v>642453.2497874013</v>
       </c>
       <c r="G23">
         <v>1984</v>
       </c>
       <c r="H23">
-        <v>0.2353767811103409</v>
+        <v>0.2353697886600697</v>
       </c>
       <c r="I23">
         <v>-51.9349033203125</v>
       </c>
       <c r="J23">
-        <v>0.4532150173817338</v>
+        <v>0.4532015535071057</v>
       </c>
       <c r="K23" t="s">
         <v>43</v>
@@ -1443,31 +1443,31 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>23.41242202910682</v>
+        <v>23.4126027926713</v>
       </c>
       <c r="C24">
-        <v>10.76351689230223</v>
+        <v>10.76343378955209</v>
       </c>
       <c r="D24">
-        <v>1.537645270328889</v>
+        <v>1.537633398507442</v>
       </c>
       <c r="E24">
-        <v>767.7597883997535</v>
+        <v>767.7623955056337</v>
       </c>
       <c r="F24">
-        <v>283036.7500560132</v>
+        <v>283039.8964616226</v>
       </c>
       <c r="G24">
         <v>1984</v>
       </c>
       <c r="H24">
-        <v>0.2341242202910682</v>
+        <v>0.234126027926713</v>
       </c>
       <c r="I24">
         <v>-76.76021575927734</v>
       </c>
       <c r="J24">
-        <v>0.3050072462345465</v>
+        <v>0.3050096011466932</v>
       </c>
       <c r="K24" t="s">
         <v>43</v>
@@ -1481,31 +1481,31 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>23.19760753025083</v>
+        <v>23.19777916236094</v>
       </c>
       <c r="C25">
-        <v>10.86318921774065</v>
+        <v>10.86310884487069</v>
       </c>
       <c r="D25">
-        <v>1.551884173962949</v>
+        <v>1.551872692124384</v>
       </c>
       <c r="E25">
-        <v>578.3997902984275</v>
+        <v>578.4011068633512</v>
       </c>
       <c r="F25">
-        <v>211272.2444488083</v>
+        <v>211274.2884940778</v>
       </c>
       <c r="G25">
         <v>1984</v>
       </c>
       <c r="H25">
-        <v>0.2319760753025083</v>
+        <v>0.2319777916236094</v>
       </c>
       <c r="I25">
         <v>-162.9592895507592</v>
       </c>
       <c r="J25">
-        <v>0.1423521641153519</v>
+        <v>0.1423532173361323</v>
       </c>
       <c r="K25" t="s">
         <v>43</v>
@@ -1519,31 +1519,31 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>22.07816069660684</v>
+        <v>22.07828457384698</v>
       </c>
       <c r="C26">
-        <v>11.41399428434858</v>
+        <v>11.41393024250211</v>
       </c>
       <c r="D26">
-        <v>1.630570612049798</v>
+        <v>1.630561463214588</v>
       </c>
       <c r="E26">
-        <v>1129.978926246995</v>
+        <v>1129.980905137649</v>
       </c>
       <c r="F26">
-        <v>392829.7375701702</v>
+        <v>392832.6296309376</v>
       </c>
       <c r="G26">
         <v>1984</v>
       </c>
       <c r="H26">
-        <v>0.2207816069660684</v>
+        <v>0.2207828457384698</v>
       </c>
       <c r="I26">
         <v>-19.08604815673828</v>
       </c>
       <c r="J26">
-        <v>1.156769621206903</v>
+        <v>1.156776111667323</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -1557,31 +1557,31 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>21.7649873870887</v>
+        <v>21.76511615073989</v>
       </c>
       <c r="C27">
-        <v>11.57822862555344</v>
+        <v>11.57816012810175</v>
       </c>
       <c r="D27">
-        <v>1.654032660793349</v>
+        <v>1.654022875443107</v>
       </c>
       <c r="E27">
-        <v>658.3889539535795</v>
+        <v>658.3919745351714</v>
       </c>
       <c r="F27">
-        <v>225637.9152439586</v>
+        <v>225640.2853346857</v>
       </c>
       <c r="G27">
         <v>1984</v>
       </c>
       <c r="H27">
-        <v>0.217649873870887</v>
+        <v>0.2176511615073989</v>
       </c>
       <c r="I27">
         <v>-0.063</v>
       </c>
       <c r="J27">
-        <v>345.4759902712492</v>
+        <v>345.4780341387284</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -1595,31 +1595,31 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>19.63847872636613</v>
+        <v>19.63833841116994</v>
       </c>
       <c r="C28">
-        <v>12.83195116644504</v>
+        <v>12.83204285025799</v>
       </c>
       <c r="D28">
-        <v>1.83313588092072</v>
+        <v>1.833148978608284</v>
       </c>
       <c r="E28">
-        <v>1990.92673638311</v>
+        <v>1990.968381652041</v>
       </c>
       <c r="F28">
-        <v>615650.5107832941</v>
+        <v>615658.9898105327</v>
       </c>
       <c r="G28">
         <v>1984</v>
       </c>
       <c r="H28">
-        <v>0.1963847872636613</v>
+        <v>0.1963833841116994</v>
       </c>
       <c r="I28">
         <v>-170.6402893066406</v>
       </c>
       <c r="J28">
-        <v>0.1150869985403961</v>
+        <v>0.1150861762539551</v>
       </c>
       <c r="K28" t="s">
         <v>44</v>
@@ -1633,31 +1633,31 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>19.46106260844935</v>
+        <v>19.45954343617745</v>
       </c>
       <c r="C29">
-        <v>12.94893321449929</v>
+        <v>12.94994411490169</v>
       </c>
       <c r="D29">
-        <v>1.849847602071327</v>
+        <v>1.849992016414527</v>
       </c>
       <c r="E29">
-        <v>15619.02493780222</v>
+        <v>15618.7559873286</v>
       </c>
       <c r="F29">
-        <v>4786208.24793525</v>
+        <v>4785752.216984787</v>
       </c>
       <c r="G29">
         <v>1984</v>
       </c>
       <c r="H29">
-        <v>0.1946106260844935</v>
+        <v>0.1945954343617745</v>
       </c>
       <c r="I29">
         <v>-451.6016235352632</v>
       </c>
       <c r="J29">
-        <v>0.04309342923991889</v>
+        <v>0.04309006527443973</v>
       </c>
       <c r="K29" t="s">
         <v>44</v>
@@ -1671,31 +1671,31 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>18.40113545860969</v>
+        <v>18.40133434703328</v>
       </c>
       <c r="C30">
-        <v>13.69480707138058</v>
+        <v>13.69465905284353</v>
       </c>
       <c r="D30">
-        <v>1.956401010197226</v>
+        <v>1.956379864691933</v>
       </c>
       <c r="E30">
-        <v>501.1862015447185</v>
+        <v>501.1842812396358</v>
       </c>
       <c r="F30">
-        <v>145216.1273513261</v>
+        <v>145217.1405133262</v>
       </c>
       <c r="G30">
         <v>1984</v>
       </c>
       <c r="H30">
-        <v>0.1840113545860969</v>
+        <v>0.1840133434703329</v>
       </c>
       <c r="I30">
         <v>-160.1418685913086</v>
       </c>
       <c r="J30">
-        <v>0.1149052126122649</v>
+        <v>0.1149064545637004</v>
       </c>
       <c r="K30" t="s">
         <v>44</v>
@@ -1709,31 +1709,31 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>17.82614074399896</v>
+        <v>17.82625918535862</v>
       </c>
       <c r="C31">
-        <v>14.13654271100905</v>
+        <v>14.13644878489016</v>
       </c>
       <c r="D31">
-        <v>2.019506101572722</v>
+        <v>2.019492683555738</v>
       </c>
       <c r="E31">
-        <v>51.45880008368957</v>
+        <v>51.45918685153374</v>
       </c>
       <c r="F31">
-        <v>14444.0209255029</v>
+        <v>14444.22545817417</v>
       </c>
       <c r="G31">
         <v>1984</v>
       </c>
       <c r="H31">
-        <v>1.426091259519917</v>
+        <v>1.42610073482869</v>
       </c>
       <c r="I31">
         <v>221.2568876953125</v>
       </c>
       <c r="J31">
-        <v>0.6445409561594091</v>
+        <v>0.6445452386515254</v>
       </c>
       <c r="K31" t="s">
         <v>44</v>
@@ -1747,31 +1747,31 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.01603043943915</v>
+        <v>17.01604057835124</v>
       </c>
       <c r="C32">
-        <v>14.80956448079239</v>
+        <v>14.80955565659666</v>
       </c>
       <c r="D32">
-        <v>2.115652068684626</v>
+        <v>2.115650808085238</v>
       </c>
       <c r="E32">
-        <v>3427.338357221291</v>
+        <v>3427.415523779759</v>
       </c>
       <c r="F32">
-        <v>918303.750194174</v>
+        <v>918324.9729913536</v>
       </c>
       <c r="G32">
         <v>1984</v>
       </c>
       <c r="H32">
-        <v>0.1701603043943914</v>
+        <v>0.1701604057835124</v>
       </c>
       <c r="I32">
         <v>-7.8607646484375</v>
       </c>
       <c r="J32">
-        <v>2.16467878132205</v>
+        <v>2.164680071134499</v>
       </c>
       <c r="K32" t="s">
         <v>44</v>
@@ -1785,31 +1785,31 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>15.9440832102215</v>
+        <v>15.94412501775627</v>
       </c>
       <c r="C33">
-        <v>15.805236129127</v>
+        <v>15.80519468577666</v>
       </c>
       <c r="D33">
-        <v>2.257890875589571</v>
+        <v>2.257884955110951</v>
       </c>
       <c r="E33">
-        <v>1277.286649847928</v>
+        <v>1277.312846760583</v>
       </c>
       <c r="F33">
-        <v>320670.5287532154</v>
+        <v>320677.9465049618</v>
       </c>
       <c r="G33">
         <v>1984</v>
       </c>
       <c r="H33">
-        <v>0.159440832102215</v>
+        <v>0.1594412501775627</v>
       </c>
       <c r="I33">
         <v>-266.0688400268555</v>
       </c>
       <c r="J33">
-        <v>0.05992465411813046</v>
+        <v>0.05992481124864888</v>
       </c>
       <c r="K33" t="s">
         <v>44</v>
@@ -1869,10 +1869,10 @@
         <v>1.006057268722467</v>
       </c>
       <c r="F2">
-        <v>1309.334475620419</v>
+        <v>1309.354961445546</v>
       </c>
       <c r="G2">
-        <v>117.6178397979531</v>
+        <v>117.6199240295791</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1892,10 +1892,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F3">
-        <v>4582.865676818092</v>
+        <v>4582.675348167124</v>
       </c>
       <c r="G3">
-        <v>460.4184620066599</v>
+        <v>460.4246370781944</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1915,10 +1915,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F4">
-        <v>2781.193732469626</v>
+        <v>2781.268481942817</v>
       </c>
       <c r="G4">
-        <v>352.8537073840405</v>
+        <v>352.8616381812393</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1938,10 +1938,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F5">
-        <v>1196.282302020106</v>
+        <v>1196.430677875789</v>
       </c>
       <c r="G5">
-        <v>114.4789016965797</v>
+        <v>114.4801041779227</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1961,10 +1961,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F6">
-        <v>7457.305079989717</v>
+        <v>7456.82645249261</v>
       </c>
       <c r="G6">
-        <v>485.3170140440412</v>
+        <v>485.3250841010128</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1984,10 +1984,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F7">
-        <v>19144.44845616249</v>
+        <v>19144.4970439702</v>
       </c>
       <c r="G7">
-        <v>1343.70490248541</v>
+        <v>1343.708952675569</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -2007,10 +2007,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F8">
-        <v>4145.303617269218</v>
+        <v>4145.298474922745</v>
       </c>
       <c r="G8">
-        <v>509.5432932458223</v>
+        <v>509.5492971370375</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2030,10 +2030,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F9">
-        <v>869.7829130955656</v>
+        <v>869.7836593477695</v>
       </c>
       <c r="G9">
-        <v>108.9295404404519</v>
+        <v>108.9304105840945</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2053,10 +2053,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F10">
-        <v>2359.297028781581</v>
+        <v>2359.294185075335</v>
       </c>
       <c r="G10">
-        <v>143.6005834885912</v>
+        <v>143.6021798384691</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2076,10 +2076,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F11">
-        <v>4229.667737531526</v>
+        <v>4229.710079622043</v>
       </c>
       <c r="G11">
-        <v>390.7125884847283</v>
+        <v>390.7189501029537</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2099,10 +2099,10 @@
         <v>1.357973990417522</v>
       </c>
       <c r="F12">
-        <v>6803.916919947763</v>
+        <v>6804.085959017637</v>
       </c>
       <c r="G12">
-        <v>628.5446613238699</v>
+        <v>628.5591875368608</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2122,10 +2122,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F13">
-        <v>5512.04294046513</v>
+        <v>5512.163928441823</v>
       </c>
       <c r="G13">
-        <v>554.7158419892617</v>
+        <v>554.7090200754529</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2145,10 +2145,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F14">
-        <v>3490.02062026206</v>
+        <v>3490.068189659779</v>
       </c>
       <c r="G14">
-        <v>325.9635342119562</v>
+        <v>325.9529425608327</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2168,10 +2168,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F15">
-        <v>1323.02510359202</v>
+        <v>1322.750416786489</v>
       </c>
       <c r="G15">
-        <v>107.1903827746364</v>
+        <v>107.1914198346412</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2191,10 +2191,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F16">
-        <v>754.6247418810801</v>
+        <v>754.6518248072589</v>
       </c>
       <c r="G16">
-        <v>89.58951162949892</v>
+        <v>89.59087892331215</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -2214,10 +2214,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F17">
-        <v>6486.490626042079</v>
+        <v>6486.89871742941</v>
       </c>
       <c r="G17">
-        <v>929.0684692150924</v>
+        <v>929.0800702070896</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2237,10 +2237,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F18">
-        <v>2117.109075449589</v>
+        <v>2117.104317135825</v>
       </c>
       <c r="G18">
-        <v>281.1234046717595</v>
+        <v>281.1261570309838</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2260,10 +2260,10 @@
         <v>1.357973990417522</v>
       </c>
       <c r="F19">
-        <v>128.5749268433929</v>
+        <v>128.5793504955643</v>
       </c>
       <c r="G19">
-        <v>9.886393515060165</v>
+        <v>9.886533510043927</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2283,10 +2283,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F20">
-        <v>8084.276290010856</v>
+        <v>8084.482118516435</v>
       </c>
       <c r="G20">
-        <v>834.3136029490231</v>
+        <v>834.3254895067491</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2306,10 +2306,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F21">
-        <v>4929.787541816194</v>
+        <v>4929.689824844304</v>
       </c>
       <c r="G21">
-        <v>470.3548937764693</v>
+        <v>470.3628298183344</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2329,10 +2329,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F22">
-        <v>110765.1428794139</v>
+        <v>110891.2995462922</v>
       </c>
       <c r="G22">
-        <v>9378.035320545319</v>
+        <v>9378.677924782693</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2352,10 +2352,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F23">
-        <v>12308.66597065689</v>
+        <v>12308.97177991711</v>
       </c>
       <c r="G23">
-        <v>775.9254072149613</v>
+        <v>775.9385622145492</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2375,10 +2375,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F24">
-        <v>21175.7833966581</v>
+        <v>21177.74632497273</v>
       </c>
       <c r="G24">
-        <v>2025.156546483714</v>
+        <v>2025.196765491255</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2398,10 +2398,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F25">
-        <v>9243.046189481685</v>
+        <v>9243.003368178152</v>
       </c>
       <c r="G25">
-        <v>922.4259787961932</v>
+        <v>922.4335976208957</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2421,10 +2421,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F26">
-        <v>82820.32399834305</v>
+        <v>82819.67182870273</v>
       </c>
       <c r="G26">
-        <v>2428.314686928082</v>
+        <v>2428.083316582845</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2444,10 +2444,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F27">
-        <v>8390.831242377202</v>
+        <v>8390.864246806283</v>
       </c>
       <c r="G27">
-        <v>745.5778287496603</v>
+        <v>745.5853052285848</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2467,10 +2467,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F28">
-        <v>3366.073485607739</v>
+        <v>3365.908958623802</v>
       </c>
       <c r="G28">
-        <v>162.6943321934122</v>
+        <v>162.69809563925</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2490,10 +2490,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F29">
-        <v>1182.717363508757</v>
+        <v>1182.684939504984</v>
       </c>
       <c r="G29">
-        <v>73.67637105597466</v>
+        <v>73.676885090475</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2513,10 +2513,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F30">
-        <v>537.3580983170499</v>
+        <v>537.3479611693675</v>
       </c>
       <c r="G30">
-        <v>67.0190862793894</v>
+        <v>67.01979895355245</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2536,10 +2536,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F31">
-        <v>3040.582567966747</v>
+        <v>3041.368145783164</v>
       </c>
       <c r="G31">
-        <v>312.3543941061868</v>
+        <v>312.3586959972261</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2559,10 +2559,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F32">
-        <v>2787.768473842686</v>
+        <v>2787.922068767069</v>
       </c>
       <c r="G32">
-        <v>199.3047882141909</v>
+        <v>199.3062555205163</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2582,10 +2582,10 @@
         <v>1.006595636732623</v>
       </c>
       <c r="F33">
-        <v>2461.901635750122</v>
+        <v>2461.971740869314</v>
       </c>
       <c r="G33">
-        <v>269.9881232266981</v>
+        <v>269.9923237674877</v>
       </c>
     </row>
   </sheetData>
@@ -2621,13 +2621,13 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>36.21304347685363</v>
+        <v>36.21314297445958</v>
       </c>
       <c r="C2">
-        <v>0.3621304347685363</v>
+        <v>0.3621314297445958</v>
       </c>
       <c r="D2">
-        <v>0.2932053047674103</v>
+        <v>0.2932061103673564</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
@@ -2638,13 +2638,13 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>35.73981517165323</v>
+        <v>35.73983427744304</v>
       </c>
       <c r="C3">
-        <v>0.3573981517165323</v>
+        <v>0.3573983427744304</v>
       </c>
       <c r="D3">
-        <v>0.3816418130809784</v>
+        <v>0.3816420170990526</v>
       </c>
       <c r="E3" t="s">
         <v>53</v>
@@ -2655,13 +2655,13 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>35.28804328874659</v>
+        <v>35.28818078629894</v>
       </c>
       <c r="C4">
-        <v>0.3528804328874658</v>
+        <v>0.3528818078629894</v>
       </c>
       <c r="D4">
-        <v>0.3827227469540423</v>
+        <v>0.3827242382081905</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -2672,13 +2672,13 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>34.28462471972859</v>
+        <v>34.28474383414597</v>
       </c>
       <c r="C5">
-        <v>0.3428462471972859</v>
+        <v>0.3428474383414597</v>
       </c>
       <c r="D5">
-        <v>0.1724603508213419</v>
+        <v>0.1724609499970476</v>
       </c>
       <c r="E5" t="s">
         <v>53</v>
@@ -2689,13 +2689,13 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>34.0091585140582</v>
+        <v>34.00927271614375</v>
       </c>
       <c r="C6">
-        <v>0.340091585140582</v>
+        <v>0.3400927271614375</v>
       </c>
       <c r="D6">
-        <v>0.1203277538943935</v>
+        <v>0.120328157952625</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
@@ -2706,13 +2706,13 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>33.25800745346309</v>
+        <v>33.25811346615763</v>
       </c>
       <c r="C7">
-        <v>0.3325800745346309</v>
+        <v>0.3325811346615763</v>
       </c>
       <c r="D7">
-        <v>0.1153218866987061</v>
+        <v>0.1153222542969143</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
@@ -2723,13 +2723,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>32.51060693467581</v>
+        <v>32.5107725123483</v>
       </c>
       <c r="C8">
-        <v>0.3251060693467581</v>
+        <v>0.325107725123483</v>
       </c>
       <c r="D8">
-        <v>0.04645248380362555</v>
+        <v>0.04645272038777068</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>32.23994760388378</v>
+        <v>32.24172325795473</v>
       </c>
       <c r="C9">
-        <v>0.3223994760388378</v>
+        <v>0.3224172325795473</v>
       </c>
       <c r="D9">
-        <v>0.1596506544260394</v>
+        <v>0.1596594473787434</v>
       </c>
       <c r="E9" t="s">
         <v>53</v>
@@ -2757,13 +2757,13 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>32.17431964099017</v>
+        <v>32.17454412208342</v>
       </c>
       <c r="C10">
-        <v>0.3217431964099017</v>
+        <v>0.3217454412208342</v>
       </c>
       <c r="D10">
-        <v>1.641404731598397</v>
+        <v>1.641416183723344</v>
       </c>
       <c r="E10" t="s">
         <v>53</v>
@@ -2774,13 +2774,13 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>31.15324841695801</v>
+        <v>31.15333849933335</v>
       </c>
       <c r="C11">
-        <v>0.3115324841695801</v>
+        <v>0.3115333849933336</v>
       </c>
       <c r="D11">
-        <v>0.06545519569145583</v>
+        <v>0.06545538496094797</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
@@ -2791,13 +2791,13 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.6279309184528</v>
+        <v>30.62816309239676</v>
       </c>
       <c r="C12">
-        <v>0.3062793091845281</v>
+        <v>0.3062816309239677</v>
       </c>
       <c r="D12">
-        <v>1.31331290602045</v>
+        <v>1.313322861542352</v>
       </c>
       <c r="E12" t="s">
         <v>53</v>
@@ -2808,13 +2808,13 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.03201167048208</v>
+        <v>30.03209660063617</v>
       </c>
       <c r="C13">
-        <v>0.3003201167048208</v>
+        <v>0.3003209660063617</v>
       </c>
       <c r="D13">
-        <v>0.3759892426434341</v>
+        <v>0.3759903059363186</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -2825,13 +2825,13 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.86684914392284</v>
+        <v>29.86701921753074</v>
       </c>
       <c r="C14">
-        <v>0.2986684914392284</v>
+        <v>0.2986701921753074</v>
       </c>
       <c r="D14">
-        <v>0.9361263635652697</v>
+        <v>0.9361316942376596</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
@@ -2842,10 +2842,10 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.72917195190471</v>
+        <v>29.72922449361318</v>
       </c>
       <c r="C15">
-        <v>0.2972917195190471</v>
+        <v>0.2972922449361318</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -2859,13 +2859,13 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.26773228693315</v>
+        <v>28.26797135488714</v>
       </c>
       <c r="C16">
-        <v>0.2826773228693314</v>
+        <v>0.2826797135488714</v>
       </c>
       <c r="D16">
-        <v>0.3184360426977569</v>
+        <v>0.3184387357985841</v>
       </c>
       <c r="E16" t="s">
         <v>53</v>
@@ -2876,13 +2876,13 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.47356228574118</v>
+        <v>27.47384700758074</v>
       </c>
       <c r="C17">
-        <v>0.2747356228574118</v>
+        <v>0.2747384700758074</v>
       </c>
       <c r="D17">
-        <v>0.3189934968007516</v>
+        <v>0.3189968026849421</v>
       </c>
       <c r="E17" t="s">
         <v>53</v>
@@ -2893,13 +2893,13 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>26.17225582665544</v>
+        <v>26.17281989001769</v>
       </c>
       <c r="C18">
-        <v>0.2617225582665544</v>
+        <v>0.2617281989001769</v>
       </c>
       <c r="D18">
-        <v>0.1144891835131441</v>
+        <v>0.1144916509792357</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
@@ -2910,13 +2910,13 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>25.68819034269129</v>
+        <v>25.6883257658199</v>
       </c>
       <c r="C19">
-        <v>0.2568819034269129</v>
+        <v>0.256883257658199</v>
       </c>
       <c r="D19">
-        <v>4.767667101464605</v>
+        <v>4.767692235675558</v>
       </c>
       <c r="E19" t="s">
         <v>53</v>
@@ -2927,10 +2927,10 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>25.51839895727322</v>
+        <v>25.51859381286541</v>
       </c>
       <c r="C20">
-        <v>0.2551839895727322</v>
+        <v>0.2551859381286541</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2944,13 +2944,13 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>24.350146537716</v>
+        <v>24.34935314196738</v>
       </c>
       <c r="C21">
-        <v>0.24350146537716</v>
+        <v>0.2434935314196738</v>
       </c>
       <c r="D21">
-        <v>0.3470747372823061</v>
+        <v>0.3470634286184923</v>
       </c>
       <c r="E21" t="s">
         <v>53</v>
@@ -2961,13 +2961,13 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>24.21587574727746</v>
+        <v>24.21616657915808</v>
       </c>
       <c r="C22">
-        <v>0.2421587574727746</v>
+        <v>0.2421616657915809</v>
       </c>
       <c r="D22">
-        <v>0.1882702651419152</v>
+        <v>0.1882725262616801</v>
       </c>
       <c r="E22" t="s">
         <v>53</v>
@@ -2978,13 +2978,13 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>23.53767811103409</v>
+        <v>23.53697886600697</v>
       </c>
       <c r="C23">
-        <v>0.2353767811103409</v>
+        <v>0.2353697886600697</v>
       </c>
       <c r="D23">
-        <v>0.4532150173817338</v>
+        <v>0.4532015535071057</v>
       </c>
       <c r="E23" t="s">
         <v>53</v>
@@ -2995,13 +2995,13 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>23.41242202910682</v>
+        <v>23.4126027926713</v>
       </c>
       <c r="C24">
-        <v>0.2341242202910682</v>
+        <v>0.234126027926713</v>
       </c>
       <c r="D24">
-        <v>0.3050072462345465</v>
+        <v>0.3050096011466932</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
@@ -3012,13 +3012,13 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>23.19760753025083</v>
+        <v>23.19777916236094</v>
       </c>
       <c r="C25">
-        <v>0.2319760753025083</v>
+        <v>0.2319777916236094</v>
       </c>
       <c r="D25">
-        <v>0.1423521641153519</v>
+        <v>0.1423532173361323</v>
       </c>
       <c r="E25" t="s">
         <v>53</v>
@@ -3029,13 +3029,13 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>22.07816069660684</v>
+        <v>22.07828457384698</v>
       </c>
       <c r="C26">
-        <v>0.2207816069660684</v>
+        <v>0.2207828457384698</v>
       </c>
       <c r="D26">
-        <v>1.156769621206903</v>
+        <v>1.156776111667323</v>
       </c>
       <c r="E26" t="s">
         <v>53</v>
@@ -3046,13 +3046,13 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>21.7649873870887</v>
+        <v>21.76511615073989</v>
       </c>
       <c r="C27">
-        <v>0.217649873870887</v>
+        <v>0.2176511615073989</v>
       </c>
       <c r="D27">
-        <v>345.4759902712492</v>
+        <v>345.4780341387284</v>
       </c>
       <c r="E27" t="s">
         <v>53</v>
@@ -3063,13 +3063,13 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>19.63847872636613</v>
+        <v>19.63833841116994</v>
       </c>
       <c r="C28">
-        <v>0.1963847872636613</v>
+        <v>0.1963833841116994</v>
       </c>
       <c r="D28">
-        <v>0.1150869985403961</v>
+        <v>0.1150861762539551</v>
       </c>
       <c r="E28" t="s">
         <v>53</v>
@@ -3080,13 +3080,13 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>19.46106260844935</v>
+        <v>19.45954343617745</v>
       </c>
       <c r="C29">
-        <v>0.1946106260844935</v>
+        <v>0.1945954343617745</v>
       </c>
       <c r="D29">
-        <v>0.04309342923991889</v>
+        <v>0.04309006527443973</v>
       </c>
       <c r="E29" t="s">
         <v>53</v>
@@ -3097,13 +3097,13 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>18.40113545860969</v>
+        <v>18.40133434703328</v>
       </c>
       <c r="C30">
-        <v>0.1840113545860969</v>
+        <v>0.1840133434703329</v>
       </c>
       <c r="D30">
-        <v>0.1149052126122649</v>
+        <v>0.1149064545637004</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -3114,13 +3114,13 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>17.82614074399896</v>
+        <v>17.82625918535862</v>
       </c>
       <c r="C31">
-        <v>1.426091259519917</v>
+        <v>1.42610073482869</v>
       </c>
       <c r="D31">
-        <v>0.6445409561594091</v>
+        <v>0.6445452386515254</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
@@ -3131,13 +3131,13 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.01603043943915</v>
+        <v>17.01604057835124</v>
       </c>
       <c r="C32">
-        <v>0.1701603043943914</v>
+        <v>0.1701604057835124</v>
       </c>
       <c r="D32">
-        <v>2.16467878132205</v>
+        <v>2.164680071134499</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
@@ -3148,13 +3148,13 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>15.9440832102215</v>
+        <v>15.94412501775627</v>
       </c>
       <c r="C33">
-        <v>0.159440832102215</v>
+        <v>0.1594412501775627</v>
       </c>
       <c r="D33">
-        <v>0.05992465411813046</v>
+        <v>0.05992481124864888</v>
       </c>
       <c r="E33" t="s">
         <v>53</v>
@@ -3217,16 +3217,16 @@
         <v>8.42911877394636</v>
       </c>
       <c r="F2">
-        <v>620.208749778591</v>
+        <v>620.2173112820382</v>
       </c>
       <c r="G2">
-        <v>2122.988110254268</v>
+        <v>2122.998332823759</v>
       </c>
       <c r="H2">
-        <v>-2055.623687808357</v>
+        <v>-2055.697801867108</v>
       </c>
       <c r="I2">
-        <v>4178.611798062625</v>
+        <v>4178.696134690867</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -3246,16 +3246,16 @@
         <v>-1.461693548387097</v>
       </c>
       <c r="F3">
-        <v>2366.312144384441</v>
+        <v>2366.343312581236</v>
       </c>
       <c r="G3">
-        <v>4572.613423247701</v>
+        <v>4572.659425529603</v>
       </c>
       <c r="H3">
-        <v>-6867.739392361063</v>
+        <v>-6868.004630611985</v>
       </c>
       <c r="I3">
-        <v>11440.35281560876</v>
+        <v>11440.66405614159</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3275,16 +3275,16 @@
         <v>3.175403225806452</v>
       </c>
       <c r="F4">
-        <v>1860.410680800024</v>
+        <v>1860.439909226242</v>
       </c>
       <c r="G4">
-        <v>5914.295308281251</v>
+        <v>5914.515704427017</v>
       </c>
       <c r="H4">
-        <v>-3617.794481288357</v>
+        <v>-3617.849227703511</v>
       </c>
       <c r="I4">
-        <v>9532.089789569607</v>
+        <v>9532.364932130527</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3304,16 +3304,16 @@
         <v>8.71975806451613</v>
       </c>
       <c r="F5">
-        <v>827.7545722733353</v>
+        <v>827.7610446556429</v>
       </c>
       <c r="G5">
-        <v>4314.745105335555</v>
+        <v>4314.821203627136</v>
       </c>
       <c r="H5">
-        <v>-1849.374436760397</v>
+        <v>-1849.383798894357</v>
       </c>
       <c r="I5">
-        <v>6164.119542095952</v>
+        <v>6164.205002521493</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3333,16 +3333,16 @@
         <v>9.828629032258064</v>
       </c>
       <c r="F6">
-        <v>3130.906919046688</v>
+        <v>3130.86174709911</v>
       </c>
       <c r="G6">
-        <v>19309.07150336377</v>
+        <v>19308.92284016448</v>
       </c>
       <c r="H6">
-        <v>-5013.935860301134</v>
+        <v>-5013.769069157467</v>
       </c>
       <c r="I6">
-        <v>24323.00736366491</v>
+        <v>24322.69190932194</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3350,28 +3350,28 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="C7">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="D7">
         <v>13</v>
       </c>
       <c r="E7">
-        <v>4.183467741935484</v>
+        <v>4.08266129032258</v>
       </c>
       <c r="F7">
-        <v>6431.708644813905</v>
+        <v>6431.714777386662</v>
       </c>
       <c r="G7">
-        <v>21979.52855326945</v>
+        <v>21979.45330646568</v>
       </c>
       <c r="H7">
-        <v>-18702.46190531276</v>
+        <v>-18702.28645408327</v>
       </c>
       <c r="I7">
-        <v>40681.99045858221</v>
+        <v>40681.73976054894</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3391,16 +3391,16 @@
         <v>1.86491935483871</v>
       </c>
       <c r="F8">
-        <v>2660.558009763759</v>
+        <v>2660.587028175543</v>
       </c>
       <c r="G8">
-        <v>6760.847927486031</v>
+        <v>6760.846067053688</v>
       </c>
       <c r="H8">
-        <v>-8009.784116565608</v>
+        <v>-8009.997209004826</v>
       </c>
       <c r="I8">
-        <v>14770.63204405164</v>
+        <v>14770.84327605851</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3420,16 +3420,16 @@
         <v>2.268145161290323</v>
       </c>
       <c r="F9">
-        <v>479.9775117224622</v>
+        <v>479.9797218708287</v>
       </c>
       <c r="G9">
-        <v>1849.738629252209</v>
+        <v>1849.738748448387</v>
       </c>
       <c r="H9">
-        <v>-1576.554186214479</v>
+        <v>-1576.551936913168</v>
       </c>
       <c r="I9">
-        <v>3426.292815466689</v>
+        <v>3426.290685361555</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3449,16 +3449,16 @@
         <v>13.35685483870968</v>
       </c>
       <c r="F10">
-        <v>882.6696046560172</v>
+        <v>882.6721136685038</v>
       </c>
       <c r="G10">
-        <v>3377.584686525204</v>
+        <v>3377.60575341587</v>
       </c>
       <c r="H10">
-        <v>-2290.280849178625</v>
+        <v>-2290.236779198098</v>
       </c>
       <c r="I10">
-        <v>5667.86553570383</v>
+        <v>5667.842532613968</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3478,16 +3478,16 @@
         <v>6.804435483870967</v>
       </c>
       <c r="F11">
-        <v>2090.383215568073</v>
+        <v>2090.4168244344</v>
       </c>
       <c r="G11">
-        <v>7037.29761326198</v>
+        <v>7037.489622822785</v>
       </c>
       <c r="H11">
-        <v>-6683.321866629703</v>
+        <v>-6683.574361353197</v>
       </c>
       <c r="I11">
-        <v>13720.61947989168</v>
+        <v>13721.06398417598</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3507,16 +3507,16 @@
         <v>11.0383064516129</v>
       </c>
       <c r="F12">
-        <v>4391.504864609921</v>
+        <v>4391.620423962324</v>
       </c>
       <c r="G12">
-        <v>11001.4802802549</v>
+        <v>11001.52427943153</v>
       </c>
       <c r="H12">
-        <v>-9957.595250968969</v>
+        <v>-9958.113972963189</v>
       </c>
       <c r="I12">
-        <v>20959.07553122387</v>
+        <v>20959.63825239472</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3536,16 +3536,16 @@
         <v>12.55040322580645</v>
       </c>
       <c r="F13">
-        <v>3140.103376025946</v>
+        <v>3140.144293950367</v>
       </c>
       <c r="G13">
-        <v>13376.59344067618</v>
+        <v>13376.2371642817</v>
       </c>
       <c r="H13">
-        <v>-4707.981917996269</v>
+        <v>-4708.031964205812</v>
       </c>
       <c r="I13">
-        <v>18084.57535867245</v>
+        <v>18084.26912848751</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3565,16 +3565,16 @@
         <v>7.308467741935484</v>
       </c>
       <c r="F14">
-        <v>2128.62507419215</v>
+        <v>2128.629357334803</v>
       </c>
       <c r="G14">
-        <v>9239.404253858986</v>
+        <v>9239.42656432446</v>
       </c>
       <c r="H14">
-        <v>-3322.801460197399</v>
+        <v>-3323.026007880733</v>
       </c>
       <c r="I14">
-        <v>12562.20571405638</v>
+        <v>12562.45257220519</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3594,16 +3594,16 @@
         <v>14.36491935483871</v>
       </c>
       <c r="F15">
-        <v>640.3183862290848</v>
+        <v>640.3194215506687</v>
       </c>
       <c r="G15">
-        <v>2877.798746481251</v>
+        <v>2877.481783478114</v>
       </c>
       <c r="H15">
-        <v>-1337.454498201607</v>
+        <v>-1337.505756689111</v>
       </c>
       <c r="I15">
-        <v>4215.253244682858</v>
+        <v>4214.987540167225</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -3623,16 +3623,16 @@
         <v>3.981854838709677</v>
       </c>
       <c r="F16">
-        <v>472.0920504266741</v>
+        <v>472.098201982139</v>
       </c>
       <c r="G16">
-        <v>1400.698349738472</v>
+        <v>1400.707010552066</v>
       </c>
       <c r="H16">
-        <v>-1348.530073084272</v>
+        <v>-1348.562930193893</v>
       </c>
       <c r="I16">
-        <v>2749.228422822744</v>
+        <v>2749.269940745959</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -3652,16 +3652,16 @@
         <v>6.90524193548387</v>
       </c>
       <c r="F17">
-        <v>4829.165927046781</v>
+        <v>4829.165775245163</v>
       </c>
       <c r="G17">
-        <v>17356.20290579283</v>
+        <v>17355.76782920236</v>
       </c>
       <c r="H17">
-        <v>-9610.514201487813</v>
+        <v>-9610.810275113245</v>
       </c>
       <c r="I17">
-        <v>26966.71710728064</v>
+        <v>26966.57810431561</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3681,16 +3681,16 @@
         <v>3.276209677419355</v>
       </c>
       <c r="F18">
-        <v>1248.072916657279</v>
+        <v>1248.079021898259</v>
       </c>
       <c r="G18">
-        <v>3909.623270801822</v>
+        <v>3909.641726304677</v>
       </c>
       <c r="H18">
-        <v>-3590.069759532757</v>
+        <v>-3590.060934131663</v>
       </c>
       <c r="I18">
-        <v>7499.69303033458</v>
+        <v>7499.70266043634</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3710,16 +3710,16 @@
         <v>13.05443548387097</v>
       </c>
       <c r="F19">
-        <v>52.40944119566903</v>
+        <v>52.41005973884766</v>
       </c>
       <c r="G19">
-        <v>187.3001639813403</v>
+        <v>187.3030807236183</v>
       </c>
       <c r="H19">
-        <v>-83.60757769149657</v>
+        <v>-83.61143027075832</v>
       </c>
       <c r="I19">
-        <v>270.9077416728369</v>
+        <v>270.9145109943766</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -3739,16 +3739,16 @@
         <v>5.796370967741935</v>
       </c>
       <c r="F20">
-        <v>4487.762176744586</v>
+        <v>4487.821902251935</v>
       </c>
       <c r="G20">
-        <v>13845.6080048607</v>
+        <v>13846.01562780497</v>
       </c>
       <c r="H20">
-        <v>-9400.177220723104</v>
+        <v>-9400.206661487702</v>
       </c>
       <c r="I20">
-        <v>23245.78522558381</v>
+        <v>23246.22228929268</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -3768,16 +3768,16 @@
         <v>3.881048387096774</v>
       </c>
       <c r="F21">
-        <v>2350.755386542321</v>
+        <v>2350.780988542538</v>
       </c>
       <c r="G21">
-        <v>7701.918245773003</v>
+        <v>7701.972076286408</v>
       </c>
       <c r="H21">
-        <v>-6035.18381465655</v>
+        <v>-6035.306533708129</v>
       </c>
       <c r="I21">
-        <v>13737.10206042955</v>
+        <v>13737.27860999454</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -3797,16 +3797,16 @@
         <v>6.098790322580645</v>
       </c>
       <c r="F22">
-        <v>44778.9138249534</v>
+        <v>44780.81834485844</v>
       </c>
       <c r="G22">
-        <v>160418.2430990447</v>
+        <v>160393.5366521343</v>
       </c>
       <c r="H22">
-        <v>-141493.7100718199</v>
+        <v>-141512.631573034</v>
       </c>
       <c r="I22">
-        <v>301911.9531708646</v>
+        <v>301906.1682251684</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -3826,16 +3826,16 @@
         <v>5.493951612903226</v>
       </c>
       <c r="F23">
-        <v>5289.840404279954</v>
+        <v>5289.85239273193</v>
       </c>
       <c r="G23">
-        <v>26702.12668621192</v>
+        <v>26702.26522904087</v>
       </c>
       <c r="H23">
-        <v>-11085.43602091126</v>
+        <v>-11085.51715589314</v>
       </c>
       <c r="I23">
-        <v>37787.56270712318</v>
+        <v>37787.78238493401</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -3855,16 +3855,16 @@
         <v>2.973790322580645</v>
       </c>
       <c r="F24">
-        <v>9539.657942279937</v>
+        <v>9539.860364407168</v>
       </c>
       <c r="G24">
-        <v>28687.45218760037</v>
+        <v>28688.25541021257</v>
       </c>
       <c r="H24">
-        <v>-38971.87688600265</v>
+        <v>-38971.72103729852</v>
       </c>
       <c r="I24">
-        <v>67659.32907360302</v>
+        <v>67659.97644751109</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -3884,16 +3884,16 @@
         <v>9.929435483870968</v>
       </c>
       <c r="F25">
-        <v>5082.972842983792</v>
+        <v>5082.963354213584</v>
       </c>
       <c r="G25">
-        <v>22548.11014543093</v>
+        <v>22548.24822219515</v>
       </c>
       <c r="H25">
-        <v>-7616.917812533184</v>
+        <v>-7616.716847738795</v>
       </c>
       <c r="I25">
-        <v>30165.02795796411</v>
+        <v>30164.96506993394</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -3913,16 +3913,16 @@
         <v>13.25604838709678</v>
       </c>
       <c r="F26">
-        <v>24318.61133530007</v>
+        <v>24318.35441950481</v>
       </c>
       <c r="G26">
-        <v>156545.6757112134</v>
+        <v>156546.5756237583</v>
       </c>
       <c r="H26">
-        <v>-22195.53396264274</v>
+        <v>-22192.56526796321</v>
       </c>
       <c r="I26">
-        <v>178741.2096738562</v>
+        <v>178739.1408917216</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -3942,16 +3942,16 @@
         <v>1.764112903225807</v>
       </c>
       <c r="F27">
-        <v>3519.052246077636</v>
+        <v>3519.08243396573</v>
       </c>
       <c r="G27">
-        <v>9688.749266936346</v>
+        <v>9688.918584950672</v>
       </c>
       <c r="H27">
-        <v>-10153.16550794626</v>
+        <v>-10153.0993456786</v>
       </c>
       <c r="I27">
-        <v>19841.91477488261</v>
+        <v>19842.01793062928</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3971,16 +3971,16 @@
         <v>9.72782258064516</v>
       </c>
       <c r="F28">
-        <v>1930.873791560613</v>
+        <v>1930.897793969071</v>
       </c>
       <c r="G28">
-        <v>10403.52290166022</v>
+        <v>10403.19571718122</v>
       </c>
       <c r="H28">
-        <v>-3357.698525379078</v>
+        <v>-3357.419507417613</v>
       </c>
       <c r="I28">
-        <v>13761.2214270393</v>
+        <v>13760.61522459883</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -4000,16 +4000,16 @@
         <v>6.098790322580645</v>
       </c>
       <c r="F29">
-        <v>809.7958960636123</v>
+        <v>809.7902783744468</v>
       </c>
       <c r="G29">
-        <v>4663.334953375759</v>
+        <v>4663.327823682696</v>
       </c>
       <c r="H29">
-        <v>-1668.142797685271</v>
+        <v>-1668.067292938357</v>
       </c>
       <c r="I29">
-        <v>6331.477751061029</v>
+        <v>6331.395116621054</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -4029,16 +4029,16 @@
         <v>10.23185483870968</v>
       </c>
       <c r="F30">
-        <v>403.1808309361782</v>
+        <v>403.1831738116775</v>
       </c>
       <c r="G30">
-        <v>1571.69072415516</v>
+        <v>1571.699712022933</v>
       </c>
       <c r="H30">
-        <v>-996.9145600624487</v>
+        <v>-996.9203915414954</v>
       </c>
       <c r="I30">
-        <v>2568.605284217609</v>
+        <v>2568.620103564428</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -4058,16 +4058,16 @@
         <v>6.90524193548387</v>
       </c>
       <c r="F31">
-        <v>2759.442997503642</v>
+        <v>2759.504527095887</v>
       </c>
       <c r="G31">
-        <v>10243.16670850429</v>
+        <v>10243.34542346352</v>
       </c>
       <c r="H31">
-        <v>-7565.887463369868</v>
+        <v>-7566.610770245635</v>
       </c>
       <c r="I31">
-        <v>17809.05417187416</v>
+        <v>17809.95619370915</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -4087,16 +4087,16 @@
         <v>11.84475806451613</v>
       </c>
       <c r="F32">
-        <v>1423.60082437615</v>
+        <v>1423.602856755335</v>
       </c>
       <c r="G32">
-        <v>7101.07043966832</v>
+        <v>7101.14669185745</v>
       </c>
       <c r="H32">
-        <v>-3178.991011235059</v>
+        <v>-3179.10444803575</v>
       </c>
       <c r="I32">
-        <v>10280.06145090338</v>
+        <v>10280.2511398932</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4116,16 +4116,16 @@
         <v>2.469758064516129</v>
       </c>
       <c r="F33">
-        <v>1194.286962736648</v>
+        <v>1194.30117302443</v>
       </c>
       <c r="G33">
-        <v>2985.470272750136</v>
+        <v>2985.466544107819</v>
       </c>
       <c r="H33">
-        <v>-3192.546971812177</v>
+        <v>-3192.588666640249</v>
       </c>
       <c r="I33">
-        <v>6178.017244562313</v>
+        <v>6178.055210748068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
learning pysystemtrade. Extracted Instrument volatility
</commit_message>
<xml_diff>
--- a/perplexity_examples/etf_turnover_analysis.xlsx
+++ b/perplexity_examples/etf_turnover_analysis.xlsx
@@ -55,37 +55,40 @@
     <t>EZA</t>
   </si>
   <si>
+    <t>ILF</t>
+  </si>
+  <si>
     <t>EMLC</t>
   </si>
   <si>
-    <t>ILF</t>
-  </si>
-  <si>
     <t>WIP</t>
   </si>
   <si>
+    <t>BBAX</t>
+  </si>
+  <si>
+    <t>BWX</t>
+  </si>
+  <si>
+    <t>PICB</t>
+  </si>
+  <si>
     <t>SPTL</t>
   </si>
   <si>
+    <t>EPOL</t>
+  </si>
+  <si>
+    <t>SCHO</t>
+  </si>
+  <si>
+    <t>FLJP</t>
+  </si>
+  <si>
     <t>SCHR</t>
   </si>
   <si>
-    <t>FLJP</t>
-  </si>
-  <si>
-    <t>SCHO</t>
-  </si>
-  <si>
-    <t>BBAX</t>
-  </si>
-  <si>
-    <t>EPOL</t>
-  </si>
-  <si>
-    <t>PICB</t>
-  </si>
-  <si>
-    <t>BWX</t>
+    <t>CMBS</t>
   </si>
   <si>
     <t>IEMG</t>
@@ -94,13 +97,13 @@
     <t>KSA</t>
   </si>
   <si>
+    <t>EMHY</t>
+  </si>
+  <si>
     <t>IHY</t>
   </si>
   <si>
-    <t>CMBS</t>
-  </si>
-  <si>
-    <t>EMHY</t>
+    <t>SCHP</t>
   </si>
   <si>
     <t>VGK</t>
@@ -112,40 +115,37 @@
     <t>HYLB</t>
   </si>
   <si>
-    <t>SCHP</t>
-  </si>
-  <si>
     <t>IAU</t>
   </si>
   <si>
+    <t>VMBS</t>
+  </si>
+  <si>
+    <t>VCLT</t>
+  </si>
+  <si>
+    <t>SPSB</t>
+  </si>
+  <si>
+    <t>VWOB</t>
+  </si>
+  <si>
     <t>FLCA</t>
   </si>
   <si>
+    <t>EMB</t>
+  </si>
+  <si>
     <t>ICVT</t>
   </si>
   <si>
-    <t>VWOB</t>
-  </si>
-  <si>
-    <t>EMB</t>
-  </si>
-  <si>
-    <t>VMBS</t>
-  </si>
-  <si>
-    <t>SPSB</t>
-  </si>
-  <si>
-    <t>VCLT</t>
+    <t>VCIT</t>
   </si>
   <si>
     <t>IVV</t>
   </si>
   <si>
     <t>HYD</t>
-  </si>
-  <si>
-    <t>VCIT</t>
   </si>
   <si>
     <t>FAST - Monitor costs carefully</t>
@@ -607,31 +607,31 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>36.21314297445958</v>
+        <v>35.53105077922309</v>
       </c>
       <c r="C2">
-        <v>6.958799466197416</v>
+        <v>7.092388051393005</v>
       </c>
       <c r="D2">
-        <v>0.9941142094567736</v>
+        <v>1.013198293056144</v>
       </c>
       <c r="E2">
-        <v>376.528993055139</v>
+        <v>131.8867283787759</v>
       </c>
       <c r="F2">
-        <v>214701.8392612503</v>
+        <v>73861.45277507885</v>
       </c>
       <c r="G2">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H2">
-        <v>0.3621314297445958</v>
+        <v>0.3553105077922309</v>
       </c>
       <c r="I2">
-        <v>-123.5074635009766</v>
+        <v>329.4358236083984</v>
       </c>
       <c r="J2">
-        <v>0.2932061103673564</v>
+        <v>0.1078542411995211</v>
       </c>
       <c r="K2" t="s">
         <v>43</v>
@@ -645,31 +645,31 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>35.73983427744304</v>
+        <v>34.79646375761699</v>
       </c>
       <c r="C3">
-        <v>7.05095602972754</v>
+        <v>7.242115226287524</v>
       </c>
       <c r="D3">
-        <v>1.00727943281822</v>
+        <v>1.034587889469646</v>
       </c>
       <c r="E3">
-        <v>4706.176142795722</v>
+        <v>862.9825075746202</v>
       </c>
       <c r="F3">
-        <v>2648450.345723546</v>
+        <v>473310.1328799962</v>
       </c>
       <c r="G3">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H3">
-        <v>0.3573983427744304</v>
+        <v>0.3479646375761699</v>
       </c>
       <c r="I3">
-        <v>93.64753532409668</v>
+        <v>650.1611022949219</v>
       </c>
       <c r="J3">
-        <v>0.3816420170990526</v>
+        <v>0.0535197563108487</v>
       </c>
       <c r="K3" t="s">
         <v>43</v>
@@ -683,31 +683,31 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>35.28818078629894</v>
+        <v>33.96942874910513</v>
       </c>
       <c r="C4">
-        <v>7.14120122899172</v>
+        <v>7.418435024658416</v>
       </c>
       <c r="D4">
-        <v>1.020171604141674</v>
+        <v>1.059776432094059</v>
       </c>
       <c r="E4">
-        <v>997.211981073113</v>
+        <v>1427.11614430399</v>
       </c>
       <c r="F4">
-        <v>554099.6555080692</v>
+        <v>764110.6657042472</v>
       </c>
       <c r="G4">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H4">
-        <v>0.3528818078629894</v>
+        <v>0.3396942874910513</v>
       </c>
       <c r="I4">
-        <v>-92.20262858581543</v>
+        <v>347.6228561401367</v>
       </c>
       <c r="J4">
-        <v>0.3827242382081905</v>
+        <v>0.09771920387021699</v>
       </c>
       <c r="K4" t="s">
         <v>43</v>
@@ -721,31 +721,31 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>34.28474383414597</v>
+        <v>32.76553843508282</v>
       </c>
       <c r="C5">
-        <v>7.350208046443679</v>
+        <v>7.691007443667635</v>
       </c>
       <c r="D5">
-        <v>1.050029720920526</v>
+        <v>1.098715349095376</v>
       </c>
       <c r="E5">
-        <v>985.7482380290448</v>
+        <v>961.412190755196</v>
       </c>
       <c r="F5">
-        <v>532154.8701457183</v>
+        <v>496518.7265322147</v>
       </c>
       <c r="G5">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H5">
-        <v>0.3428474383414597</v>
+        <v>0.3276553843508282</v>
       </c>
       <c r="I5">
-        <v>-198.7971412353516</v>
+        <v>260</v>
       </c>
       <c r="J5">
-        <v>0.1724609499970476</v>
+        <v>0.1260213016733955</v>
       </c>
       <c r="K5" t="s">
         <v>43</v>
@@ -759,31 +759,31 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>34.00927271614375</v>
+        <v>32.46534136057391</v>
       </c>
       <c r="C6">
-        <v>7.409743869070713</v>
+        <v>7.762123835421309</v>
       </c>
       <c r="D6">
-        <v>1.058534838438673</v>
+        <v>1.108874833631616</v>
       </c>
       <c r="E6">
-        <v>2744.198336791616</v>
+        <v>1360.199099013959</v>
       </c>
       <c r="F6">
-        <v>1469548.636605541</v>
+        <v>641011.1986989444</v>
       </c>
       <c r="G6">
-        <v>1984</v>
+        <v>1829</v>
       </c>
       <c r="H6">
-        <v>0.3400927271614375</v>
+        <v>0.3246534136057391</v>
       </c>
       <c r="I6">
-        <v>-282.6376909179788</v>
+        <v>1919.777921386719</v>
       </c>
       <c r="J6">
-        <v>0.120328157952625</v>
+        <v>0.01691098798402844</v>
       </c>
       <c r="K6" t="s">
         <v>43</v>
@@ -797,31 +797,31 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>33.25811346615763</v>
+        <v>31.72232097291986</v>
       </c>
       <c r="C7">
-        <v>7.57709845016997</v>
+        <v>7.943933239157464</v>
       </c>
       <c r="D7">
-        <v>1.082442635738567</v>
+        <v>1.134847605593923</v>
       </c>
       <c r="E7">
-        <v>7622.283821387688</v>
+        <v>7395.352574495175</v>
       </c>
       <c r="F7">
-        <v>3991662.824783263</v>
+        <v>3697707.36253195</v>
       </c>
       <c r="G7">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H7">
-        <v>0.3325811346615763</v>
+        <v>0.3172232097291986</v>
       </c>
       <c r="I7">
-        <v>-288.3928489685059</v>
+        <v>410.0483374328369</v>
       </c>
       <c r="J7">
-        <v>0.1153222542969143</v>
+        <v>0.07736239383756983</v>
       </c>
       <c r="K7" t="s">
         <v>43</v>
@@ -835,31 +835,31 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>32.5107725123483</v>
+        <v>31.45381835686403</v>
       </c>
       <c r="C8">
-        <v>7.751276900734516</v>
+        <v>8.011745891735497</v>
       </c>
       <c r="D8">
-        <v>1.107325271533502</v>
+        <v>1.144535127390785</v>
       </c>
       <c r="E8">
-        <v>1504.363153432152</v>
+        <v>5304.666532342906</v>
       </c>
       <c r="F8">
-        <v>770107.0506529219</v>
+        <v>2629905.609987067</v>
       </c>
       <c r="G8">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H8">
-        <v>0.325107725123483</v>
+        <v>0.3145381835686403</v>
       </c>
       <c r="I8">
-        <v>699.8680000000001</v>
+        <v>329.6970653533936</v>
       </c>
       <c r="J8">
-        <v>0.04645272038777068</v>
+        <v>0.09540217873383107</v>
       </c>
       <c r="K8" t="s">
         <v>43</v>
@@ -873,31 +873,31 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>32.24172325795473</v>
+        <v>31.09978841063272</v>
       </c>
       <c r="C9">
-        <v>7.815959400923961</v>
+        <v>8.102949019223669</v>
       </c>
       <c r="D9">
-        <v>1.116565628703423</v>
+        <v>1.157564145603381</v>
       </c>
       <c r="E9">
-        <v>36411.52575049087</v>
+        <v>320.8105489799257</v>
       </c>
       <c r="F9">
-        <v>18485374.18974669</v>
+        <v>157258.7335209904</v>
       </c>
       <c r="G9">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H9">
-        <v>0.3224172325795473</v>
+        <v>0.3109978841063272</v>
       </c>
       <c r="I9">
-        <v>-201.9405915985107</v>
+        <v>-40.57173899841309</v>
       </c>
       <c r="J9">
-        <v>0.1596594473787434</v>
+        <v>0.7665382154767668</v>
       </c>
       <c r="K9" t="s">
         <v>43</v>
@@ -911,31 +911,31 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>32.17454412208342</v>
+        <v>30.7490083596401</v>
       </c>
       <c r="C10">
-        <v>7.832278805375101</v>
+        <v>8.195386239862126</v>
       </c>
       <c r="D10">
-        <v>1.118896972196443</v>
+        <v>1.170769462837447</v>
       </c>
       <c r="E10">
-        <v>457.8427425093408</v>
+        <v>370.8194555764189</v>
       </c>
       <c r="F10">
-        <v>213597.7820377157</v>
+        <v>179722.4480263562</v>
       </c>
       <c r="G10">
-        <v>1827</v>
+        <v>1986</v>
       </c>
       <c r="H10">
-        <v>0.3217454412208342</v>
+        <v>0.3074900835964011</v>
       </c>
       <c r="I10">
-        <v>19.60169787597656</v>
+        <v>237.601318359375</v>
       </c>
       <c r="J10">
-        <v>1.641416183723344</v>
+        <v>0.1294143002739229</v>
       </c>
       <c r="K10" t="s">
         <v>43</v>
@@ -949,31 +949,31 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>31.15333849933335</v>
+        <v>30.6411366691306</v>
       </c>
       <c r="C11">
-        <v>8.089020700153613</v>
+        <v>8.224237981806899</v>
       </c>
       <c r="D11">
-        <v>1.15557438573623</v>
+        <v>1.174891140258129</v>
       </c>
       <c r="E11">
-        <v>2047.373673141135</v>
+        <v>6907.978694227357</v>
       </c>
       <c r="F11">
-        <v>1004321.664657101</v>
+        <v>3336295.889560665</v>
       </c>
       <c r="G11">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H11">
-        <v>0.3115333849933336</v>
+        <v>0.306411366691306</v>
       </c>
       <c r="I11">
-        <v>475.9476782226562</v>
+        <v>61.79141426086426</v>
       </c>
       <c r="J11">
-        <v>0.06545538496094797</v>
+        <v>0.4958801645123899</v>
       </c>
       <c r="K11" t="s">
         <v>43</v>
@@ -987,31 +987,31 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.62816309239676</v>
+        <v>30.19005749576751</v>
       </c>
       <c r="C12">
-        <v>8.227721631224998</v>
+        <v>8.347118916064638</v>
       </c>
       <c r="D12">
-        <v>1.175388804460714</v>
+        <v>1.192445559437805</v>
       </c>
       <c r="E12">
-        <v>1922.328235984836</v>
+        <v>1786.025231053582</v>
       </c>
       <c r="F12">
-        <v>927085.1375719371</v>
+        <v>849885.1267221952</v>
       </c>
       <c r="G12">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H12">
-        <v>0.3062816309239677</v>
+        <v>0.3019005749576751</v>
       </c>
       <c r="I12">
-        <v>-23.32112231445312</v>
+        <v>1347.286296508789</v>
       </c>
       <c r="J12">
-        <v>1.313322861542352</v>
+        <v>0.02240804910878908</v>
       </c>
       <c r="K12" t="s">
         <v>43</v>
@@ -1025,31 +1025,31 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.03209660063617</v>
+        <v>30.060948377805</v>
       </c>
       <c r="C13">
-        <v>8.391022556668982</v>
+        <v>8.382969054497961</v>
       </c>
       <c r="D13">
-        <v>1.198717508095569</v>
+        <v>1.197567007785423</v>
       </c>
       <c r="E13">
-        <v>1919.059339413511</v>
+        <v>1702.494331473112</v>
       </c>
       <c r="F13">
-        <v>907496.9596811212</v>
+        <v>806672.1278164352</v>
       </c>
       <c r="G13">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H13">
-        <v>0.3003209660063617</v>
+        <v>0.30060948377805</v>
       </c>
       <c r="I13">
-        <v>-79.87465667724609</v>
+        <v>-0.246</v>
       </c>
       <c r="J13">
-        <v>0.3759903059363186</v>
+        <v>122.1989771455488</v>
       </c>
       <c r="K13" t="s">
         <v>43</v>
@@ -1063,31 +1063,31 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.86701921753074</v>
+        <v>29.92529558764737</v>
       </c>
       <c r="C14">
-        <v>8.437400403589191</v>
+        <v>8.420969452479564</v>
       </c>
       <c r="D14">
-        <v>1.205342914798456</v>
+        <v>1.202995636068509</v>
       </c>
       <c r="E14">
-        <v>375.4805258440902</v>
+        <v>427.380886537042</v>
       </c>
       <c r="F14">
-        <v>176583.6223578482</v>
+        <v>201586.870835315</v>
       </c>
       <c r="G14">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H14">
-        <v>0.2986701921753074</v>
+        <v>0.2992529558764737</v>
       </c>
       <c r="I14">
-        <v>-31.90471960449219</v>
+        <v>-23.54904174804688</v>
       </c>
       <c r="J14">
-        <v>0.9361316942376596</v>
+        <v>1.270764895991122</v>
       </c>
       <c r="K14" t="s">
         <v>43</v>
@@ -1101,31 +1101,31 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.72922449361318</v>
+        <v>29.81229920922454</v>
       </c>
       <c r="C15">
-        <v>8.476507688726892</v>
+        <v>8.452887119891308</v>
       </c>
       <c r="D15">
-        <v>1.210929669818128</v>
+        <v>1.207555302841615</v>
       </c>
       <c r="E15">
-        <v>3512.913313264904</v>
+        <v>756.5529725517482</v>
       </c>
       <c r="F15">
-        <v>1644455.539817803</v>
+        <v>355503.1984165647</v>
       </c>
       <c r="G15">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H15">
-        <v>0.2972922449361318</v>
+        <v>0.2981229920922455</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>1267.498016357422</v>
       </c>
       <c r="J15">
-        <v>0</v>
+        <v>0.02352058845417378</v>
       </c>
       <c r="K15" t="s">
         <v>43</v>
@@ -1139,31 +1139,31 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.26797135488714</v>
+        <v>28.37034549788314</v>
       </c>
       <c r="C16">
-        <v>8.914682869750139</v>
+        <v>8.882514314772903</v>
       </c>
       <c r="D16">
-        <v>1.27352612425002</v>
+        <v>1.268930616396129</v>
       </c>
       <c r="E16">
-        <v>4114.092036692101</v>
+        <v>353.982020614</v>
       </c>
       <c r="F16">
-        <v>1831216.818378174</v>
+        <v>158290.3822108566</v>
       </c>
       <c r="G16">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H16">
-        <v>0.2826797135488714</v>
+        <v>0.2837034549788314</v>
       </c>
       <c r="I16">
-        <v>88.7705174560388</v>
+        <v>-0.979995880126953</v>
       </c>
       <c r="J16">
-        <v>0.3184387357985841</v>
+        <v>28.94945384281403</v>
       </c>
       <c r="K16" t="s">
         <v>43</v>
@@ -1177,31 +1177,31 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.47384700758074</v>
+        <v>28.04668130067836</v>
       </c>
       <c r="C17">
-        <v>9.172359441707115</v>
+        <v>8.985020270255822</v>
       </c>
       <c r="D17">
-        <v>1.310337063101016</v>
+        <v>1.28357432432226</v>
       </c>
       <c r="E17">
-        <v>1607.683194958874</v>
+        <v>1332.027958693151</v>
       </c>
       <c r="F17">
-        <v>695490.2888552226</v>
+        <v>588848.4269138499</v>
       </c>
       <c r="G17">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H17">
-        <v>0.2747384700758074</v>
+        <v>0.2804668130067836</v>
       </c>
       <c r="I17">
-        <v>-86.12577548219299</v>
+        <v>474.6198309326172</v>
       </c>
       <c r="J17">
-        <v>0.3189968026849421</v>
+        <v>0.05909294022874534</v>
       </c>
       <c r="K17" t="s">
         <v>43</v>
@@ -1215,31 +1215,31 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>26.17281989001769</v>
+        <v>27.91093853595413</v>
       </c>
       <c r="C18">
-        <v>9.628309103067368</v>
+        <v>9.028718245191946</v>
       </c>
       <c r="D18">
-        <v>1.375472729009624</v>
+        <v>1.289816892170278</v>
       </c>
       <c r="E18">
-        <v>2321.120693690204</v>
+        <v>10275.01718887366</v>
       </c>
       <c r="F18">
-        <v>956575.7407630963</v>
+        <v>4520283.739714653</v>
       </c>
       <c r="G18">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H18">
-        <v>0.2617281989001769</v>
+        <v>0.2791093853595413</v>
       </c>
       <c r="I18">
-        <v>228.6002487182617</v>
+        <v>285.0876213226318</v>
       </c>
       <c r="J18">
-        <v>0.1144916509792357</v>
+        <v>0.09790301804920355</v>
       </c>
       <c r="K18" t="s">
         <v>43</v>
@@ -1253,31 +1253,31 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>25.6883257658199</v>
+        <v>27.81889025807012</v>
       </c>
       <c r="C19">
-        <v>9.809903623042006</v>
+        <v>9.058592836099782</v>
       </c>
       <c r="D19">
-        <v>1.401414803291715</v>
+        <v>1.294084690871397</v>
       </c>
       <c r="E19">
-        <v>326.5749147811169</v>
+        <v>1548.727921231333</v>
       </c>
       <c r="F19">
-        <v>132096.0237374518</v>
+        <v>679084.2037425573</v>
       </c>
       <c r="G19">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H19">
-        <v>0.256883257658199</v>
+        <v>0.2781889025807012</v>
       </c>
       <c r="I19">
-        <v>5.388</v>
+        <v>-132.5408213348389</v>
       </c>
       <c r="J19">
-        <v>4.767692235675558</v>
+        <v>0.2098892249037075</v>
       </c>
       <c r="K19" t="s">
         <v>43</v>
@@ -1291,31 +1291,31 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>25.51859381286541</v>
+        <v>26.92235337367029</v>
       </c>
       <c r="C20">
-        <v>9.875152284956711</v>
+        <v>9.360251553879859</v>
       </c>
       <c r="D20">
-        <v>1.410736040708102</v>
+        <v>1.337178793411409</v>
       </c>
       <c r="E20">
-        <v>4524.742566357086</v>
+        <v>2173.882830181468</v>
       </c>
       <c r="F20">
-        <v>1818116.620910785</v>
+        <v>922481.8961090518</v>
       </c>
       <c r="G20">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H20">
-        <v>0.2551859381286541</v>
+        <v>0.2692235337367029</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>1400.558096313477</v>
       </c>
       <c r="J20">
-        <v>0</v>
+        <v>0.01922258951237711</v>
       </c>
       <c r="K20" t="s">
         <v>43</v>
@@ -1329,31 +1329,31 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>24.34935314196738</v>
+        <v>26.58743165837271</v>
       </c>
       <c r="C21">
-        <v>10.34935090598628</v>
+        <v>9.478162585916497</v>
       </c>
       <c r="D21">
-        <v>1.478478700855183</v>
+        <v>1.3540232265595</v>
       </c>
       <c r="E21">
-        <v>2851.630828696694</v>
+        <v>1030.095512779254</v>
       </c>
       <c r="F21">
-        <v>1093331.478568718</v>
+        <v>431680.6490362142</v>
       </c>
       <c r="G21">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H21">
-        <v>0.2434935314196738</v>
+        <v>0.2658743165837271</v>
       </c>
       <c r="I21">
-        <v>-70.15822219843648</v>
+        <v>87.86901187133789</v>
       </c>
       <c r="J21">
-        <v>0.3470634286184923</v>
+        <v>0.3025802964223989</v>
       </c>
       <c r="K21" t="s">
         <v>43</v>
@@ -1367,31 +1367,31 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>24.21616657915808</v>
+        <v>25.6455933751288</v>
       </c>
       <c r="C22">
-        <v>10.40627133019834</v>
+        <v>9.826249535890662</v>
       </c>
       <c r="D22">
-        <v>1.486610190028334</v>
+        <v>1.403749933698666</v>
       </c>
       <c r="E22">
-        <v>4010.859435164335</v>
+        <v>639.1384303605672</v>
       </c>
       <c r="F22">
-        <v>1529374.906124876</v>
+        <v>258354.7096091598</v>
       </c>
       <c r="G22">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H22">
-        <v>0.2421616657915809</v>
+        <v>0.256455933751288</v>
       </c>
       <c r="I22">
-        <v>-128.6229438781738</v>
+        <v>76.79066491699218</v>
       </c>
       <c r="J22">
-        <v>0.1882725262616801</v>
+        <v>0.3339675910196991</v>
       </c>
       <c r="K22" t="s">
         <v>43</v>
@@ -1405,31 +1405,31 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>23.53697886600697</v>
+        <v>25.42183042278921</v>
       </c>
       <c r="C23">
-        <v>10.70655675202005</v>
+        <v>9.912740184675942</v>
       </c>
       <c r="D23">
-        <v>1.529508107431435</v>
+        <v>1.416105740667992</v>
       </c>
       <c r="E23">
-        <v>1733.483412139244</v>
+        <v>3715.291070653996</v>
       </c>
       <c r="F23">
-        <v>642453.2497874013</v>
+        <v>1488704.017023533</v>
       </c>
       <c r="G23">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H23">
-        <v>0.2353697886600697</v>
+        <v>0.2542183042278922</v>
       </c>
       <c r="I23">
-        <v>-51.9349033203125</v>
+        <v>-197.96314062502</v>
       </c>
       <c r="J23">
-        <v>0.4532015535071057</v>
+        <v>0.1284169888521976</v>
       </c>
       <c r="K23" t="s">
         <v>43</v>
@@ -1443,31 +1443,31 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>23.4126027926713</v>
+        <v>25.00347188885532</v>
       </c>
       <c r="C24">
-        <v>10.76343378955209</v>
+        <v>10.07860032879365</v>
       </c>
       <c r="D24">
-        <v>1.537633398507442</v>
+        <v>1.439800046970521</v>
       </c>
       <c r="E24">
-        <v>767.7623955056337</v>
+        <v>876.1939186406656</v>
       </c>
       <c r="F24">
-        <v>283039.8964616226</v>
+        <v>345310.0759336578</v>
       </c>
       <c r="G24">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H24">
-        <v>0.234126027926713</v>
+        <v>0.2500347188885532</v>
       </c>
       <c r="I24">
-        <v>-76.76021575927734</v>
+        <v>-0.042</v>
       </c>
       <c r="J24">
-        <v>0.3050096011466932</v>
+        <v>595.32075925846</v>
       </c>
       <c r="K24" t="s">
         <v>43</v>
@@ -1481,31 +1481,31 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>23.19777916236094</v>
+        <v>24.89364732160354</v>
       </c>
       <c r="C25">
-        <v>10.86310884487069</v>
+        <v>10.12306460135739</v>
       </c>
       <c r="D25">
-        <v>1.551872692124384</v>
+        <v>1.446152085908199</v>
       </c>
       <c r="E25">
-        <v>578.4011068633512</v>
+        <v>196.2200725990104</v>
       </c>
       <c r="F25">
-        <v>211274.2884940778</v>
+        <v>76991.12463025894</v>
       </c>
       <c r="G25">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H25">
-        <v>0.2319777916236094</v>
+        <v>0.2489364732160354</v>
       </c>
       <c r="I25">
-        <v>-162.9592895507592</v>
+        <v>-0.008</v>
       </c>
       <c r="J25">
-        <v>0.1423532173361323</v>
+        <v>3111.705915200442</v>
       </c>
       <c r="K25" t="s">
         <v>43</v>
@@ -1519,31 +1519,31 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>22.07828457384698</v>
+        <v>24.7140392990936</v>
       </c>
       <c r="C26">
-        <v>11.41393024250211</v>
+        <v>10.19663345802166</v>
       </c>
       <c r="D26">
-        <v>1.630561463214588</v>
+        <v>1.456661922574523</v>
       </c>
       <c r="E26">
-        <v>1129.980905137649</v>
+        <v>4432.801795592814</v>
       </c>
       <c r="F26">
-        <v>392832.6296309376</v>
+        <v>1726755.090744506</v>
       </c>
       <c r="G26">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H26">
-        <v>0.2207828457384698</v>
+        <v>0.247140392990936</v>
       </c>
       <c r="I26">
-        <v>-19.08604815673828</v>
+        <v>87.00199127198812</v>
       </c>
       <c r="J26">
-        <v>1.156776111667323</v>
+        <v>0.2840629155467472</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -1557,31 +1557,31 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>21.76511615073989</v>
+        <v>24.34048680833812</v>
       </c>
       <c r="C27">
-        <v>11.57816012810175</v>
+        <v>10.35312078941964</v>
       </c>
       <c r="D27">
-        <v>1.654022875443107</v>
+        <v>1.479017255631378</v>
       </c>
       <c r="E27">
-        <v>658.3919745351714</v>
+        <v>1149.286758102964</v>
       </c>
       <c r="F27">
-        <v>225640.2853346857</v>
+        <v>440926.6631806454</v>
       </c>
       <c r="G27">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H27">
-        <v>0.2176511615073989</v>
+        <v>0.2434048680833812</v>
       </c>
       <c r="I27">
-        <v>-0.063</v>
+        <v>430.4526871948242</v>
       </c>
       <c r="J27">
-        <v>345.4780341387284</v>
+        <v>0.05654625358935568</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -1595,34 +1595,34 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>19.63833841116994</v>
+        <v>24.19983584259504</v>
       </c>
       <c r="C28">
-        <v>12.83204285025799</v>
+        <v>10.41329377765635</v>
       </c>
       <c r="D28">
-        <v>1.833148978608284</v>
+        <v>1.48761339680805</v>
       </c>
       <c r="E28">
-        <v>1990.968381652041</v>
+        <v>1005.15506470526</v>
       </c>
       <c r="F28">
-        <v>615658.9898105327</v>
+        <v>383401.8325283293</v>
       </c>
       <c r="G28">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H28">
-        <v>0.1963833841116994</v>
+        <v>0.2419983584259504</v>
       </c>
       <c r="I28">
-        <v>-170.6402893066406</v>
+        <v>155.2505493164062</v>
       </c>
       <c r="J28">
-        <v>0.1150861762539551</v>
+        <v>0.1558760078412019</v>
       </c>
       <c r="K28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L28" t="s">
         <v>45</v>
@@ -1633,34 +1633,34 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>19.45954343617745</v>
+        <v>23.91022815399812</v>
       </c>
       <c r="C29">
-        <v>12.94994411490169</v>
+        <v>10.53942264276814</v>
       </c>
       <c r="D29">
-        <v>1.849992016414527</v>
+        <v>1.505631806109734</v>
       </c>
       <c r="E29">
-        <v>15618.7559873286</v>
+        <v>1393.811191059378</v>
       </c>
       <c r="F29">
-        <v>4785752.216984787</v>
+        <v>525286.6535992508</v>
       </c>
       <c r="G29">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H29">
-        <v>0.1945954343617745</v>
+        <v>0.2391022815399812</v>
       </c>
       <c r="I29">
-        <v>-451.6016235352632</v>
+        <v>619.2100501098632</v>
       </c>
       <c r="J29">
-        <v>0.04309006527443973</v>
+        <v>0.03861408281366856</v>
       </c>
       <c r="K29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L29" t="s">
         <v>45</v>
@@ -1671,34 +1671,34 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>18.40133434703328</v>
+        <v>22.2948038443046</v>
       </c>
       <c r="C30">
-        <v>13.69465905284353</v>
+        <v>11.30308217824377</v>
       </c>
       <c r="D30">
-        <v>1.956379864691933</v>
+        <v>1.614726025463396</v>
       </c>
       <c r="E30">
-        <v>501.1842812396358</v>
+        <v>120.3584006634644</v>
       </c>
       <c r="F30">
-        <v>145217.1405133262</v>
+        <v>42294.97405189708</v>
       </c>
       <c r="G30">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H30">
-        <v>0.1840133434703329</v>
+        <v>0.222948038443046</v>
       </c>
       <c r="I30">
-        <v>-160.1418685913086</v>
+        <v>91.95933532714672</v>
       </c>
       <c r="J30">
-        <v>0.1149064545637004</v>
+        <v>0.2424419855253466</v>
       </c>
       <c r="K30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L30" t="s">
         <v>45</v>
@@ -1709,37 +1709,37 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>17.82625918535862</v>
+        <v>21.84530409795105</v>
       </c>
       <c r="C31">
-        <v>14.13644878489016</v>
+        <v>11.5356599693037</v>
       </c>
       <c r="D31">
-        <v>2.019492683555738</v>
+        <v>1.647951424186243</v>
       </c>
       <c r="E31">
-        <v>51.45918685153374</v>
+        <v>492.7358766665794</v>
       </c>
       <c r="F31">
-        <v>14444.22545817417</v>
+        <v>169660.5922268519</v>
       </c>
       <c r="G31">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H31">
-        <v>1.42610073482869</v>
+        <v>0.2184530409795105</v>
       </c>
       <c r="I31">
-        <v>221.2568876953125</v>
+        <v>57.72181359863281</v>
       </c>
       <c r="J31">
-        <v>0.6445452386515254</v>
+        <v>0.3784583805673852</v>
       </c>
       <c r="K31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1747,31 +1747,31 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.01604057835124</v>
+        <v>17.39791500300628</v>
       </c>
       <c r="C32">
-        <v>14.80955565659666</v>
+        <v>14.48449426017172</v>
       </c>
       <c r="D32">
-        <v>2.115650808085238</v>
+        <v>2.069213465738817</v>
       </c>
       <c r="E32">
-        <v>3427.415523779759</v>
+        <v>297.6602621210547</v>
       </c>
       <c r="F32">
-        <v>918324.9729913536</v>
+        <v>81625.67086624759</v>
       </c>
       <c r="G32">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H32">
-        <v>0.1701604057835124</v>
+        <v>1.391833200240503</v>
       </c>
       <c r="I32">
-        <v>-7.8607646484375</v>
+        <v>1879.27271484375</v>
       </c>
       <c r="J32">
-        <v>2.164680071134499</v>
+        <v>0.07406233215897166</v>
       </c>
       <c r="K32" t="s">
         <v>44</v>
@@ -1785,31 +1785,31 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>15.94412501775627</v>
+        <v>16.81460346266623</v>
       </c>
       <c r="C33">
-        <v>15.80519468577666</v>
+        <v>14.98697251823512</v>
       </c>
       <c r="D33">
-        <v>2.257884955110951</v>
+        <v>2.140996074033589</v>
       </c>
       <c r="E33">
-        <v>1277.312846760583</v>
+        <v>467.1058987220708</v>
       </c>
       <c r="F33">
-        <v>320677.9465049618</v>
+        <v>123797.1596642757</v>
       </c>
       <c r="G33">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="H33">
-        <v>0.1594412501775627</v>
+        <v>0.1681460346266623</v>
       </c>
       <c r="I33">
-        <v>-266.0688400268555</v>
+        <v>4.550228118896484</v>
       </c>
       <c r="J33">
-        <v>0.05992481124864888</v>
+        <v>3.695331975299755</v>
       </c>
       <c r="K33" t="s">
         <v>44</v>
@@ -1854,163 +1854,163 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B2">
-        <v>1816</v>
+        <v>1818</v>
       </c>
       <c r="C2">
-        <v>1827</v>
+        <v>1829</v>
       </c>
       <c r="D2">
-        <v>99.39792008757526</v>
+        <v>99.39857845817387</v>
       </c>
       <c r="E2">
-        <v>1.006057268722467</v>
+        <v>1.006050605060506</v>
       </c>
       <c r="F2">
-        <v>1309.354961445546</v>
+        <v>2536.041290790004</v>
       </c>
       <c r="G2">
-        <v>117.6199240295791</v>
+        <v>352.5914184262621</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B3">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C3">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D3">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E3">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F3">
-        <v>4582.675348167124</v>
+        <v>17582.04604487296</v>
       </c>
       <c r="G3">
-        <v>460.4246370781944</v>
+        <v>1874.15477067002</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C4">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D4">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E4">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F4">
-        <v>2781.268481942817</v>
+        <v>905.6567427295582</v>
       </c>
       <c r="G4">
-        <v>352.8616381812393</v>
+        <v>102.1727677827243</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C5">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D5">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E5">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F5">
-        <v>1196.430677875789</v>
+        <v>2100.564521639196</v>
       </c>
       <c r="G5">
-        <v>114.4801041779227</v>
+        <v>266.2375335019011</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C6">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D6">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E6">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F6">
-        <v>7456.82645249261</v>
+        <v>2743.223889893975</v>
       </c>
       <c r="G6">
-        <v>485.3250841010128</v>
+        <v>298.4533334586163</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C7">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D7">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E7">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F7">
-        <v>19144.4970439702</v>
+        <v>3090.909441674646</v>
       </c>
       <c r="G7">
-        <v>1343.708952675569</v>
+        <v>387.2836622930802</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C8">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D8">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E8">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F8">
-        <v>4145.298474922745</v>
+        <v>596.0671506925451</v>
       </c>
       <c r="G8">
-        <v>509.5492971370375</v>
+        <v>91.09095186333313</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2018,114 +2018,114 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C9">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D9">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E9">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F9">
-        <v>869.7836593477695</v>
+        <v>231.6689697663349</v>
       </c>
       <c r="G9">
-        <v>108.9304105840945</v>
+        <v>37.43611392553414</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B10">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C10">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D10">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E10">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F10">
-        <v>2359.294185075335</v>
+        <v>2102.064972948719</v>
       </c>
       <c r="G10">
-        <v>143.6021798384691</v>
+        <v>194.3242942363554</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C11">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D11">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E11">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F11">
-        <v>4229.710079622043</v>
+        <v>2999.740855127723</v>
       </c>
       <c r="G11">
-        <v>390.7189501029537</v>
+        <v>430.7577935743514</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12">
-        <v>1461</v>
+        <v>1463</v>
       </c>
       <c r="C12">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D12">
-        <v>73.63911290322581</v>
+        <v>73.66565961732124</v>
       </c>
       <c r="E12">
-        <v>1.357973990417522</v>
+        <v>1.357484620642515</v>
       </c>
       <c r="F12">
-        <v>6804.085959017637</v>
+        <v>840.4108043968342</v>
       </c>
       <c r="G12">
-        <v>628.5591875368608</v>
+        <v>84.61870106922466</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C13">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D13">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E13">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F13">
-        <v>5512.163928441823</v>
+        <v>1268.804664388339</v>
       </c>
       <c r="G13">
-        <v>554.7090200754529</v>
+        <v>130.9451138414393</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2133,436 +2133,436 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C14">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D14">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E14">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F14">
-        <v>3490.068189659779</v>
+        <v>7459.477721260409</v>
       </c>
       <c r="G14">
-        <v>325.9529425608327</v>
+        <v>754.5382752273355</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B15">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C15">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D15">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E15">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F15">
-        <v>1322.750416786489</v>
+        <v>235.6504768447492</v>
       </c>
       <c r="G15">
-        <v>107.1914198346412</v>
+        <v>21.43688497308519</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C16">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D16">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E16">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F16">
-        <v>754.6518248072589</v>
+        <v>1413.16313193184</v>
       </c>
       <c r="G16">
-        <v>89.59087892331215</v>
+        <v>180.1840843469664</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C17">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D17">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E17">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F17">
-        <v>6486.89871742941</v>
+        <v>19503.35133428763</v>
       </c>
       <c r="G17">
-        <v>929.0800702070896</v>
+        <v>2291.071332850813</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C18">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D18">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E18">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F18">
-        <v>2117.104317135825</v>
+        <v>1887.403594098616</v>
       </c>
       <c r="G18">
-        <v>281.1261570309838</v>
+        <v>239.8936304510878</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19">
-        <v>1461</v>
+        <v>1463</v>
       </c>
       <c r="C19">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D19">
-        <v>73.63911290322581</v>
+        <v>73.66565961732124</v>
       </c>
       <c r="E19">
-        <v>1.357973990417522</v>
+        <v>1.357484620642515</v>
       </c>
       <c r="F19">
-        <v>128.5793504955643</v>
+        <v>582.3511021391829</v>
       </c>
       <c r="G19">
-        <v>9.886533510043927</v>
+        <v>55.79334987440026</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C20">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D20">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E20">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F20">
-        <v>8084.482118516435</v>
+        <v>719.4238656769149</v>
       </c>
       <c r="G20">
-        <v>834.3254895067491</v>
+        <v>80.22827278806723</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B21">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C21">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D21">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E21">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F21">
-        <v>4929.689824844304</v>
+        <v>10717.19405479059</v>
       </c>
       <c r="G21">
-        <v>470.3628298183344</v>
+        <v>1332.947597560602</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B22">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C22">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D22">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E22">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F22">
-        <v>110891.2995462922</v>
+        <v>19361.52035938888</v>
       </c>
       <c r="G22">
-        <v>9378.677924782693</v>
+        <v>1690.976122433181</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B23">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C23">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D23">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E23">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F23">
-        <v>12308.97177991711</v>
+        <v>2775.931924451952</v>
       </c>
       <c r="G23">
-        <v>775.9385622145492</v>
+        <v>344.1886486277533</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C24">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D24">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E24">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F24">
-        <v>21177.74632497273</v>
+        <v>4167.663546269498</v>
       </c>
       <c r="G24">
-        <v>2025.196765491255</v>
+        <v>408.8556147067588</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C25">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D25">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E25">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F25">
-        <v>9243.003368178152</v>
+        <v>1982.304259946316</v>
       </c>
       <c r="G25">
-        <v>922.4335976208957</v>
+        <v>218.7940441136413</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B26">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C26">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D26">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E26">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F26">
-        <v>82819.67182870273</v>
+        <v>8032.797503369997</v>
       </c>
       <c r="G26">
-        <v>2428.083316582845</v>
+        <v>875.1926460945291</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B27">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C27">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D27">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E27">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F27">
-        <v>8390.864246806283</v>
+        <v>687.3233793479387</v>
       </c>
       <c r="G27">
-        <v>745.5853052285848</v>
+        <v>79.7053895190017</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B28">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C28">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D28">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E28">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F28">
-        <v>3365.908958623802</v>
+        <v>679.7965490388582</v>
       </c>
       <c r="G28">
-        <v>162.69809563925</v>
+        <v>85.99117700296598</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B29">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C29">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D29">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E29">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F29">
-        <v>1182.684939504984</v>
+        <v>310.2230419140228</v>
       </c>
       <c r="G29">
-        <v>73.676885090475</v>
+        <v>39.02236423226505</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C30">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D30">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E30">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F30">
-        <v>537.3479611693675</v>
+        <v>3004.951472180855</v>
       </c>
       <c r="G30">
-        <v>67.01979895355245</v>
+        <v>467.5529123715417</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B31">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C31">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D31">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E31">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F31">
-        <v>3041.368145783164</v>
+        <v>1975.074870176226</v>
       </c>
       <c r="G31">
-        <v>312.3586959972261</v>
+        <v>175.017777969416</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B32">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C32">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D32">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E32">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F32">
-        <v>2787.922068767069</v>
+        <v>2058.969043256369</v>
       </c>
       <c r="G32">
-        <v>199.3062555205163</v>
+        <v>223.4803158543565</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2570,22 +2570,22 @@
         <v>14</v>
       </c>
       <c r="B33">
-        <v>1971</v>
+        <v>1973</v>
       </c>
       <c r="C33">
-        <v>1984</v>
+        <v>1986</v>
       </c>
       <c r="D33">
-        <v>99.34475806451613</v>
+        <v>99.34541792547836</v>
       </c>
       <c r="E33">
-        <v>1.006595636732623</v>
+        <v>1.00658895083629</v>
       </c>
       <c r="F33">
-        <v>2461.971740869314</v>
+        <v>1963.330268151673</v>
       </c>
       <c r="G33">
-        <v>269.9923237674877</v>
+        <v>251.6567291090799</v>
       </c>
     </row>
   </sheetData>
@@ -2621,13 +2621,13 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>36.21314297445958</v>
+        <v>35.53105077922309</v>
       </c>
       <c r="C2">
-        <v>0.3621314297445958</v>
+        <v>0.3553105077922309</v>
       </c>
       <c r="D2">
-        <v>0.2932061103673564</v>
+        <v>0.1078542411995211</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
@@ -2638,13 +2638,13 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>35.73983427744304</v>
+        <v>34.79646375761699</v>
       </c>
       <c r="C3">
-        <v>0.3573983427744304</v>
+        <v>0.3479646375761699</v>
       </c>
       <c r="D3">
-        <v>0.3816420170990526</v>
+        <v>0.0535197563108487</v>
       </c>
       <c r="E3" t="s">
         <v>53</v>
@@ -2655,13 +2655,13 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>35.28818078629894</v>
+        <v>33.96942874910513</v>
       </c>
       <c r="C4">
-        <v>0.3528818078629894</v>
+        <v>0.3396942874910513</v>
       </c>
       <c r="D4">
-        <v>0.3827242382081905</v>
+        <v>0.09771920387021699</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -2672,13 +2672,13 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>34.28474383414597</v>
+        <v>32.76553843508282</v>
       </c>
       <c r="C5">
-        <v>0.3428474383414597</v>
+        <v>0.3276553843508282</v>
       </c>
       <c r="D5">
-        <v>0.1724609499970476</v>
+        <v>0.1260213016733955</v>
       </c>
       <c r="E5" t="s">
         <v>53</v>
@@ -2689,13 +2689,13 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>34.00927271614375</v>
+        <v>32.46534136057391</v>
       </c>
       <c r="C6">
-        <v>0.3400927271614375</v>
+        <v>0.3246534136057391</v>
       </c>
       <c r="D6">
-        <v>0.120328157952625</v>
+        <v>0.01691098798402844</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
@@ -2706,13 +2706,13 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>33.25811346615763</v>
+        <v>31.72232097291986</v>
       </c>
       <c r="C7">
-        <v>0.3325811346615763</v>
+        <v>0.3172232097291986</v>
       </c>
       <c r="D7">
-        <v>0.1153222542969143</v>
+        <v>0.07736239383756983</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
@@ -2723,13 +2723,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>32.5107725123483</v>
+        <v>31.45381835686403</v>
       </c>
       <c r="C8">
-        <v>0.325107725123483</v>
+        <v>0.3145381835686403</v>
       </c>
       <c r="D8">
-        <v>0.04645272038777068</v>
+        <v>0.09540217873383107</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>32.24172325795473</v>
+        <v>31.09978841063272</v>
       </c>
       <c r="C9">
-        <v>0.3224172325795473</v>
+        <v>0.3109978841063272</v>
       </c>
       <c r="D9">
-        <v>0.1596594473787434</v>
+        <v>0.7665382154767668</v>
       </c>
       <c r="E9" t="s">
         <v>53</v>
@@ -2757,13 +2757,13 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>32.17454412208342</v>
+        <v>30.7490083596401</v>
       </c>
       <c r="C10">
-        <v>0.3217454412208342</v>
+        <v>0.3074900835964011</v>
       </c>
       <c r="D10">
-        <v>1.641416183723344</v>
+        <v>0.1294143002739229</v>
       </c>
       <c r="E10" t="s">
         <v>53</v>
@@ -2774,13 +2774,13 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>31.15333849933335</v>
+        <v>30.6411366691306</v>
       </c>
       <c r="C11">
-        <v>0.3115333849933336</v>
+        <v>0.306411366691306</v>
       </c>
       <c r="D11">
-        <v>0.06545538496094797</v>
+        <v>0.4958801645123899</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
@@ -2791,13 +2791,13 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.62816309239676</v>
+        <v>30.19005749576751</v>
       </c>
       <c r="C12">
-        <v>0.3062816309239677</v>
+        <v>0.3019005749576751</v>
       </c>
       <c r="D12">
-        <v>1.313322861542352</v>
+        <v>0.02240804910878908</v>
       </c>
       <c r="E12" t="s">
         <v>53</v>
@@ -2808,13 +2808,13 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.03209660063617</v>
+        <v>30.060948377805</v>
       </c>
       <c r="C13">
-        <v>0.3003209660063617</v>
+        <v>0.30060948377805</v>
       </c>
       <c r="D13">
-        <v>0.3759903059363186</v>
+        <v>122.1989771455488</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -2825,13 +2825,13 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.86701921753074</v>
+        <v>29.92529558764737</v>
       </c>
       <c r="C14">
-        <v>0.2986701921753074</v>
+        <v>0.2992529558764737</v>
       </c>
       <c r="D14">
-        <v>0.9361316942376596</v>
+        <v>1.270764895991122</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
@@ -2842,13 +2842,13 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.72922449361318</v>
+        <v>29.81229920922454</v>
       </c>
       <c r="C15">
-        <v>0.2972922449361318</v>
+        <v>0.2981229920922455</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>0.02352058845417378</v>
       </c>
       <c r="E15" t="s">
         <v>53</v>
@@ -2859,13 +2859,13 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.26797135488714</v>
+        <v>28.37034549788314</v>
       </c>
       <c r="C16">
-        <v>0.2826797135488714</v>
+        <v>0.2837034549788314</v>
       </c>
       <c r="D16">
-        <v>0.3184387357985841</v>
+        <v>28.94945384281403</v>
       </c>
       <c r="E16" t="s">
         <v>53</v>
@@ -2876,13 +2876,13 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.47384700758074</v>
+        <v>28.04668130067836</v>
       </c>
       <c r="C17">
-        <v>0.2747384700758074</v>
+        <v>0.2804668130067836</v>
       </c>
       <c r="D17">
-        <v>0.3189968026849421</v>
+        <v>0.05909294022874534</v>
       </c>
       <c r="E17" t="s">
         <v>53</v>
@@ -2893,13 +2893,13 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>26.17281989001769</v>
+        <v>27.91093853595413</v>
       </c>
       <c r="C18">
-        <v>0.2617281989001769</v>
+        <v>0.2791093853595413</v>
       </c>
       <c r="D18">
-        <v>0.1144916509792357</v>
+        <v>0.09790301804920355</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
@@ -2910,13 +2910,13 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>25.6883257658199</v>
+        <v>27.81889025807012</v>
       </c>
       <c r="C19">
-        <v>0.256883257658199</v>
+        <v>0.2781889025807012</v>
       </c>
       <c r="D19">
-        <v>4.767692235675558</v>
+        <v>0.2098892249037075</v>
       </c>
       <c r="E19" t="s">
         <v>53</v>
@@ -2927,13 +2927,13 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>25.51859381286541</v>
+        <v>26.92235337367029</v>
       </c>
       <c r="C20">
-        <v>0.2551859381286541</v>
+        <v>0.2692235337367029</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>0.01922258951237711</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
@@ -2944,13 +2944,13 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>24.34935314196738</v>
+        <v>26.58743165837271</v>
       </c>
       <c r="C21">
-        <v>0.2434935314196738</v>
+        <v>0.2658743165837271</v>
       </c>
       <c r="D21">
-        <v>0.3470634286184923</v>
+        <v>0.3025802964223989</v>
       </c>
       <c r="E21" t="s">
         <v>53</v>
@@ -2961,13 +2961,13 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>24.21616657915808</v>
+        <v>25.6455933751288</v>
       </c>
       <c r="C22">
-        <v>0.2421616657915809</v>
+        <v>0.256455933751288</v>
       </c>
       <c r="D22">
-        <v>0.1882725262616801</v>
+        <v>0.3339675910196991</v>
       </c>
       <c r="E22" t="s">
         <v>53</v>
@@ -2978,13 +2978,13 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>23.53697886600697</v>
+        <v>25.42183042278921</v>
       </c>
       <c r="C23">
-        <v>0.2353697886600697</v>
+        <v>0.2542183042278922</v>
       </c>
       <c r="D23">
-        <v>0.4532015535071057</v>
+        <v>0.1284169888521976</v>
       </c>
       <c r="E23" t="s">
         <v>53</v>
@@ -2995,13 +2995,13 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>23.4126027926713</v>
+        <v>25.00347188885532</v>
       </c>
       <c r="C24">
-        <v>0.234126027926713</v>
+        <v>0.2500347188885532</v>
       </c>
       <c r="D24">
-        <v>0.3050096011466932</v>
+        <v>595.32075925846</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
@@ -3012,13 +3012,13 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>23.19777916236094</v>
+        <v>24.89364732160354</v>
       </c>
       <c r="C25">
-        <v>0.2319777916236094</v>
+        <v>0.2489364732160354</v>
       </c>
       <c r="D25">
-        <v>0.1423532173361323</v>
+        <v>3111.705915200442</v>
       </c>
       <c r="E25" t="s">
         <v>53</v>
@@ -3029,13 +3029,13 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>22.07828457384698</v>
+        <v>24.7140392990936</v>
       </c>
       <c r="C26">
-        <v>0.2207828457384698</v>
+        <v>0.247140392990936</v>
       </c>
       <c r="D26">
-        <v>1.156776111667323</v>
+        <v>0.2840629155467472</v>
       </c>
       <c r="E26" t="s">
         <v>53</v>
@@ -3046,13 +3046,13 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>21.76511615073989</v>
+        <v>24.34048680833812</v>
       </c>
       <c r="C27">
-        <v>0.2176511615073989</v>
+        <v>0.2434048680833812</v>
       </c>
       <c r="D27">
-        <v>345.4780341387284</v>
+        <v>0.05654625358935568</v>
       </c>
       <c r="E27" t="s">
         <v>53</v>
@@ -3063,13 +3063,13 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>19.63833841116994</v>
+        <v>24.19983584259504</v>
       </c>
       <c r="C28">
-        <v>0.1963833841116994</v>
+        <v>0.2419983584259504</v>
       </c>
       <c r="D28">
-        <v>0.1150861762539551</v>
+        <v>0.1558760078412019</v>
       </c>
       <c r="E28" t="s">
         <v>53</v>
@@ -3080,13 +3080,13 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>19.45954343617745</v>
+        <v>23.91022815399812</v>
       </c>
       <c r="C29">
-        <v>0.1945954343617745</v>
+        <v>0.2391022815399812</v>
       </c>
       <c r="D29">
-        <v>0.04309006527443973</v>
+        <v>0.03861408281366856</v>
       </c>
       <c r="E29" t="s">
         <v>53</v>
@@ -3097,13 +3097,13 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>18.40133434703328</v>
+        <v>22.2948038443046</v>
       </c>
       <c r="C30">
-        <v>0.1840133434703329</v>
+        <v>0.222948038443046</v>
       </c>
       <c r="D30">
-        <v>0.1149064545637004</v>
+        <v>0.2424419855253466</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -3114,13 +3114,13 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>17.82625918535862</v>
+        <v>21.84530409795105</v>
       </c>
       <c r="C31">
-        <v>1.42610073482869</v>
+        <v>0.2184530409795105</v>
       </c>
       <c r="D31">
-        <v>0.6445452386515254</v>
+        <v>0.3784583805673852</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
@@ -3131,13 +3131,13 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.01604057835124</v>
+        <v>17.39791500300628</v>
       </c>
       <c r="C32">
-        <v>0.1701604057835124</v>
+        <v>1.391833200240503</v>
       </c>
       <c r="D32">
-        <v>2.164680071134499</v>
+        <v>0.07406233215897166</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
@@ -3148,13 +3148,13 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>15.94412501775627</v>
+        <v>16.81460346266623</v>
       </c>
       <c r="C33">
-        <v>0.1594412501775627</v>
+        <v>0.1681460346266623</v>
       </c>
       <c r="D33">
-        <v>0.05992481124864888</v>
+        <v>3.695331975299755</v>
       </c>
       <c r="E33" t="s">
         <v>53</v>
@@ -3202,205 +3202,205 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B2">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="C2">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2">
-        <v>8.42911877394636</v>
+        <v>7.763805358119191</v>
       </c>
       <c r="F2">
-        <v>620.2173112820382</v>
+        <v>1582.189431414851</v>
       </c>
       <c r="G2">
-        <v>2122.998332823759</v>
+        <v>5647.085722722305</v>
       </c>
       <c r="H2">
-        <v>-2055.697801867108</v>
+        <v>-3560.670555754781</v>
       </c>
       <c r="I2">
-        <v>4178.696134690867</v>
+        <v>9207.756278477085</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B3">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="C3">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="D3">
         <v>13</v>
       </c>
       <c r="E3">
-        <v>-1.461693548387097</v>
+        <v>-1.158106747230614</v>
       </c>
       <c r="F3">
-        <v>2366.343312581236</v>
+        <v>8782.881084599507</v>
       </c>
       <c r="G3">
-        <v>4572.659425529603</v>
+        <v>22104.68892496204</v>
       </c>
       <c r="H3">
-        <v>-6868.004630611985</v>
+        <v>-22305.10721949036</v>
       </c>
       <c r="I3">
-        <v>11440.66405614159</v>
+        <v>44409.7961444524</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="C4">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="D4">
         <v>13</v>
       </c>
       <c r="E4">
-        <v>3.175403225806452</v>
+        <v>3.474320241691843</v>
       </c>
       <c r="F4">
-        <v>1860.439909226242</v>
+        <v>489.1409000525189</v>
       </c>
       <c r="G4">
-        <v>5914.515704427017</v>
+        <v>1270.057371895645</v>
       </c>
       <c r="H4">
-        <v>-3617.849227703511</v>
+        <v>-1225.869492165333</v>
       </c>
       <c r="I4">
-        <v>9532.364932130527</v>
+        <v>2495.926864060978</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="C5">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="D5">
         <v>13</v>
       </c>
       <c r="E5">
-        <v>8.71975806451613</v>
+        <v>9.013091641490432</v>
       </c>
       <c r="F5">
-        <v>827.7610446556429</v>
+        <v>1610.62115145263</v>
       </c>
       <c r="G5">
-        <v>4314.821203627136</v>
+        <v>6330.800651699886</v>
       </c>
       <c r="H5">
-        <v>-1849.383798894357</v>
+        <v>-3576.666976329087</v>
       </c>
       <c r="I5">
-        <v>6164.205002521493</v>
+        <v>9907.467628028971</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="C6">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="D6">
         <v>13</v>
       </c>
       <c r="E6">
-        <v>9.828629032258064</v>
+        <v>10.32225579053374</v>
       </c>
       <c r="F6">
-        <v>3130.86174709911</v>
+        <v>1550.377984447354</v>
       </c>
       <c r="G6">
-        <v>19308.92284016448</v>
+        <v>5874.518203809105</v>
       </c>
       <c r="H6">
-        <v>-5013.769069157467</v>
+        <v>-3635.816778056384</v>
       </c>
       <c r="I6">
-        <v>24322.69190932194</v>
+        <v>9510.33498186549</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="C7">
-        <v>945</v>
+        <v>953</v>
       </c>
       <c r="D7">
         <v>13</v>
       </c>
       <c r="E7">
-        <v>4.08266129032258</v>
+        <v>3.37361530715005</v>
       </c>
       <c r="F7">
-        <v>6431.714777386662</v>
+        <v>1715.121904479063</v>
       </c>
       <c r="G7">
-        <v>21979.45330646568</v>
+        <v>4632.613040087208</v>
       </c>
       <c r="H7">
-        <v>-18702.28645408327</v>
+        <v>-4241.50875976167</v>
       </c>
       <c r="I7">
-        <v>40681.73976054894</v>
+        <v>8874.121799848879</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>1004</v>
+        <v>1013</v>
       </c>
       <c r="C8">
-        <v>967</v>
+        <v>960</v>
       </c>
       <c r="D8">
         <v>13</v>
       </c>
       <c r="E8">
-        <v>1.86491935483871</v>
+        <v>2.668680765357502</v>
       </c>
       <c r="F8">
-        <v>2660.587028175543</v>
+        <v>452.3907500348874</v>
       </c>
       <c r="G8">
-        <v>6760.846067053688</v>
+        <v>1367.273144392322</v>
       </c>
       <c r="H8">
-        <v>-8009.997209004826</v>
+        <v>-1094.355800564404</v>
       </c>
       <c r="I8">
-        <v>14770.84327605851</v>
+        <v>2461.628944956727</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3408,144 +3408,144 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1008</v>
+        <v>1011</v>
       </c>
       <c r="C9">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="D9">
         <v>13</v>
       </c>
       <c r="E9">
-        <v>2.268145161290323</v>
+        <v>2.467270896273917</v>
       </c>
       <c r="F9">
-        <v>479.9797218708287</v>
+        <v>160.9553564028679</v>
       </c>
       <c r="G9">
-        <v>1849.738748448387</v>
+        <v>469.4501568015831</v>
       </c>
       <c r="H9">
-        <v>-1576.551936913168</v>
+        <v>-389.7762883397514</v>
       </c>
       <c r="I9">
-        <v>3426.290685361555</v>
+        <v>859.2264451413345</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B10">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="C10">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="D10">
         <v>13</v>
       </c>
       <c r="E10">
-        <v>13.35685483870968</v>
+        <v>13.34340382678751</v>
       </c>
       <c r="F10">
-        <v>882.6721136685038</v>
+        <v>1156.422950345222</v>
       </c>
       <c r="G10">
-        <v>3377.60575341587</v>
+        <v>6260.442658118053</v>
       </c>
       <c r="H10">
-        <v>-2290.236779198098</v>
+        <v>-1710.419040321226</v>
       </c>
       <c r="I10">
-        <v>5667.842532613968</v>
+        <v>7970.861698439279</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="C11">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="D11">
         <v>13</v>
       </c>
       <c r="E11">
-        <v>6.804435483870967</v>
+        <v>7.200402819738168</v>
       </c>
       <c r="F11">
-        <v>2090.4168244344</v>
+        <v>2160.837187202707</v>
       </c>
       <c r="G11">
-        <v>7037.489622822785</v>
+        <v>7985.511459797283</v>
       </c>
       <c r="H11">
-        <v>-6683.574361353197</v>
+        <v>-4162.080012931879</v>
       </c>
       <c r="I11">
-        <v>13721.06398417598</v>
+        <v>12147.59147272916</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="C12">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D12">
         <v>523</v>
       </c>
       <c r="E12">
-        <v>11.0383064516129</v>
+        <v>11.22860020140987</v>
       </c>
       <c r="F12">
-        <v>4391.620423962324</v>
+        <v>566.1653622162919</v>
       </c>
       <c r="G12">
-        <v>11001.52427943153</v>
+        <v>1482.191367068195</v>
       </c>
       <c r="H12">
-        <v>-9958.113972963189</v>
+        <v>-1209.45700995785</v>
       </c>
       <c r="I12">
-        <v>20959.63825239472</v>
+        <v>2691.648377026045</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="C13">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="D13">
         <v>13</v>
       </c>
       <c r="E13">
-        <v>12.55040322580645</v>
+        <v>12.73917421953676</v>
       </c>
       <c r="F13">
-        <v>3140.144293950367</v>
+        <v>687.6316796193344</v>
       </c>
       <c r="G13">
-        <v>13376.2371642817</v>
+        <v>2785.521431382404</v>
       </c>
       <c r="H13">
-        <v>-4708.031964205812</v>
+        <v>-1305.140250346389</v>
       </c>
       <c r="I13">
-        <v>18084.26912848751</v>
+        <v>4090.661681728794</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3553,529 +3553,529 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>1058</v>
+        <v>1051</v>
       </c>
       <c r="C14">
-        <v>913</v>
+        <v>922</v>
       </c>
       <c r="D14">
         <v>13</v>
       </c>
       <c r="E14">
-        <v>7.308467741935484</v>
+        <v>6.495468277945619</v>
       </c>
       <c r="F14">
-        <v>2128.629357334803</v>
+        <v>4366.914375140721</v>
       </c>
       <c r="G14">
-        <v>9239.42656432446</v>
+        <v>14065.60359733634</v>
       </c>
       <c r="H14">
-        <v>-3323.026007880733</v>
+        <v>-11448.93332399753</v>
       </c>
       <c r="I14">
-        <v>12562.45257220519</v>
+        <v>25514.53692133387</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B15">
-        <v>1128</v>
+        <v>1123</v>
       </c>
       <c r="C15">
-        <v>843</v>
+        <v>850</v>
       </c>
       <c r="D15">
         <v>13</v>
       </c>
       <c r="E15">
-        <v>14.36491935483871</v>
+        <v>13.74622356495468</v>
       </c>
       <c r="F15">
-        <v>640.3194215506687</v>
+        <v>137.4548687182613</v>
       </c>
       <c r="G15">
-        <v>2877.481783478114</v>
+        <v>655.8764562485604</v>
       </c>
       <c r="H15">
-        <v>-1337.505756689111</v>
+        <v>-248.0002345845859</v>
       </c>
       <c r="I15">
-        <v>4214.987540167225</v>
+        <v>903.8766908331463</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16">
-        <v>1025</v>
+        <v>1042</v>
       </c>
       <c r="C16">
-        <v>946</v>
+        <v>931</v>
       </c>
       <c r="D16">
         <v>13</v>
       </c>
       <c r="E16">
-        <v>3.981854838709677</v>
+        <v>5.589123867069486</v>
       </c>
       <c r="F16">
-        <v>472.098201982139</v>
+        <v>925.6173538191006</v>
       </c>
       <c r="G16">
-        <v>1400.707010552066</v>
+        <v>2951.401446474801</v>
       </c>
       <c r="H16">
-        <v>-1348.562930193893</v>
+        <v>-2006.186875264088</v>
       </c>
       <c r="I16">
-        <v>2749.269940745959</v>
+        <v>4957.588321738888</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17">
-        <v>1054</v>
+        <v>1061</v>
       </c>
       <c r="C17">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="D17">
         <v>13</v>
       </c>
       <c r="E17">
-        <v>6.90524193548387</v>
+        <v>7.502517623363544</v>
       </c>
       <c r="F17">
-        <v>4829.165775245163</v>
+        <v>12408.97788661713</v>
       </c>
       <c r="G17">
-        <v>17355.76782920236</v>
+        <v>49346.74105115823</v>
       </c>
       <c r="H17">
-        <v>-9610.810275113245</v>
+        <v>-26083.96669982222</v>
       </c>
       <c r="I17">
-        <v>26966.57810431561</v>
+        <v>75430.70775098045</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18">
-        <v>1018</v>
+        <v>1029</v>
       </c>
       <c r="C18">
-        <v>953</v>
+        <v>944</v>
       </c>
       <c r="D18">
         <v>13</v>
       </c>
       <c r="E18">
-        <v>3.276209677419355</v>
+        <v>4.279959718026183</v>
       </c>
       <c r="F18">
-        <v>1248.079021898259</v>
+        <v>1065.51520858952</v>
       </c>
       <c r="G18">
-        <v>3909.641726304677</v>
+        <v>2740.084893256197</v>
       </c>
       <c r="H18">
-        <v>-3590.060934131663</v>
+        <v>-2876.544612893996</v>
       </c>
       <c r="I18">
-        <v>7499.70266043634</v>
+        <v>5616.629506150192</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19">
-        <v>860</v>
+        <v>854</v>
       </c>
       <c r="C19">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="D19">
         <v>523</v>
       </c>
       <c r="E19">
-        <v>13.05443548387097</v>
+        <v>12.33635448136959</v>
       </c>
       <c r="F19">
-        <v>52.41005973884766</v>
+        <v>286.9781824283578</v>
       </c>
       <c r="G19">
-        <v>187.3030807236183</v>
+        <v>913.1325860090519</v>
       </c>
       <c r="H19">
-        <v>-83.61143027075832</v>
+        <v>-365.9222591223181</v>
       </c>
       <c r="I19">
-        <v>270.9145109943766</v>
+        <v>1279.05484513137</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20">
-        <v>1043</v>
+        <v>1036</v>
       </c>
       <c r="C20">
-        <v>928</v>
+        <v>937</v>
       </c>
       <c r="D20">
         <v>13</v>
       </c>
       <c r="E20">
-        <v>5.796370967741935</v>
+        <v>4.984894259818732</v>
       </c>
       <c r="F20">
-        <v>4487.821902251935</v>
+        <v>409.9650932796765</v>
       </c>
       <c r="G20">
-        <v>13846.01562780497</v>
+        <v>1182.942825847605</v>
       </c>
       <c r="H20">
-        <v>-9400.206661487702</v>
+        <v>-798.4339010962238</v>
       </c>
       <c r="I20">
-        <v>23246.22228929268</v>
+        <v>1981.376726943829</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B21">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C21">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="D21">
         <v>13</v>
       </c>
       <c r="E21">
-        <v>3.881048387096774</v>
+        <v>4.179254783484391</v>
       </c>
       <c r="F21">
-        <v>2350.780988542538</v>
+        <v>6354.526707670042</v>
       </c>
       <c r="G21">
-        <v>7701.972076286408</v>
+        <v>17096.86659413722</v>
       </c>
       <c r="H21">
-        <v>-6035.306533708129</v>
+        <v>-15706.74525724996</v>
       </c>
       <c r="I21">
-        <v>13737.27860999454</v>
+        <v>32803.61185138718</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B22">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="C22">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="D22">
         <v>13</v>
       </c>
       <c r="E22">
-        <v>6.098790322580645</v>
+        <v>5.790533736153072</v>
       </c>
       <c r="F22">
-        <v>44780.81834485844</v>
+        <v>7851.713522911727</v>
       </c>
       <c r="G22">
-        <v>160393.5366521343</v>
+        <v>27844.62434917884</v>
       </c>
       <c r="H22">
-        <v>-141512.631573034</v>
+        <v>-24633.26803745599</v>
       </c>
       <c r="I22">
-        <v>301906.1682251684</v>
+        <v>52477.89238663482</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B23">
         <v>1040</v>
       </c>
       <c r="C23">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="D23">
         <v>13</v>
       </c>
       <c r="E23">
-        <v>5.493951612903226</v>
+        <v>5.387713997985901</v>
       </c>
       <c r="F23">
-        <v>5289.85239273193</v>
+        <v>1741.734942865157</v>
       </c>
       <c r="G23">
-        <v>26702.26522904087</v>
+        <v>5998.231447341955</v>
       </c>
       <c r="H23">
-        <v>-11085.51715589314</v>
+        <v>-4075.14839230742</v>
       </c>
       <c r="I23">
-        <v>37787.78238493401</v>
+        <v>10073.37983964937</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="C24">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="D24">
         <v>13</v>
       </c>
       <c r="E24">
-        <v>2.973790322580645</v>
+        <v>2.668680765357502</v>
       </c>
       <c r="F24">
-        <v>9539.860364407168</v>
+        <v>2007.665202612201</v>
       </c>
       <c r="G24">
-        <v>28688.25541021257</v>
+        <v>6423.208814278197</v>
       </c>
       <c r="H24">
-        <v>-38971.72103729852</v>
+        <v>-7169.48652390584</v>
       </c>
       <c r="I24">
-        <v>67659.97644751109</v>
+        <v>13592.69533818404</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="C25">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="D25">
         <v>13</v>
       </c>
       <c r="E25">
-        <v>9.929435483870968</v>
+        <v>9.919436052366565</v>
       </c>
       <c r="F25">
-        <v>5082.963354213584</v>
+        <v>1142.743387000225</v>
       </c>
       <c r="G25">
-        <v>22548.24822219515</v>
+        <v>4707.727207601418</v>
       </c>
       <c r="H25">
-        <v>-7616.716847738795</v>
+        <v>-2075.528555865812</v>
       </c>
       <c r="I25">
-        <v>30164.96506993394</v>
+        <v>6783.25576346723</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B26">
-        <v>1117</v>
+        <v>1108</v>
       </c>
       <c r="C26">
-        <v>854</v>
+        <v>865</v>
       </c>
       <c r="D26">
         <v>13</v>
       </c>
       <c r="E26">
-        <v>13.25604838709678</v>
+        <v>12.23564954682779</v>
       </c>
       <c r="F26">
-        <v>24318.35441950481</v>
+        <v>4422.557137796106</v>
       </c>
       <c r="G26">
-        <v>156546.5756237583</v>
+        <v>15254.72954350493</v>
       </c>
       <c r="H26">
-        <v>-22192.56526796321</v>
+        <v>-9918.33461749922</v>
       </c>
       <c r="I26">
-        <v>178739.1408917216</v>
+        <v>25173.06416100415</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B27">
-        <v>1003</v>
+        <v>992</v>
       </c>
       <c r="C27">
-        <v>968</v>
+        <v>981</v>
       </c>
       <c r="D27">
         <v>13</v>
       </c>
       <c r="E27">
-        <v>1.764112903225807</v>
+        <v>0.5538771399798591</v>
       </c>
       <c r="F27">
-        <v>3519.08243396573</v>
+        <v>377.7833992112438</v>
       </c>
       <c r="G27">
-        <v>9688.918584950672</v>
+        <v>891.568737568358</v>
       </c>
       <c r="H27">
-        <v>-10153.0993456786</v>
+        <v>-941.1108661211183</v>
       </c>
       <c r="I27">
-        <v>19842.01793062928</v>
+        <v>1832.679603689476</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B28">
-        <v>1082</v>
+        <v>1075</v>
       </c>
       <c r="C28">
-        <v>889</v>
+        <v>898</v>
       </c>
       <c r="D28">
         <v>13</v>
       </c>
       <c r="E28">
-        <v>9.72782258064516</v>
+        <v>8.91238670694864</v>
       </c>
       <c r="F28">
-        <v>1930.897793969071</v>
+        <v>555.064546107067</v>
       </c>
       <c r="G28">
-        <v>10403.19571718122</v>
+        <v>1926.218810395844</v>
       </c>
       <c r="H28">
-        <v>-3357.419507417613</v>
+        <v>-998.5300014715955</v>
       </c>
       <c r="I28">
-        <v>13760.61522459883</v>
+        <v>2924.748811867439</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B29">
         <v>1046</v>
       </c>
       <c r="C29">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="D29">
         <v>13</v>
       </c>
       <c r="E29">
-        <v>6.098790322580645</v>
+        <v>5.991943605236657</v>
       </c>
       <c r="F29">
-        <v>809.7902783744468</v>
+        <v>233.9377835530735</v>
       </c>
       <c r="G29">
-        <v>4663.327823682696</v>
+        <v>841.6915621339455</v>
       </c>
       <c r="H29">
-        <v>-1668.067292938357</v>
+        <v>-512.8158277324183</v>
       </c>
       <c r="I29">
-        <v>6331.395116621054</v>
+        <v>1354.507389866364</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30">
-        <v>1087</v>
+        <v>1098</v>
       </c>
       <c r="C30">
-        <v>884</v>
+        <v>875</v>
       </c>
       <c r="D30">
         <v>13</v>
       </c>
       <c r="E30">
-        <v>10.23185483870968</v>
+        <v>11.22860020140987</v>
       </c>
       <c r="F30">
-        <v>403.1831738116775</v>
+        <v>2495.375017771291</v>
       </c>
       <c r="G30">
-        <v>1571.699712022933</v>
+        <v>9347.600380386177</v>
       </c>
       <c r="H30">
-        <v>-996.9203915414954</v>
+        <v>-4110.049455808958</v>
       </c>
       <c r="I30">
-        <v>2568.620103564428</v>
+        <v>13457.64983619513</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B31">
-        <v>1054</v>
+        <v>1061</v>
       </c>
       <c r="C31">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="D31">
         <v>13</v>
       </c>
       <c r="E31">
-        <v>6.90524193548387</v>
+        <v>7.502517623363544</v>
       </c>
       <c r="F31">
-        <v>2759.504527095887</v>
+        <v>1110.638014220193</v>
       </c>
       <c r="G31">
-        <v>10243.34542346352</v>
+        <v>4654.362468800805</v>
       </c>
       <c r="H31">
-        <v>-7566.610770245635</v>
+        <v>-2958.999453996267</v>
       </c>
       <c r="I31">
-        <v>17809.95619370915</v>
+        <v>7613.361922797072</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B32">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="C32">
         <v>868</v>
@@ -4084,19 +4084,19 @@
         <v>13</v>
       </c>
       <c r="E32">
-        <v>11.84475806451613</v>
+        <v>11.93353474320242</v>
       </c>
       <c r="F32">
-        <v>1423.602856755335</v>
+        <v>1318.138313231797</v>
       </c>
       <c r="G32">
-        <v>7101.14669185745</v>
+        <v>5109.117808694491</v>
       </c>
       <c r="H32">
-        <v>-3179.10444803575</v>
+        <v>-2727.438579157316</v>
       </c>
       <c r="I32">
-        <v>10280.2511398932</v>
+        <v>7836.556387851808</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4104,28 +4104,28 @@
         <v>14</v>
       </c>
       <c r="B33">
-        <v>1010</v>
+        <v>1013</v>
       </c>
       <c r="C33">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="D33">
         <v>13</v>
       </c>
       <c r="E33">
-        <v>2.469758064516129</v>
+        <v>2.668680765357502</v>
       </c>
       <c r="F33">
-        <v>1194.30117302443</v>
+        <v>1175.171547424419</v>
       </c>
       <c r="G33">
-        <v>2985.466544107819</v>
+        <v>3493.550367468168</v>
       </c>
       <c r="H33">
-        <v>-3192.588666640249</v>
+        <v>-2663.489736303672</v>
       </c>
       <c r="I33">
-        <v>6178.055210748068</v>
+        <v>6157.04010377184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
learning pysystemtrade. Backup before reorganise
</commit_message>
<xml_diff>
--- a/perplexity_examples/etf_turnover_analysis.xlsx
+++ b/perplexity_examples/etf_turnover_analysis.xlsx
@@ -100,10 +100,10 @@
     <t>EMHY</t>
   </si>
   <si>
+    <t>SCHP</t>
+  </si>
+  <si>
     <t>IHY</t>
-  </si>
-  <si>
-    <t>SCHP</t>
   </si>
   <si>
     <t>VGK</t>
@@ -607,31 +607,31 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>35.53095150788038</v>
+        <v>35.42572289384545</v>
       </c>
       <c r="C2">
-        <v>7.09240786709889</v>
+        <v>7.113475164787117</v>
       </c>
       <c r="D2">
-        <v>1.01320112387127</v>
+        <v>1.016210737826731</v>
       </c>
       <c r="E2">
-        <v>131.8864800005121</v>
+        <v>132.1796456838034</v>
       </c>
       <c r="F2">
-        <v>73861.10731055759</v>
+        <v>73917.54639603154</v>
       </c>
       <c r="G2">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H2">
-        <v>0.3553095150788038</v>
+        <v>0.3542572289384545</v>
       </c>
       <c r="I2">
-        <v>329.4358236083984</v>
+        <v>-6.600151062011719</v>
       </c>
       <c r="J2">
-        <v>0.1078539398620963</v>
+        <v>5.367410921508171</v>
       </c>
       <c r="K2" t="s">
         <v>43</v>
@@ -645,31 +645,31 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>34.79640690476695</v>
+        <v>34.74690486441447</v>
       </c>
       <c r="C3">
-        <v>7.242127058971631</v>
+        <v>7.252444526593851</v>
       </c>
       <c r="D3">
-        <v>1.03458957985309</v>
+        <v>1.036063503799121</v>
       </c>
       <c r="E3">
-        <v>862.9809263947607</v>
+        <v>863.9608714153385</v>
       </c>
       <c r="F3">
-        <v>473308.4923432323</v>
+        <v>473886.6093891166</v>
       </c>
       <c r="G3">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H3">
-        <v>0.3479640690476695</v>
+        <v>0.3474690486441447</v>
       </c>
       <c r="I3">
-        <v>650.1611022949219</v>
+        <v>401.9526816101074</v>
       </c>
       <c r="J3">
-        <v>0.05351966886659858</v>
+        <v>0.08644526197767438</v>
       </c>
       <c r="K3" t="s">
         <v>43</v>
@@ -683,31 +683,31 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>33.9693074045411</v>
+        <v>33.9259451318414</v>
       </c>
       <c r="C4">
-        <v>7.418461524661879</v>
+        <v>7.427943393196257</v>
       </c>
       <c r="D4">
-        <v>1.05978021780884</v>
+        <v>1.061134770456608</v>
       </c>
       <c r="E4">
-        <v>1427.118001661653</v>
+        <v>1429.40589897577</v>
       </c>
       <c r="F4">
-        <v>764108.9306395568</v>
+        <v>765511.5777179936</v>
       </c>
       <c r="G4">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H4">
-        <v>0.339693074045411</v>
+        <v>0.339259451318414</v>
       </c>
       <c r="I4">
-        <v>347.6228561401367</v>
+        <v>245.2347645568738</v>
       </c>
       <c r="J4">
-        <v>0.09771885480063802</v>
+        <v>0.1383406842547132</v>
       </c>
       <c r="K4" t="s">
         <v>43</v>
@@ -721,31 +721,31 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>32.76543145076051</v>
+        <v>32.78771739399839</v>
       </c>
       <c r="C5">
-        <v>7.691032556024862</v>
+        <v>7.685804930297685</v>
       </c>
       <c r="D5">
-        <v>1.09871893657498</v>
+        <v>1.097972132899669</v>
       </c>
       <c r="E5">
-        <v>961.4089533486929</v>
+        <v>961.3348606746271</v>
       </c>
       <c r="F5">
-        <v>496515.4333808627</v>
+        <v>497565.3312106048</v>
       </c>
       <c r="G5">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H5">
-        <v>0.3276543145076051</v>
+        <v>0.3278771739399839</v>
       </c>
       <c r="I5">
-        <v>260</v>
+        <v>106.2224682617187</v>
       </c>
       <c r="J5">
-        <v>0.1260208901952327</v>
+        <v>0.308670264686503</v>
       </c>
       <c r="K5" t="s">
         <v>43</v>
@@ -759,31 +759,31 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>32.46525622786795</v>
+        <v>32.37954735576731</v>
       </c>
       <c r="C6">
-        <v>7.762144189814987</v>
+        <v>7.78269063588731</v>
       </c>
       <c r="D6">
-        <v>1.108877741402141</v>
+        <v>1.111812947983901</v>
       </c>
       <c r="E6">
-        <v>1360.196764444022</v>
+        <v>1363.594079057384</v>
       </c>
       <c r="F6">
-        <v>641008.4176051393</v>
+        <v>641964.1920016565</v>
       </c>
       <c r="G6">
-        <v>1829</v>
+        <v>1832</v>
       </c>
       <c r="H6">
-        <v>0.3246525622786795</v>
+        <v>0.3237954735576731</v>
       </c>
       <c r="I6">
-        <v>1919.777921386719</v>
+        <v>214.404259765625</v>
       </c>
       <c r="J6">
-        <v>0.01691094363894821</v>
+        <v>0.151021007657044</v>
       </c>
       <c r="K6" t="s">
         <v>43</v>
@@ -797,31 +797,31 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>31.72237763757622</v>
+        <v>31.78169146795513</v>
       </c>
       <c r="C7">
-        <v>7.943919049166653</v>
+        <v>7.929093398131021</v>
       </c>
       <c r="D7">
-        <v>1.134845578452379</v>
+        <v>1.132727628304431</v>
       </c>
       <c r="E7">
-        <v>7395.319253691568</v>
+        <v>7389.10853344669</v>
       </c>
       <c r="F7">
-        <v>3697697.307067142</v>
+        <v>3707091.374781814</v>
       </c>
       <c r="G7">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H7">
-        <v>0.3172237763757622</v>
+        <v>0.3178169146795513</v>
       </c>
       <c r="I7">
-        <v>410.0483374328369</v>
+        <v>-13.821</v>
       </c>
       <c r="J7">
-        <v>0.07736253202775667</v>
+        <v>2.29952184848818</v>
       </c>
       <c r="K7" t="s">
         <v>43</v>
@@ -835,31 +835,31 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>31.4536911902056</v>
+        <v>31.44654654213385</v>
       </c>
       <c r="C8">
-        <v>8.011778283067475</v>
+        <v>8.013598557232866</v>
       </c>
       <c r="D8">
-        <v>1.144539754723925</v>
+        <v>1.14479979389041</v>
       </c>
       <c r="E8">
-        <v>5304.679461762385</v>
+        <v>5305.564665988628</v>
       </c>
       <c r="F8">
-        <v>2629901.387392493</v>
+        <v>2633715.189320714</v>
       </c>
       <c r="G8">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H8">
-        <v>0.314536911902056</v>
+        <v>0.3144654654213385</v>
       </c>
       <c r="I8">
-        <v>329.6970653533936</v>
+        <v>-77.23868273925781</v>
       </c>
       <c r="J8">
-        <v>0.09540179302624736</v>
+        <v>0.4071346820904629</v>
       </c>
       <c r="K8" t="s">
         <v>43</v>
@@ -873,31 +873,31 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>31.09975466141803</v>
+        <v>31.18931185426068</v>
       </c>
       <c r="C9">
-        <v>8.102957812481657</v>
+        <v>8.079690926735692</v>
       </c>
       <c r="D9">
-        <v>1.157565401783094</v>
+        <v>1.154241560962242</v>
       </c>
       <c r="E9">
-        <v>320.8111700326966</v>
+        <v>320.6075848334035</v>
       </c>
       <c r="F9">
-        <v>157258.867299916</v>
+        <v>157849.7227223206</v>
       </c>
       <c r="G9">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H9">
-        <v>0.3109975466141803</v>
+        <v>0.3118931185426068</v>
       </c>
       <c r="I9">
-        <v>-40.57173899841309</v>
+        <v>-19.38998184204144</v>
       </c>
       <c r="J9">
-        <v>0.7665373836362906</v>
+        <v>1.60852713057399</v>
       </c>
       <c r="K9" t="s">
         <v>43</v>
@@ -911,31 +911,31 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>30.74894225061348</v>
+        <v>30.71965126342241</v>
       </c>
       <c r="C10">
-        <v>8.195403859622921</v>
+        <v>8.203218123769977</v>
       </c>
       <c r="D10">
-        <v>1.170771979946132</v>
+        <v>1.171888303395711</v>
       </c>
       <c r="E10">
-        <v>370.8187168601524</v>
+        <v>370.8858484260435</v>
       </c>
       <c r="F10">
-        <v>179721.7036033042</v>
+        <v>179854.2819145171</v>
       </c>
       <c r="G10">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H10">
-        <v>0.3074894225061348</v>
+        <v>0.3071965126342242</v>
       </c>
       <c r="I10">
-        <v>237.601318359375</v>
+        <v>88.70015106201171</v>
       </c>
       <c r="J10">
-        <v>0.1294140220388227</v>
+        <v>0.3463314424565727</v>
       </c>
       <c r="K10" t="s">
         <v>43</v>
@@ -949,31 +949,31 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>30.64220773900106</v>
+        <v>30.64016474060952</v>
       </c>
       <c r="C11">
-        <v>8.223950511217808</v>
+        <v>8.224498860673783</v>
       </c>
       <c r="D11">
-        <v>1.174850073031115</v>
+        <v>1.174928408667683</v>
       </c>
       <c r="E11">
-        <v>6908.051265163407</v>
+        <v>6904.944411892532</v>
       </c>
       <c r="F11">
-        <v>3336447.561035469</v>
+        <v>3339762.012959683</v>
       </c>
       <c r="G11">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H11">
-        <v>0.3064220773900106</v>
+        <v>0.3064016474060952</v>
       </c>
       <c r="I11">
-        <v>61.80141448974609</v>
+        <v>61.13944287107135</v>
       </c>
       <c r="J11">
-        <v>0.4958172558345752</v>
+        <v>0.5011521744681643</v>
       </c>
       <c r="K11" t="s">
         <v>43</v>
@@ -987,31 +987,31 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.18988606545343</v>
+        <v>30.13623579359739</v>
       </c>
       <c r="C12">
-        <v>8.347166314362676</v>
+        <v>8.36202642313871</v>
       </c>
       <c r="D12">
-        <v>1.19245233062324</v>
+        <v>1.19457520330553</v>
       </c>
       <c r="E12">
-        <v>1786.026595595413</v>
+        <v>1787.52291772588</v>
       </c>
       <c r="F12">
-        <v>849880.9500774428</v>
+        <v>850363.9915603739</v>
       </c>
       <c r="G12">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H12">
-        <v>0.3018988606545343</v>
+        <v>0.3013623579359739</v>
       </c>
       <c r="I12">
-        <v>1347.286296508789</v>
+        <v>1609.20613861084</v>
       </c>
       <c r="J12">
-        <v>0.02240792186759727</v>
+        <v>0.01872739301107361</v>
       </c>
       <c r="K12" t="s">
         <v>43</v>
@@ -1025,31 +1025,31 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.06060034708136</v>
+        <v>30.12615794086164</v>
       </c>
       <c r="C13">
-        <v>8.383066109472001</v>
+        <v>8.364823702201985</v>
       </c>
       <c r="D13">
-        <v>1.197580872781714</v>
+        <v>1.194974814600284</v>
       </c>
       <c r="E13">
-        <v>1702.504056385121</v>
+        <v>1701.633073447972</v>
       </c>
       <c r="F13">
-        <v>806667.3963504771</v>
+        <v>809233.5962076656</v>
       </c>
       <c r="G13">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H13">
-        <v>0.3006060034708136</v>
+        <v>0.3012615794086164</v>
       </c>
       <c r="I13">
-        <v>-0.246</v>
+        <v>-65.74945568847656</v>
       </c>
       <c r="J13">
-        <v>122.1975623865096</v>
+        <v>0.4581963093900052</v>
       </c>
       <c r="K13" t="s">
         <v>43</v>
@@ -1063,31 +1063,31 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.92527547559689</v>
+        <v>29.9263870009361</v>
       </c>
       <c r="C14">
-        <v>8.420975112008508</v>
+        <v>8.420662340299129</v>
       </c>
       <c r="D14">
-        <v>1.202996444572644</v>
+        <v>1.202951762899876</v>
       </c>
       <c r="E14">
-        <v>427.3806032932925</v>
+        <v>427.7724841566396</v>
       </c>
       <c r="F14">
-        <v>201586.6017535432</v>
+        <v>202083.7403527408</v>
       </c>
       <c r="G14">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H14">
-        <v>0.2992527547559689</v>
+        <v>0.2992638700093609</v>
       </c>
       <c r="I14">
-        <v>-23.54904174804688</v>
+        <v>32.81060238647461</v>
       </c>
       <c r="J14">
-        <v>1.270764041941488</v>
+        <v>0.91209501881235</v>
       </c>
       <c r="K14" t="s">
         <v>43</v>
@@ -1101,31 +1101,31 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.81218446214374</v>
+        <v>29.75340933964809</v>
       </c>
       <c r="C15">
-        <v>8.452919655048959</v>
+        <v>8.469617620061976</v>
       </c>
       <c r="D15">
-        <v>1.20755995072128</v>
+        <v>1.209945374294568</v>
       </c>
       <c r="E15">
-        <v>756.5528294791501</v>
+        <v>758.0791458059637</v>
       </c>
       <c r="F15">
-        <v>355501.7628608679</v>
+        <v>356053.7178057463</v>
       </c>
       <c r="G15">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H15">
-        <v>0.2981218446214374</v>
+        <v>0.2975340933964809</v>
       </c>
       <c r="I15">
-        <v>1267.498016357422</v>
+        <v>285.4496398010254</v>
       </c>
       <c r="J15">
-        <v>0.02352049792379084</v>
+        <v>0.1042334800646023</v>
       </c>
       <c r="K15" t="s">
         <v>43</v>
@@ -1139,31 +1139,31 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.370249166628</v>
+        <v>28.36780912356847</v>
       </c>
       <c r="C16">
-        <v>8.882544475373457</v>
+        <v>8.883308503039594</v>
       </c>
       <c r="D16">
-        <v>1.268934925053351</v>
+        <v>1.269044071862799</v>
       </c>
       <c r="E16">
-        <v>353.9819096207835</v>
+        <v>354.0185952983485</v>
       </c>
       <c r="F16">
-        <v>158289.7951045314</v>
+        <v>158531.6970152459</v>
       </c>
       <c r="G16">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H16">
-        <v>0.28370249166628</v>
+        <v>0.2836780912356848</v>
       </c>
       <c r="I16">
-        <v>-0.979995880126953</v>
+        <v>13.96031951904297</v>
       </c>
       <c r="J16">
-        <v>28.94935554520167</v>
+        <v>2.032031507937377</v>
       </c>
       <c r="K16" t="s">
         <v>43</v>
@@ -1177,31 +1177,31 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>28.04633464108334</v>
+        <v>27.99073492158428</v>
       </c>
       <c r="C17">
-        <v>8.985131327316502</v>
+        <v>9.002979046672946</v>
       </c>
       <c r="D17">
-        <v>1.283590189616643</v>
+        <v>1.286139863810421</v>
       </c>
       <c r="E17">
-        <v>1332.039660112637</v>
+        <v>1334.65123620699</v>
       </c>
       <c r="F17">
-        <v>588846.3214646816</v>
+        <v>589720.6458115036</v>
       </c>
       <c r="G17">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H17">
-        <v>0.2804633464108334</v>
+        <v>0.2799073492158428</v>
       </c>
       <c r="I17">
-        <v>474.6198309326172</v>
+        <v>-161.1098327636719</v>
       </c>
       <c r="J17">
-        <v>0.05909220983449624</v>
+        <v>0.1737369745932467</v>
       </c>
       <c r="K17" t="s">
         <v>43</v>
@@ -1215,31 +1215,31 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>27.91074965424614</v>
+        <v>27.86734463674831</v>
       </c>
       <c r="C18">
-        <v>9.028779345654822</v>
+        <v>9.042842197016892</v>
       </c>
       <c r="D18">
-        <v>1.289825620807832</v>
+        <v>1.291834599573842</v>
       </c>
       <c r="E18">
-        <v>10275.1012313029</v>
+        <v>1548.506461507993</v>
       </c>
       <c r="F18">
-        <v>4520290.122094586</v>
+        <v>681197.1910679678</v>
       </c>
       <c r="G18">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H18">
-        <v>0.2791074965424614</v>
+        <v>0.2786734463674831</v>
       </c>
       <c r="I18">
-        <v>285.0876213226318</v>
+        <v>-153.2633368530196</v>
       </c>
       <c r="J18">
-        <v>0.09790235551006166</v>
+        <v>0.1818265555804337</v>
       </c>
       <c r="K18" t="s">
         <v>43</v>
@@ -1253,31 +1253,31 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>27.81855794495917</v>
+        <v>27.86341678813201</v>
       </c>
       <c r="C19">
-        <v>9.058701047645908</v>
+        <v>9.044116947901934</v>
       </c>
       <c r="D19">
-        <v>1.294100149663701</v>
+        <v>1.292016706843133</v>
       </c>
       <c r="E19">
-        <v>1548.741277119357</v>
+        <v>10280.66305484551</v>
       </c>
       <c r="F19">
-        <v>679081.9478822197</v>
+        <v>4521887.307269136</v>
       </c>
       <c r="G19">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H19">
-        <v>0.2781855794495917</v>
+        <v>0.2786341678813201</v>
       </c>
       <c r="I19">
-        <v>-132.5408213348389</v>
+        <v>256.4348703612825</v>
       </c>
       <c r="J19">
-        <v>0.2098867176526764</v>
+        <v>0.1086568950192935</v>
       </c>
       <c r="K19" t="s">
         <v>43</v>
@@ -1291,31 +1291,31 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>26.92219524279917</v>
+        <v>26.89127375582474</v>
       </c>
       <c r="C20">
-        <v>9.360306532484641</v>
+        <v>9.37106967442983</v>
       </c>
       <c r="D20">
-        <v>1.337186647497806</v>
+        <v>1.338724239204261</v>
       </c>
       <c r="E20">
-        <v>2173.887246427608</v>
+        <v>2175.075453597677</v>
       </c>
       <c r="F20">
-        <v>922478.351840731</v>
+        <v>923315.1022258305</v>
       </c>
       <c r="G20">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H20">
-        <v>0.2692219524279917</v>
+        <v>0.2689127375582474</v>
       </c>
       <c r="I20">
-        <v>1400.558096313477</v>
+        <v>530.7916837158203</v>
       </c>
       <c r="J20">
-        <v>0.01922247660676361</v>
+        <v>0.05066257550904286</v>
       </c>
       <c r="K20" t="s">
         <v>43</v>
@@ -1329,31 +1329,31 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>26.58709734155243</v>
+        <v>26.58290038321374</v>
       </c>
       <c r="C21">
-        <v>9.478281768132483</v>
+        <v>9.479778217095152</v>
       </c>
       <c r="D21">
-        <v>1.354040252590355</v>
+        <v>1.354254031013593</v>
       </c>
       <c r="E21">
-        <v>1030.099815237907</v>
+        <v>1030.994687356777</v>
       </c>
       <c r="F21">
-        <v>431677.0239814393</v>
+        <v>432636.3731705531</v>
       </c>
       <c r="G21">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H21">
-        <v>0.2658709734155243</v>
+        <v>0.2658290038321374</v>
       </c>
       <c r="I21">
-        <v>87.86901187133789</v>
+        <v>-19.27043487548828</v>
       </c>
       <c r="J21">
-        <v>0.3025764917042946</v>
+        <v>1.379465515696629</v>
       </c>
       <c r="K21" t="s">
         <v>43</v>
@@ -1367,31 +1367,31 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>25.64555893993454</v>
+        <v>25.64371883857743</v>
       </c>
       <c r="C22">
-        <v>9.826262729941625</v>
+        <v>9.826967827337928</v>
       </c>
       <c r="D22">
-        <v>1.403751818563089</v>
+        <v>1.403852546762561</v>
       </c>
       <c r="E22">
-        <v>639.1387134007819</v>
+        <v>639.694927808536</v>
       </c>
       <c r="F22">
-        <v>258354.4771189918</v>
+        <v>258951.333466582</v>
       </c>
       <c r="G22">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H22">
-        <v>0.2564555893993454</v>
+        <v>0.2564371883857743</v>
       </c>
       <c r="I22">
-        <v>76.79066491699218</v>
+        <v>-0.414</v>
       </c>
       <c r="J22">
-        <v>0.3339671425902669</v>
+        <v>61.9413498516363</v>
       </c>
       <c r="K22" t="s">
         <v>43</v>
@@ -1405,31 +1405,31 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>25.42170725018393</v>
+        <v>25.43585740375006</v>
       </c>
       <c r="C23">
-        <v>9.912788213630961</v>
+        <v>9.907273657024323</v>
       </c>
       <c r="D23">
-        <v>1.41611260194728</v>
+        <v>1.415324808146332</v>
       </c>
       <c r="E23">
-        <v>3715.292505647067</v>
+        <v>3711.10209343682</v>
       </c>
       <c r="F23">
-        <v>1488697.379021754</v>
+        <v>1490093.504909373</v>
       </c>
       <c r="G23">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H23">
-        <v>0.2542170725018393</v>
+        <v>0.2543585740375006</v>
       </c>
       <c r="I23">
-        <v>-197.96314062502</v>
+        <v>80.23801611326658</v>
       </c>
       <c r="J23">
-        <v>0.1284163666525047</v>
+        <v>0.3170050636327296</v>
       </c>
       <c r="K23" t="s">
         <v>43</v>
@@ -1443,31 +1443,31 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>25.00351546734926</v>
+        <v>25.02641650667483</v>
       </c>
       <c r="C24">
-        <v>10.07858276285481</v>
+        <v>10.06936010726061</v>
       </c>
       <c r="D24">
-        <v>1.439797537550688</v>
+        <v>1.438480015322944</v>
       </c>
       <c r="E24">
-        <v>876.1943809604093</v>
+        <v>875.8442398051288</v>
       </c>
       <c r="F24">
-        <v>345310.8599754106</v>
+        <v>346010.9032581476</v>
       </c>
       <c r="G24">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H24">
-        <v>0.2500351546734926</v>
+        <v>0.2502641650667483</v>
       </c>
       <c r="I24">
-        <v>-0.042</v>
+        <v>-35.22479742431022</v>
       </c>
       <c r="J24">
-        <v>595.3217968416491</v>
+        <v>0.7104772301515914</v>
       </c>
       <c r="K24" t="s">
         <v>43</v>
@@ -1481,31 +1481,31 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>24.89356445131572</v>
+        <v>24.92259108613786</v>
       </c>
       <c r="C25">
-        <v>10.12309830088157</v>
+        <v>10.11130821546739</v>
       </c>
       <c r="D25">
-        <v>1.446156900125938</v>
+        <v>1.444472602209627</v>
       </c>
       <c r="E25">
-        <v>196.2191107761579</v>
+        <v>196.2664625466855</v>
       </c>
       <c r="F25">
-        <v>76990.490938434</v>
+        <v>77215.32875601551</v>
       </c>
       <c r="G25">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H25">
-        <v>0.2489356445131572</v>
+        <v>0.2492259108613786</v>
       </c>
       <c r="I25">
-        <v>-0.008</v>
+        <v>-61.650341796875</v>
       </c>
       <c r="J25">
-        <v>3111.695556414465</v>
+        <v>0.4042571437519778</v>
       </c>
       <c r="K25" t="s">
         <v>43</v>
@@ -1519,31 +1519,31 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>24.71480783542341</v>
+        <v>24.70927993073185</v>
       </c>
       <c r="C26">
-        <v>10.19631638158286</v>
+        <v>10.19859747861686</v>
       </c>
       <c r="D26">
-        <v>1.456616625940408</v>
+        <v>1.456942496945265</v>
       </c>
       <c r="E26">
-        <v>4432.730604756447</v>
+        <v>4432.410688160371</v>
       </c>
       <c r="F26">
-        <v>1726781.055352008</v>
+        <v>1728877.89271719</v>
       </c>
       <c r="G26">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H26">
-        <v>0.2471480783542341</v>
+        <v>0.2470927993073185</v>
       </c>
       <c r="I26">
-        <v>87.00199127198812</v>
+        <v>47.55514326477051</v>
       </c>
       <c r="J26">
-        <v>0.2840717490954807</v>
+        <v>0.5195921667853921</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -1557,31 +1557,31 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>24.34039125780323</v>
+        <v>24.29880101543948</v>
       </c>
       <c r="C27">
-        <v>10.35316143158594</v>
+        <v>10.37088207932066</v>
       </c>
       <c r="D27">
-        <v>1.479023061655134</v>
+        <v>1.481554582760095</v>
       </c>
       <c r="E27">
-        <v>1149.282507421121</v>
+        <v>1151.275118243466</v>
       </c>
       <c r="F27">
-        <v>440923.3015095966</v>
+        <v>441599.1219786872</v>
       </c>
       <c r="G27">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H27">
-        <v>0.2434039125780323</v>
+        <v>0.2429880101543948</v>
       </c>
       <c r="I27">
-        <v>430.4526871948242</v>
+        <v>-208.0047607421875</v>
       </c>
       <c r="J27">
-        <v>0.05654603161249798</v>
+        <v>0.1168184849651434</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -1595,31 +1595,31 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>24.19971116355993</v>
+        <v>24.1887757609856</v>
       </c>
       <c r="C28">
-        <v>10.41334742785952</v>
+        <v>10.41805515459175</v>
       </c>
       <c r="D28">
-        <v>1.487621061122788</v>
+        <v>1.488293593513107</v>
       </c>
       <c r="E28">
-        <v>1005.155876648543</v>
+        <v>1005.38259205839</v>
       </c>
       <c r="F28">
-        <v>383400.1669210294</v>
+        <v>383892.376442789</v>
       </c>
       <c r="G28">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H28">
-        <v>0.2419971116355993</v>
+        <v>0.241887757609856</v>
       </c>
       <c r="I28">
-        <v>155.2505493164062</v>
+        <v>12.41065533446382</v>
       </c>
       <c r="J28">
-        <v>0.155875204758471</v>
+        <v>1.94903291640164</v>
       </c>
       <c r="K28" t="s">
         <v>43</v>
@@ -1633,31 +1633,31 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>23.91003170481376</v>
+        <v>23.84761048073232</v>
       </c>
       <c r="C29">
-        <v>10.53950923658814</v>
+        <v>10.56709644782245</v>
       </c>
       <c r="D29">
-        <v>1.505644176655449</v>
+        <v>1.509585206831779</v>
       </c>
       <c r="E29">
-        <v>1393.813134048975</v>
+        <v>1396.958348183458</v>
       </c>
       <c r="F29">
-        <v>525283.0700336023</v>
+        <v>525887.1570363058</v>
       </c>
       <c r="G29">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H29">
-        <v>0.2391003170481376</v>
+        <v>0.2384761048073232</v>
       </c>
       <c r="I29">
-        <v>619.2100501098632</v>
+        <v>-283.9264984130859</v>
       </c>
       <c r="J29">
-        <v>0.03861376555592327</v>
+        <v>0.0839921973257893</v>
       </c>
       <c r="K29" t="s">
         <v>43</v>
@@ -1671,31 +1671,31 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>22.29468225530591</v>
+        <v>22.27320123866313</v>
       </c>
       <c r="C30">
-        <v>11.3031438221115</v>
+        <v>11.31404495024108</v>
       </c>
       <c r="D30">
-        <v>1.614734831730215</v>
+        <v>1.616292135748726</v>
       </c>
       <c r="E30">
-        <v>120.3583622319383</v>
+        <v>120.4841164011092</v>
       </c>
       <c r="F30">
-        <v>42294.72988303121</v>
+        <v>42362.02146548832</v>
       </c>
       <c r="G30">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H30">
-        <v>0.2229468225530591</v>
+        <v>0.2227320123866313</v>
       </c>
       <c r="I30">
-        <v>91.95933532714672</v>
+        <v>46.23067474365234</v>
       </c>
       <c r="J30">
-        <v>0.2424406633213718</v>
+        <v>0.4817840397564462</v>
       </c>
       <c r="K30" t="s">
         <v>43</v>
@@ -1709,31 +1709,31 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>21.84516409866361</v>
+        <v>21.84782342798901</v>
       </c>
       <c r="C31">
-        <v>11.53573389798506</v>
+        <v>11.53432976198286</v>
       </c>
       <c r="D31">
-        <v>1.647961985426436</v>
+        <v>1.64776139456898</v>
       </c>
       <c r="E31">
-        <v>492.7399961816288</v>
+        <v>492.9679489466685</v>
       </c>
       <c r="F31">
-        <v>169660.9233657242</v>
+        <v>170016.5108312916</v>
       </c>
       <c r="G31">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H31">
-        <v>0.2184516409866361</v>
+        <v>0.2184782342798901</v>
       </c>
       <c r="I31">
-        <v>57.72181359863281</v>
+        <v>-44.9818754272461</v>
       </c>
       <c r="J31">
-        <v>0.3784559551535129</v>
+        <v>0.4857028129768797</v>
       </c>
       <c r="K31" t="s">
         <v>43</v>
@@ -1747,31 +1747,31 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.39784661786715</v>
+        <v>17.37297547796422</v>
       </c>
       <c r="C32">
-        <v>14.4845511938933</v>
+        <v>14.50528726755157</v>
       </c>
       <c r="D32">
-        <v>2.069221599127613</v>
+        <v>2.07218389536451</v>
       </c>
       <c r="E32">
-        <v>297.6601301479577</v>
+        <v>297.7613105732244</v>
       </c>
       <c r="F32">
-        <v>81625.31383410413</v>
+        <v>81659.49916138576</v>
       </c>
       <c r="G32">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H32">
-        <v>1.391827729429372</v>
+        <v>1.389838038237137</v>
       </c>
       <c r="I32">
-        <v>1879.27271484375</v>
+        <v>-480.3542290039063</v>
       </c>
       <c r="J32">
-        <v>0.07406204104576135</v>
+        <v>0.28933606790955</v>
       </c>
       <c r="K32" t="s">
         <v>44</v>
@@ -1785,31 +1785,31 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>16.81448622390124</v>
+        <v>16.87583236079463</v>
       </c>
       <c r="C33">
-        <v>14.98707701468691</v>
+        <v>14.93259678174086</v>
       </c>
       <c r="D33">
-        <v>2.141011002098131</v>
+        <v>2.133228111677265</v>
       </c>
       <c r="E33">
-        <v>467.1044604191011</v>
+        <v>466.5545903109585</v>
       </c>
       <c r="F33">
-        <v>123795.915305332</v>
+        <v>124288.7749119698</v>
       </c>
       <c r="G33">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="H33">
-        <v>0.1681448622390124</v>
+        <v>0.1687583236079463</v>
       </c>
       <c r="I33">
-        <v>4.550228118896484</v>
+        <v>2.178061798095703</v>
       </c>
       <c r="J33">
-        <v>3.695306209829995</v>
+        <v>7.748096209000729</v>
       </c>
       <c r="K33" t="s">
         <v>44</v>
@@ -1857,22 +1857,22 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>1818</v>
+        <v>1821</v>
       </c>
       <c r="C2">
-        <v>1829</v>
+        <v>1832</v>
       </c>
       <c r="D2">
-        <v>99.39857845817387</v>
+        <v>99.3995633187773</v>
       </c>
       <c r="E2">
-        <v>1.006050605060506</v>
+        <v>1.00604063701263</v>
       </c>
       <c r="F2">
-        <v>2536.02348974973</v>
+        <v>2536.3252852842</v>
       </c>
       <c r="G2">
-        <v>352.5898886716938</v>
+        <v>352.5338780898718</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1880,22 +1880,22 @@
         <v>16</v>
       </c>
       <c r="B3">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C3">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D3">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E3">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F3">
-        <v>17580.09972234901</v>
+        <v>17578.13890013053</v>
       </c>
       <c r="G3">
-        <v>1874.149674134385</v>
+        <v>1876.058388047477</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1903,22 +1903,22 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C4">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D4">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E4">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F4">
-        <v>905.691892245428</v>
+        <v>905.8277320879109</v>
       </c>
       <c r="G4">
-        <v>102.1726314006808</v>
+        <v>102.2690993687959</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1926,22 +1926,22 @@
         <v>38</v>
       </c>
       <c r="B5">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C5">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D5">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E5">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F5">
-        <v>2100.370146450509</v>
+        <v>2100.659255908095</v>
       </c>
       <c r="G5">
-        <v>266.2357171989874</v>
+        <v>266.1372252208025</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1949,22 +1949,22 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C6">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D6">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E6">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F6">
-        <v>2743.278572626191</v>
+        <v>2743.93922526841</v>
       </c>
       <c r="G6">
-        <v>298.4522663277656</v>
+        <v>298.4416223742428</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1972,22 +1972,22 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C7">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D7">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E7">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F7">
-        <v>3090.912382549592</v>
+        <v>3091.094400408224</v>
       </c>
       <c r="G7">
-        <v>387.2827828887769</v>
+        <v>387.4046445941264</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1995,22 +1995,22 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C8">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D8">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E8">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F8">
-        <v>596.0699181450391</v>
+        <v>595.89963506841</v>
       </c>
       <c r="G8">
-        <v>91.0905745581876</v>
+        <v>91.01937343852077</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2018,22 +2018,22 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C9">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D9">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E9">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F9">
-        <v>231.6694736324231</v>
+        <v>231.6647731693357</v>
       </c>
       <c r="G9">
-        <v>37.43593882947673</v>
+        <v>37.40766518017791</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2041,22 +2041,22 @@
         <v>37</v>
       </c>
       <c r="B10">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C10">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D10">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E10">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F10">
-        <v>2102.014226577742</v>
+        <v>2102.209875198344</v>
       </c>
       <c r="G10">
-        <v>194.3234500360007</v>
+        <v>194.277518442707</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2064,22 +2064,22 @@
         <v>21</v>
       </c>
       <c r="B11">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C11">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D11">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E11">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F11">
-        <v>2999.708796578201</v>
+        <v>3000.123140814967</v>
       </c>
       <c r="G11">
-        <v>430.7556766738179</v>
+        <v>430.346149575088</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2087,22 +2087,22 @@
         <v>42</v>
       </c>
       <c r="B12">
-        <v>1463</v>
+        <v>1466</v>
       </c>
       <c r="C12">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D12">
-        <v>73.66565961732124</v>
+        <v>73.70537958773254</v>
       </c>
       <c r="E12">
-        <v>1.357484620642515</v>
+        <v>1.35675306957708</v>
       </c>
       <c r="F12">
-        <v>840.360954151688</v>
+        <v>840.4597962792304</v>
       </c>
       <c r="G12">
-        <v>84.61785051628983</v>
+        <v>84.78088329602305</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2110,22 +2110,22 @@
         <v>31</v>
       </c>
       <c r="B13">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C13">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D13">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E13">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F13">
-        <v>1268.793996615524</v>
+        <v>1268.785533698076</v>
       </c>
       <c r="G13">
-        <v>130.9449960055711</v>
+        <v>131.0482456814686</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2133,22 +2133,22 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C14">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D14">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E14">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F14">
-        <v>7459.430098187071</v>
+        <v>7459.24938905485</v>
       </c>
       <c r="G14">
-        <v>754.5349108067685</v>
+        <v>754.0959032942169</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2156,22 +2156,22 @@
         <v>39</v>
       </c>
       <c r="B15">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C15">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D15">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E15">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F15">
-        <v>235.6185562489733</v>
+        <v>235.6321441883392</v>
       </c>
       <c r="G15">
-        <v>21.43676121795804</v>
+        <v>21.43826997241312</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2179,45 +2179,45 @@
         <v>24</v>
       </c>
       <c r="B16">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C16">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D16">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E16">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F16">
-        <v>1413.167297071424</v>
+        <v>1413.223811445337</v>
       </c>
       <c r="G16">
-        <v>180.1833567465119</v>
+        <v>180.1891284442036</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C17">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D17">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E17">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F17">
-        <v>19501.85968373436</v>
+        <v>19503.985233106</v>
       </c>
       <c r="G17">
-        <v>2291.074567711397</v>
+        <v>2288.404507727296</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2225,22 +2225,22 @@
         <v>12</v>
       </c>
       <c r="B18">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C18">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D18">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E18">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F18">
-        <v>1887.408362840276</v>
+        <v>1887.674489773472</v>
       </c>
       <c r="G18">
-        <v>239.892798957543</v>
+        <v>239.8211585977311</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2248,22 +2248,22 @@
         <v>41</v>
       </c>
       <c r="B19">
-        <v>1463</v>
+        <v>1466</v>
       </c>
       <c r="C19">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D19">
-        <v>73.66565961732124</v>
+        <v>73.70537958773254</v>
       </c>
       <c r="E19">
-        <v>1.357484620642515</v>
+        <v>1.35675306957708</v>
       </c>
       <c r="F19">
-        <v>582.3463144865</v>
+        <v>582.3430045612386</v>
       </c>
       <c r="G19">
-        <v>55.79310583329059</v>
+        <v>55.70225045114989</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2271,22 +2271,22 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C20">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D20">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E20">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F20">
-        <v>719.416600462283</v>
+        <v>719.5490401151328</v>
       </c>
       <c r="G20">
-        <v>80.22797521770472</v>
+        <v>80.22859160690582</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2294,22 +2294,22 @@
         <v>17</v>
       </c>
       <c r="B21">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C21">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D21">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E21">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F21">
-        <v>10717.05676124123</v>
+        <v>10716.16304696409</v>
       </c>
       <c r="G21">
-        <v>1332.945457370752</v>
+        <v>1332.851816457851</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2317,45 +2317,45 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C22">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D22">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E22">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F22">
-        <v>19340.0632356595</v>
+        <v>19322.98451931082</v>
       </c>
       <c r="G22">
-        <v>1691.052995963238</v>
+        <v>1690.162962024131</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C23">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D23">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E23">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F23">
-        <v>2775.833123968815</v>
+        <v>2775.579566284877</v>
       </c>
       <c r="G23">
-        <v>344.1875052621488</v>
+        <v>344.7354205809553</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2363,22 +2363,22 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C24">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D24">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E24">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F24">
-        <v>4167.547157980252</v>
+        <v>4167.414539511426</v>
       </c>
       <c r="G24">
-        <v>408.8532165993295</v>
+        <v>409.5311721698713</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2386,22 +2386,22 @@
         <v>30</v>
       </c>
       <c r="B25">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C25">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D25">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E25">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F25">
-        <v>1982.601767959275</v>
+        <v>1983.271493201893</v>
       </c>
       <c r="G25">
-        <v>218.7922067822804</v>
+        <v>218.9455329810492</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2409,22 +2409,22 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C26">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D26">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E26">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F26">
-        <v>8032.125522220082</v>
+        <v>8030.714677376631</v>
       </c>
       <c r="G26">
-        <v>875.205806057784</v>
+        <v>874.9382048163915</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2432,22 +2432,22 @@
         <v>18</v>
       </c>
       <c r="B27">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C27">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D27">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E27">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F27">
-        <v>687.3248254137718</v>
+        <v>687.5183892232208</v>
       </c>
       <c r="G27">
-        <v>79.70545732382972</v>
+        <v>79.88346291615417</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2455,22 +2455,22 @@
         <v>40</v>
       </c>
       <c r="B28">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C28">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D28">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E28">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F28">
-        <v>679.8524952789594</v>
+        <v>679.7745287204093</v>
       </c>
       <c r="G28">
-        <v>85.99134483817753</v>
+        <v>86.04074434781961</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2478,22 +2478,22 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C29">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D29">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E29">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F29">
-        <v>310.2274806604548</v>
+        <v>310.2423300543782</v>
       </c>
       <c r="G29">
-        <v>39.02204305039736</v>
+        <v>39.07658337855036</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2501,22 +2501,22 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C30">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D30">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E30">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F30">
-        <v>3005.019291012577</v>
+        <v>3004.969998653595</v>
       </c>
       <c r="G30">
-        <v>467.5511159861789</v>
+        <v>467.2647278470802</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2524,22 +2524,22 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C31">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D31">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E31">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F31">
-        <v>1975.16544220027</v>
+        <v>1975.293542450192</v>
       </c>
       <c r="G31">
-        <v>175.0181753549978</v>
+        <v>175.1067324180909</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2547,22 +2547,22 @@
         <v>36</v>
       </c>
       <c r="B32">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C32">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D32">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E32">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F32">
-        <v>2058.931701867994</v>
+        <v>2059.427694914544</v>
       </c>
       <c r="G32">
-        <v>223.4786120170282</v>
+        <v>223.4813370337486</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2570,22 +2570,22 @@
         <v>14</v>
       </c>
       <c r="B33">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="C33">
-        <v>1986</v>
+        <v>1989</v>
       </c>
       <c r="D33">
-        <v>99.34541792547836</v>
+        <v>99.34640522875817</v>
       </c>
       <c r="E33">
-        <v>1.00658895083629</v>
+        <v>1.006578947368421</v>
       </c>
       <c r="F33">
-        <v>1963.265373584764</v>
+        <v>1963.267245896327</v>
       </c>
       <c r="G33">
-        <v>251.6550600004373</v>
+        <v>251.8043174142737</v>
       </c>
     </row>
   </sheetData>
@@ -2621,13 +2621,13 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>35.53095150788038</v>
+        <v>35.42572289384545</v>
       </c>
       <c r="C2">
-        <v>0.3553095150788038</v>
+        <v>0.3542572289384545</v>
       </c>
       <c r="D2">
-        <v>0.1078539398620963</v>
+        <v>5.367410921508171</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
@@ -2638,13 +2638,13 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>34.79640690476695</v>
+        <v>34.74690486441447</v>
       </c>
       <c r="C3">
-        <v>0.3479640690476695</v>
+        <v>0.3474690486441447</v>
       </c>
       <c r="D3">
-        <v>0.05351966886659858</v>
+        <v>0.08644526197767438</v>
       </c>
       <c r="E3" t="s">
         <v>53</v>
@@ -2655,13 +2655,13 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>33.9693074045411</v>
+        <v>33.9259451318414</v>
       </c>
       <c r="C4">
-        <v>0.339693074045411</v>
+        <v>0.339259451318414</v>
       </c>
       <c r="D4">
-        <v>0.09771885480063802</v>
+        <v>0.1383406842547132</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -2672,13 +2672,13 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>32.76543145076051</v>
+        <v>32.78771739399839</v>
       </c>
       <c r="C5">
-        <v>0.3276543145076051</v>
+        <v>0.3278771739399839</v>
       </c>
       <c r="D5">
-        <v>0.1260208901952327</v>
+        <v>0.308670264686503</v>
       </c>
       <c r="E5" t="s">
         <v>53</v>
@@ -2689,13 +2689,13 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>32.46525622786795</v>
+        <v>32.37954735576731</v>
       </c>
       <c r="C6">
-        <v>0.3246525622786795</v>
+        <v>0.3237954735576731</v>
       </c>
       <c r="D6">
-        <v>0.01691094363894821</v>
+        <v>0.151021007657044</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
@@ -2706,13 +2706,13 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>31.72237763757622</v>
+        <v>31.78169146795513</v>
       </c>
       <c r="C7">
-        <v>0.3172237763757622</v>
+        <v>0.3178169146795513</v>
       </c>
       <c r="D7">
-        <v>0.07736253202775667</v>
+        <v>2.29952184848818</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
@@ -2723,13 +2723,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>31.4536911902056</v>
+        <v>31.44654654213385</v>
       </c>
       <c r="C8">
-        <v>0.314536911902056</v>
+        <v>0.3144654654213385</v>
       </c>
       <c r="D8">
-        <v>0.09540179302624736</v>
+        <v>0.4071346820904629</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>31.09975466141803</v>
+        <v>31.18931185426068</v>
       </c>
       <c r="C9">
-        <v>0.3109975466141803</v>
+        <v>0.3118931185426068</v>
       </c>
       <c r="D9">
-        <v>0.7665373836362906</v>
+        <v>1.60852713057399</v>
       </c>
       <c r="E9" t="s">
         <v>53</v>
@@ -2757,13 +2757,13 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>30.74894225061348</v>
+        <v>30.71965126342241</v>
       </c>
       <c r="C10">
-        <v>0.3074894225061348</v>
+        <v>0.3071965126342242</v>
       </c>
       <c r="D10">
-        <v>0.1294140220388227</v>
+        <v>0.3463314424565727</v>
       </c>
       <c r="E10" t="s">
         <v>53</v>
@@ -2774,13 +2774,13 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>30.64220773900106</v>
+        <v>30.64016474060952</v>
       </c>
       <c r="C11">
-        <v>0.3064220773900106</v>
+        <v>0.3064016474060952</v>
       </c>
       <c r="D11">
-        <v>0.4958172558345752</v>
+        <v>0.5011521744681643</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
@@ -2791,13 +2791,13 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.18988606545343</v>
+        <v>30.13623579359739</v>
       </c>
       <c r="C12">
-        <v>0.3018988606545343</v>
+        <v>0.3013623579359739</v>
       </c>
       <c r="D12">
-        <v>0.02240792186759727</v>
+        <v>0.01872739301107361</v>
       </c>
       <c r="E12" t="s">
         <v>53</v>
@@ -2808,13 +2808,13 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.06060034708136</v>
+        <v>30.12615794086164</v>
       </c>
       <c r="C13">
-        <v>0.3006060034708136</v>
+        <v>0.3012615794086164</v>
       </c>
       <c r="D13">
-        <v>122.1975623865096</v>
+        <v>0.4581963093900052</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -2825,13 +2825,13 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.92527547559689</v>
+        <v>29.9263870009361</v>
       </c>
       <c r="C14">
-        <v>0.2992527547559689</v>
+        <v>0.2992638700093609</v>
       </c>
       <c r="D14">
-        <v>1.270764041941488</v>
+        <v>0.91209501881235</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
@@ -2842,13 +2842,13 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.81218446214374</v>
+        <v>29.75340933964809</v>
       </c>
       <c r="C15">
-        <v>0.2981218446214374</v>
+        <v>0.2975340933964809</v>
       </c>
       <c r="D15">
-        <v>0.02352049792379084</v>
+        <v>0.1042334800646023</v>
       </c>
       <c r="E15" t="s">
         <v>53</v>
@@ -2859,13 +2859,13 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.370249166628</v>
+        <v>28.36780912356847</v>
       </c>
       <c r="C16">
-        <v>0.28370249166628</v>
+        <v>0.2836780912356848</v>
       </c>
       <c r="D16">
-        <v>28.94935554520167</v>
+        <v>2.032031507937377</v>
       </c>
       <c r="E16" t="s">
         <v>53</v>
@@ -2876,13 +2876,13 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>28.04633464108334</v>
+        <v>27.99073492158428</v>
       </c>
       <c r="C17">
-        <v>0.2804633464108334</v>
+        <v>0.2799073492158428</v>
       </c>
       <c r="D17">
-        <v>0.05909220983449624</v>
+        <v>0.1737369745932467</v>
       </c>
       <c r="E17" t="s">
         <v>53</v>
@@ -2893,13 +2893,13 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>27.91074965424614</v>
+        <v>27.86734463674831</v>
       </c>
       <c r="C18">
-        <v>0.2791074965424614</v>
+        <v>0.2786734463674831</v>
       </c>
       <c r="D18">
-        <v>0.09790235551006166</v>
+        <v>0.1818265555804337</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
@@ -2910,13 +2910,13 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>27.81855794495917</v>
+        <v>27.86341678813201</v>
       </c>
       <c r="C19">
-        <v>0.2781855794495917</v>
+        <v>0.2786341678813201</v>
       </c>
       <c r="D19">
-        <v>0.2098867176526764</v>
+        <v>0.1086568950192935</v>
       </c>
       <c r="E19" t="s">
         <v>53</v>
@@ -2927,13 +2927,13 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>26.92219524279917</v>
+        <v>26.89127375582474</v>
       </c>
       <c r="C20">
-        <v>0.2692219524279917</v>
+        <v>0.2689127375582474</v>
       </c>
       <c r="D20">
-        <v>0.01922247660676361</v>
+        <v>0.05066257550904286</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
@@ -2944,13 +2944,13 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>26.58709734155243</v>
+        <v>26.58290038321374</v>
       </c>
       <c r="C21">
-        <v>0.2658709734155243</v>
+        <v>0.2658290038321374</v>
       </c>
       <c r="D21">
-        <v>0.3025764917042946</v>
+        <v>1.379465515696629</v>
       </c>
       <c r="E21" t="s">
         <v>53</v>
@@ -2961,13 +2961,13 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>25.64555893993454</v>
+        <v>25.64371883857743</v>
       </c>
       <c r="C22">
-        <v>0.2564555893993454</v>
+        <v>0.2564371883857743</v>
       </c>
       <c r="D22">
-        <v>0.3339671425902669</v>
+        <v>61.9413498516363</v>
       </c>
       <c r="E22" t="s">
         <v>53</v>
@@ -2978,13 +2978,13 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>25.42170725018393</v>
+        <v>25.43585740375006</v>
       </c>
       <c r="C23">
-        <v>0.2542170725018393</v>
+        <v>0.2543585740375006</v>
       </c>
       <c r="D23">
-        <v>0.1284163666525047</v>
+        <v>0.3170050636327296</v>
       </c>
       <c r="E23" t="s">
         <v>53</v>
@@ -2995,13 +2995,13 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>25.00351546734926</v>
+        <v>25.02641650667483</v>
       </c>
       <c r="C24">
-        <v>0.2500351546734926</v>
+        <v>0.2502641650667483</v>
       </c>
       <c r="D24">
-        <v>595.3217968416491</v>
+        <v>0.7104772301515914</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
@@ -3012,13 +3012,13 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>24.89356445131572</v>
+        <v>24.92259108613786</v>
       </c>
       <c r="C25">
-        <v>0.2489356445131572</v>
+        <v>0.2492259108613786</v>
       </c>
       <c r="D25">
-        <v>3111.695556414465</v>
+        <v>0.4042571437519778</v>
       </c>
       <c r="E25" t="s">
         <v>53</v>
@@ -3029,13 +3029,13 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>24.71480783542341</v>
+        <v>24.70927993073185</v>
       </c>
       <c r="C26">
-        <v>0.2471480783542341</v>
+        <v>0.2470927993073185</v>
       </c>
       <c r="D26">
-        <v>0.2840717490954807</v>
+        <v>0.5195921667853921</v>
       </c>
       <c r="E26" t="s">
         <v>53</v>
@@ -3046,13 +3046,13 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>24.34039125780323</v>
+        <v>24.29880101543948</v>
       </c>
       <c r="C27">
-        <v>0.2434039125780323</v>
+        <v>0.2429880101543948</v>
       </c>
       <c r="D27">
-        <v>0.05654603161249798</v>
+        <v>0.1168184849651434</v>
       </c>
       <c r="E27" t="s">
         <v>53</v>
@@ -3063,13 +3063,13 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>24.19971116355993</v>
+        <v>24.1887757609856</v>
       </c>
       <c r="C28">
-        <v>0.2419971116355993</v>
+        <v>0.241887757609856</v>
       </c>
       <c r="D28">
-        <v>0.155875204758471</v>
+        <v>1.94903291640164</v>
       </c>
       <c r="E28" t="s">
         <v>53</v>
@@ -3080,13 +3080,13 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>23.91003170481376</v>
+        <v>23.84761048073232</v>
       </c>
       <c r="C29">
-        <v>0.2391003170481376</v>
+        <v>0.2384761048073232</v>
       </c>
       <c r="D29">
-        <v>0.03861376555592327</v>
+        <v>0.0839921973257893</v>
       </c>
       <c r="E29" t="s">
         <v>53</v>
@@ -3097,13 +3097,13 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>22.29468225530591</v>
+        <v>22.27320123866313</v>
       </c>
       <c r="C30">
-        <v>0.2229468225530591</v>
+        <v>0.2227320123866313</v>
       </c>
       <c r="D30">
-        <v>0.2424406633213718</v>
+        <v>0.4817840397564462</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -3114,13 +3114,13 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>21.84516409866361</v>
+        <v>21.84782342798901</v>
       </c>
       <c r="C31">
-        <v>0.2184516409866361</v>
+        <v>0.2184782342798901</v>
       </c>
       <c r="D31">
-        <v>0.3784559551535129</v>
+        <v>0.4857028129768797</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
@@ -3131,13 +3131,13 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.39784661786715</v>
+        <v>17.37297547796422</v>
       </c>
       <c r="C32">
-        <v>1.391827729429372</v>
+        <v>1.389838038237137</v>
       </c>
       <c r="D32">
-        <v>0.07406204104576135</v>
+        <v>0.28933606790955</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
@@ -3148,13 +3148,13 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>16.81448622390124</v>
+        <v>16.87583236079463</v>
       </c>
       <c r="C33">
-        <v>0.1681448622390124</v>
+        <v>0.1687583236079463</v>
       </c>
       <c r="D33">
-        <v>3.695306209829995</v>
+        <v>7.748096209000729</v>
       </c>
       <c r="E33" t="s">
         <v>53</v>
@@ -3205,28 +3205,28 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="C2">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2">
-        <v>7.763805358119191</v>
+        <v>7.696506550218341</v>
       </c>
       <c r="F2">
-        <v>1582.18550269756</v>
+        <v>1585.009293976932</v>
       </c>
       <c r="G2">
-        <v>5647.08500666927</v>
+        <v>5647.092381292968</v>
       </c>
       <c r="H2">
-        <v>-3560.672350357786</v>
+        <v>-3561.013608007631</v>
       </c>
       <c r="I2">
-        <v>9207.757357027056</v>
+        <v>9208.105989300599</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -3234,28 +3234,28 @@
         <v>16</v>
       </c>
       <c r="B3">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="C3">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="D3">
         <v>13</v>
       </c>
       <c r="E3">
-        <v>-1.158106747230614</v>
+        <v>-1.206636500754148</v>
       </c>
       <c r="F3">
-        <v>8782.851034597345</v>
+        <v>8778.177991933831</v>
       </c>
       <c r="G3">
-        <v>22104.4451622506</v>
+        <v>22104.53632504945</v>
       </c>
       <c r="H3">
-        <v>-22304.95333234101</v>
+        <v>-22303.62506864941</v>
       </c>
       <c r="I3">
-        <v>44409.39849459161</v>
+        <v>44408.16139369886</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3263,28 +3263,28 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="C4">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="D4">
         <v>13</v>
       </c>
       <c r="E4">
-        <v>3.474320241691843</v>
+        <v>3.418803418803419</v>
       </c>
       <c r="F4">
-        <v>489.1394320136766</v>
+        <v>489.2715518923671</v>
       </c>
       <c r="G4">
-        <v>1270.019007027972</v>
+        <v>1270.118216005645</v>
       </c>
       <c r="H4">
-        <v>-1225.824591817038</v>
+        <v>-1225.901388765083</v>
       </c>
       <c r="I4">
-        <v>2495.843598845009</v>
+        <v>2496.019604770727</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3292,28 +3292,28 @@
         <v>38</v>
       </c>
       <c r="B5">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="C5">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="D5">
         <v>13</v>
       </c>
       <c r="E5">
-        <v>9.013091641490432</v>
+        <v>8.949220713926596</v>
       </c>
       <c r="F5">
-        <v>1610.624237679394</v>
+        <v>1613.233263281603</v>
       </c>
       <c r="G5">
-        <v>6330.922228694834</v>
+        <v>6330.998957244219</v>
       </c>
       <c r="H5">
-        <v>-3576.600178267585</v>
+        <v>-3576.945365825717</v>
       </c>
       <c r="I5">
-        <v>9907.52240696242</v>
+        <v>9907.944323069936</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3321,28 +3321,28 @@
         <v>26</v>
       </c>
       <c r="B6">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C6">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="D6">
         <v>13</v>
       </c>
       <c r="E6">
-        <v>10.32225579053374</v>
+        <v>10.25641025641026</v>
       </c>
       <c r="F6">
-        <v>1550.394591692891</v>
+        <v>1552.29101435198</v>
       </c>
       <c r="G6">
-        <v>5874.704994812187</v>
+        <v>5874.361641401896</v>
       </c>
       <c r="H6">
-        <v>-3635.856719494201</v>
+        <v>-3637.012817908294</v>
       </c>
       <c r="I6">
-        <v>9510.561714306388</v>
+        <v>9511.374459310191</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3350,28 +3350,28 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="C7">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="D7">
         <v>13</v>
       </c>
       <c r="E7">
-        <v>3.37361530715005</v>
+        <v>3.418803418803419</v>
       </c>
       <c r="F7">
-        <v>1715.123927007434</v>
+        <v>1717.031286571692</v>
       </c>
       <c r="G7">
-        <v>4632.65441010321</v>
+        <v>4632.636963088779</v>
       </c>
       <c r="H7">
-        <v>-4241.537864060496</v>
+        <v>-4241.471664834472</v>
       </c>
       <c r="I7">
-        <v>8874.192274163706</v>
+        <v>8874.108627923251</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3379,28 +3379,28 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C8">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="D8">
         <v>13</v>
       </c>
       <c r="E8">
-        <v>2.668680765357502</v>
+        <v>2.61437908496732</v>
       </c>
       <c r="F8">
-        <v>452.3898452300301</v>
+        <v>452.2598470245931</v>
       </c>
       <c r="G8">
-        <v>1367.270940718231</v>
+        <v>1367.273490200258</v>
       </c>
       <c r="H8">
-        <v>-1094.344792285929</v>
+        <v>-1094.147509371898</v>
       </c>
       <c r="I8">
-        <v>2461.61573300416</v>
+        <v>2461.420999572157</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3408,28 +3408,28 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C9">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="D9">
         <v>13</v>
       </c>
       <c r="E9">
-        <v>2.467270896273917</v>
+        <v>2.413273001508296</v>
       </c>
       <c r="F9">
-        <v>160.9550660773171</v>
+        <v>161.2664368512376</v>
       </c>
       <c r="G9">
-        <v>469.4479732270972</v>
+        <v>469.4436033030745</v>
       </c>
       <c r="H9">
-        <v>-389.7768638411682</v>
+        <v>-389.769584041486</v>
       </c>
       <c r="I9">
-        <v>859.2248370682653</v>
+        <v>859.2131873445605</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3437,28 +3437,28 @@
         <v>37</v>
       </c>
       <c r="B10">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="C10">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="D10">
         <v>13</v>
       </c>
       <c r="E10">
-        <v>13.34340382678751</v>
+        <v>13.27300150829563</v>
       </c>
       <c r="F10">
-        <v>1156.424715557943</v>
+        <v>1155.693789803296</v>
       </c>
       <c r="G10">
-        <v>6260.490184733791</v>
+        <v>6260.359337443201</v>
       </c>
       <c r="H10">
-        <v>-1710.393336261974</v>
+        <v>-1710.401176537438</v>
       </c>
       <c r="I10">
-        <v>7970.883520995765</v>
+        <v>7970.760513980638</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3466,28 +3466,28 @@
         <v>21</v>
       </c>
       <c r="B11">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="C11">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="D11">
         <v>13</v>
       </c>
       <c r="E11">
-        <v>7.200402819738168</v>
+        <v>7.239819004524888</v>
       </c>
       <c r="F11">
-        <v>2160.839328937651</v>
+        <v>2160.661860351579</v>
       </c>
       <c r="G11">
-        <v>7985.546445169778</v>
+        <v>7985.426603950807</v>
       </c>
       <c r="H11">
-        <v>-4162.077370477952</v>
+        <v>-4162.32250779399</v>
       </c>
       <c r="I11">
-        <v>12147.62381564773</v>
+        <v>12147.7491117448</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3495,28 +3495,28 @@
         <v>42</v>
       </c>
       <c r="B12">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C12">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="D12">
         <v>523</v>
       </c>
       <c r="E12">
-        <v>11.22860020140987</v>
+        <v>11.16138763197587</v>
       </c>
       <c r="F12">
-        <v>566.1636402505877</v>
+        <v>565.7810746915433</v>
       </c>
       <c r="G12">
-        <v>1482.20122706736</v>
+        <v>1482.194988097972</v>
       </c>
       <c r="H12">
-        <v>-1209.457105624324</v>
+        <v>-1209.557057933266</v>
       </c>
       <c r="I12">
-        <v>2691.658332691683</v>
+        <v>2691.752046031238</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3527,25 +3527,25 @@
         <v>1113</v>
       </c>
       <c r="C13">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="D13">
         <v>13</v>
       </c>
       <c r="E13">
-        <v>12.73917421953676</v>
+        <v>12.56913021618904</v>
       </c>
       <c r="F13">
-        <v>687.6332181306867</v>
+        <v>687.5088571755219</v>
       </c>
       <c r="G13">
-        <v>2785.523422243646</v>
+        <v>2785.462298799501</v>
       </c>
       <c r="H13">
-        <v>-1305.125501319638</v>
+        <v>-1305.248720480039</v>
       </c>
       <c r="I13">
-        <v>4090.648923563283</v>
+        <v>4090.71101927954</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3556,25 +3556,25 @@
         <v>1051</v>
       </c>
       <c r="C14">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="D14">
         <v>13</v>
       </c>
       <c r="E14">
-        <v>6.495468277945619</v>
+        <v>6.334841628959276</v>
       </c>
       <c r="F14">
-        <v>4366.912797068665</v>
+        <v>4363.65315664418</v>
       </c>
       <c r="G14">
-        <v>14065.59776483566</v>
+        <v>14065.5896457944</v>
       </c>
       <c r="H14">
-        <v>-11448.93404199938</v>
+        <v>-11448.92569371443</v>
       </c>
       <c r="I14">
-        <v>25514.53180683504</v>
+        <v>25514.51533950883</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3582,28 +3582,28 @@
         <v>39</v>
       </c>
       <c r="B15">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="C15">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="D15">
         <v>13</v>
       </c>
       <c r="E15">
-        <v>13.74622356495468</v>
+        <v>13.77576671694319</v>
       </c>
       <c r="F15">
-        <v>137.4547764192454</v>
+        <v>137.438110803502</v>
       </c>
       <c r="G15">
-        <v>655.8785328240326</v>
+        <v>655.8597916156754</v>
       </c>
       <c r="H15">
-        <v>-247.9996126297238</v>
+        <v>-248.0128773374849</v>
       </c>
       <c r="I15">
-        <v>903.8781454537565</v>
+        <v>903.8726689531602</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -3611,36 +3611,36 @@
         <v>24</v>
       </c>
       <c r="B16">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C16">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="D16">
         <v>13</v>
       </c>
       <c r="E16">
-        <v>5.589123867069486</v>
+        <v>5.530417295123177</v>
       </c>
       <c r="F16">
-        <v>925.617104963203</v>
+        <v>926.827847227338</v>
       </c>
       <c r="G16">
-        <v>2951.394275712775</v>
+        <v>2951.36214092612</v>
       </c>
       <c r="H16">
-        <v>-2006.17108766435</v>
+        <v>-2006.211329380025</v>
       </c>
       <c r="I16">
-        <v>4957.565363377125</v>
+        <v>4957.573470306144</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17">
-        <v>1061</v>
+        <v>1064</v>
       </c>
       <c r="C17">
         <v>912</v>
@@ -3649,19 +3649,19 @@
         <v>13</v>
       </c>
       <c r="E17">
-        <v>7.502517623363544</v>
+        <v>7.642031171442937</v>
       </c>
       <c r="F17">
-        <v>12409.13482501274</v>
+        <v>12406.43304259666</v>
       </c>
       <c r="G17">
-        <v>49348.41717659444</v>
+        <v>49348.67379146895</v>
       </c>
       <c r="H17">
-        <v>-26084.33759885255</v>
+        <v>-26081.95127362661</v>
       </c>
       <c r="I17">
-        <v>75432.754775447</v>
+        <v>75430.62506509556</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3669,28 +3669,28 @@
         <v>12</v>
       </c>
       <c r="B18">
-        <v>1029</v>
+        <v>1031</v>
       </c>
       <c r="C18">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="D18">
         <v>13</v>
       </c>
       <c r="E18">
-        <v>4.279959718026183</v>
+        <v>4.323780794369029</v>
       </c>
       <c r="F18">
-        <v>1065.513421735786</v>
+        <v>1066.107729250353</v>
       </c>
       <c r="G18">
-        <v>2740.065434057728</v>
+        <v>2740.147639785808</v>
       </c>
       <c r="H18">
-        <v>-2876.551855667558</v>
+        <v>-2876.596390259504</v>
       </c>
       <c r="I18">
-        <v>5616.617289725285</v>
+        <v>5616.744030045312</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3698,28 +3698,28 @@
         <v>41</v>
       </c>
       <c r="B19">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="C19">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D19">
         <v>523</v>
       </c>
       <c r="E19">
-        <v>12.33635448136959</v>
+        <v>12.36802413273002</v>
       </c>
       <c r="F19">
-        <v>286.9776129381477</v>
+        <v>286.7246322488215</v>
       </c>
       <c r="G19">
-        <v>913.1261561402706</v>
+        <v>913.1242359262289</v>
       </c>
       <c r="H19">
-        <v>-365.9226854831737</v>
+        <v>-365.9213364631102</v>
       </c>
       <c r="I19">
-        <v>1279.048841623444</v>
+        <v>1279.045572389339</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -3727,28 +3727,28 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C20">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="D20">
         <v>13</v>
       </c>
       <c r="E20">
-        <v>4.984894259818732</v>
+        <v>4.927099044746104</v>
       </c>
       <c r="F20">
-        <v>409.9648659393378</v>
+        <v>410.1719105721406</v>
       </c>
       <c r="G20">
-        <v>1182.937747314905</v>
+        <v>1183.026220440097</v>
       </c>
       <c r="H20">
-        <v>-798.435920413271</v>
+        <v>-798.6481471121839</v>
       </c>
       <c r="I20">
-        <v>1981.373667728176</v>
+        <v>1981.674367552281</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -3756,28 +3756,28 @@
         <v>17</v>
       </c>
       <c r="B21">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C21">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="D21">
         <v>13</v>
       </c>
       <c r="E21">
-        <v>4.179254783484391</v>
+        <v>4.122674710910005</v>
       </c>
       <c r="F21">
-        <v>6354.544104641453</v>
+        <v>6352.937380486177</v>
       </c>
       <c r="G21">
-        <v>17097.19812753373</v>
+        <v>17096.5200419668</v>
       </c>
       <c r="H21">
-        <v>-15706.78355053223</v>
+        <v>-15706.48856670671</v>
       </c>
       <c r="I21">
-        <v>32803.98167806596</v>
+        <v>32803.00860867351</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -3785,57 +3785,57 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="C22">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="D22">
         <v>13</v>
       </c>
       <c r="E22">
-        <v>5.790533736153072</v>
+        <v>5.832076420311714</v>
       </c>
       <c r="F22">
-        <v>7851.912546941659</v>
+        <v>7846.13566433406</v>
       </c>
       <c r="G22">
-        <v>27847.82032510472</v>
+        <v>27843.83666164801</v>
       </c>
       <c r="H22">
-        <v>-24636.61950858963</v>
+        <v>-24637.97202697679</v>
       </c>
       <c r="I22">
-        <v>52484.43983369436</v>
+        <v>52481.8086886248</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="C23">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="D23">
         <v>13</v>
       </c>
       <c r="E23">
-        <v>5.387713997985901</v>
+        <v>5.329311211664153</v>
       </c>
       <c r="F23">
-        <v>1741.741198767982</v>
+        <v>1740.782286402502</v>
       </c>
       <c r="G23">
-        <v>5998.107191266442</v>
+        <v>5998.138664117503</v>
       </c>
       <c r="H23">
-        <v>-4075.019710365549</v>
+        <v>-4074.417671189571</v>
       </c>
       <c r="I23">
-        <v>10073.12690163199</v>
+        <v>10072.55633530707</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -3843,28 +3843,28 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C24">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="D24">
         <v>13</v>
       </c>
       <c r="E24">
-        <v>2.668680765357502</v>
+        <v>2.61437908496732</v>
       </c>
       <c r="F24">
-        <v>2007.680693683339</v>
+        <v>2006.636464335872</v>
       </c>
       <c r="G24">
-        <v>6423.095741478633</v>
+        <v>6423.42976944728</v>
       </c>
       <c r="H24">
-        <v>-7169.727991355255</v>
+        <v>-7169.941195106214</v>
       </c>
       <c r="I24">
-        <v>13592.82373283389</v>
+        <v>13593.37096455349</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -3872,28 +3872,28 @@
         <v>30</v>
       </c>
       <c r="B25">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C25">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="D25">
         <v>13</v>
       </c>
       <c r="E25">
-        <v>9.919436052366565</v>
+        <v>9.854198089492208</v>
       </c>
       <c r="F25">
-        <v>1142.747496011017</v>
+        <v>1142.582012013234</v>
       </c>
       <c r="G25">
-        <v>4707.667503827134</v>
+        <v>4707.481513579053</v>
       </c>
       <c r="H25">
-        <v>-2075.540382065944</v>
+        <v>-2076.174657615929</v>
       </c>
       <c r="I25">
-        <v>6783.207885893078</v>
+        <v>6783.656171194983</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -3901,28 +3901,28 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C26">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="D26">
         <v>13</v>
       </c>
       <c r="E26">
-        <v>12.23564954682779</v>
+        <v>12.16691804927099</v>
       </c>
       <c r="F26">
-        <v>4422.58808674209</v>
+        <v>4419.687736443002</v>
       </c>
       <c r="G26">
-        <v>15255.47290251223</v>
+        <v>15255.18736558071</v>
       </c>
       <c r="H26">
-        <v>-9918.728530411707</v>
+        <v>-9917.756211744476</v>
       </c>
       <c r="I26">
-        <v>25174.20143292394</v>
+        <v>25172.94357732519</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -3930,28 +3930,28 @@
         <v>18</v>
       </c>
       <c r="B27">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="C27">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="D27">
         <v>13</v>
       </c>
       <c r="E27">
-        <v>0.5538771399798591</v>
+        <v>0.5027652086475616</v>
       </c>
       <c r="F27">
-        <v>377.7840457136699</v>
+        <v>377.5852281798587</v>
       </c>
       <c r="G27">
-        <v>891.5597399883815</v>
+        <v>891.5954418183245</v>
       </c>
       <c r="H27">
-        <v>-941.1109382317464</v>
+        <v>-941.1139484531096</v>
       </c>
       <c r="I27">
-        <v>1832.670678220128</v>
+        <v>1832.709390271434</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3959,28 +3959,28 @@
         <v>40</v>
       </c>
       <c r="B28">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C28">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="D28">
         <v>13</v>
       </c>
       <c r="E28">
-        <v>8.91238670694864</v>
+        <v>8.848667672197084</v>
       </c>
       <c r="F28">
-        <v>555.0698388277211</v>
+        <v>554.8874634674929</v>
       </c>
       <c r="G28">
-        <v>1926.340622583054</v>
+        <v>1926.177013913394</v>
       </c>
       <c r="H28">
-        <v>-998.4053112693439</v>
+        <v>-998.5254631997432</v>
       </c>
       <c r="I28">
-        <v>2924.745933852398</v>
+        <v>2924.702477113137</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -3988,28 +3988,28 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C29">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="D29">
         <v>13</v>
       </c>
       <c r="E29">
-        <v>5.991943605236657</v>
+        <v>5.932629462041226</v>
       </c>
       <c r="F29">
-        <v>233.9362858407761</v>
+        <v>233.8591731048626</v>
       </c>
       <c r="G29">
-        <v>841.676700890844</v>
+        <v>841.6696479396144</v>
       </c>
       <c r="H29">
-        <v>-512.8126176442734</v>
+        <v>-512.8142704891862</v>
       </c>
       <c r="I29">
-        <v>1354.489318535117</v>
+        <v>1354.483918428801</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -4017,7 +4017,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>1098</v>
+        <v>1101</v>
       </c>
       <c r="C30">
         <v>875</v>
@@ -4026,19 +4026,19 @@
         <v>13</v>
       </c>
       <c r="E30">
-        <v>11.22860020140987</v>
+        <v>11.36249371543489</v>
       </c>
       <c r="F30">
-        <v>2495.380843643699</v>
+        <v>2494.472949303092</v>
       </c>
       <c r="G30">
-        <v>9347.63001203728</v>
+        <v>9347.542840980799</v>
       </c>
       <c r="H30">
-        <v>-4110.066022308999</v>
+        <v>-4110.045844454616</v>
       </c>
       <c r="I30">
-        <v>13457.69603434628</v>
+        <v>13457.58868543541</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -4046,28 +4046,28 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C31">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="D31">
         <v>13</v>
       </c>
       <c r="E31">
-        <v>7.502517623363544</v>
+        <v>7.440925087983912</v>
       </c>
       <c r="F31">
-        <v>1110.632465201031</v>
+        <v>1109.858721229039</v>
       </c>
       <c r="G31">
-        <v>4654.210717852787</v>
+        <v>4654.141362070584</v>
       </c>
       <c r="H31">
-        <v>-2958.818390573676</v>
+        <v>-2959.446948303254</v>
       </c>
       <c r="I31">
-        <v>7613.029108426463</v>
+        <v>7613.588310373838</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -4078,25 +4078,25 @@
         <v>1105</v>
       </c>
       <c r="C32">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="D32">
         <v>13</v>
       </c>
       <c r="E32">
-        <v>11.93353474320242</v>
+        <v>11.76470588235294</v>
       </c>
       <c r="F32">
-        <v>1318.131280050635</v>
+        <v>1319.260478011091</v>
       </c>
       <c r="G32">
-        <v>5108.965485607055</v>
+        <v>5108.877694986662</v>
       </c>
       <c r="H32">
-        <v>-2727.629891746783</v>
+        <v>-2727.577603954907</v>
       </c>
       <c r="I32">
-        <v>7836.595377353837</v>
+        <v>7836.45529894157</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4104,28 +4104,28 @@
         <v>14</v>
       </c>
       <c r="B33">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C33">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="D33">
         <v>13</v>
       </c>
       <c r="E33">
-        <v>2.668680765357502</v>
+        <v>2.61437908496732</v>
       </c>
       <c r="F33">
-        <v>1175.168401514772</v>
+        <v>1174.727185976258</v>
       </c>
       <c r="G33">
-        <v>3493.569774832687</v>
+        <v>3493.573101921227</v>
       </c>
       <c r="H33">
-        <v>-2663.473171399757</v>
+        <v>-2663.491714014139</v>
       </c>
       <c r="I33">
-        <v>6157.042946232443</v>
+        <v>6157.064815935366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
learning pysystemtrade. Output leverage report
</commit_message>
<xml_diff>
--- a/perplexity_examples/etf_turnover_analysis.xlsx
+++ b/perplexity_examples/etf_turnover_analysis.xlsx
@@ -607,31 +607,31 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>35.42572289384545</v>
+        <v>35.4262885326072</v>
       </c>
       <c r="C2">
-        <v>7.113475164787117</v>
+        <v>7.113361586496797</v>
       </c>
       <c r="D2">
-        <v>1.016210737826731</v>
+        <v>1.016194512356685</v>
       </c>
       <c r="E2">
-        <v>132.1796456838034</v>
+        <v>132.1809580652812</v>
       </c>
       <c r="F2">
-        <v>73917.54639603154</v>
+        <v>73919.46055179287</v>
       </c>
       <c r="G2">
         <v>1989</v>
       </c>
       <c r="H2">
-        <v>0.3542572289384545</v>
+        <v>0.354262885326072</v>
       </c>
       <c r="I2">
         <v>-6.600151062011719</v>
       </c>
       <c r="J2">
-        <v>5.367410921508171</v>
+        <v>5.367496622389322</v>
       </c>
       <c r="K2" t="s">
         <v>43</v>
@@ -645,31 +645,31 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>34.74690486441447</v>
+        <v>34.74734176259139</v>
       </c>
       <c r="C3">
-        <v>7.252444526593851</v>
+        <v>7.25235333746596</v>
       </c>
       <c r="D3">
-        <v>1.036063503799121</v>
+        <v>1.036050476780851</v>
       </c>
       <c r="E3">
-        <v>863.9608714153385</v>
+        <v>863.9673522510199</v>
       </c>
       <c r="F3">
-        <v>473886.6093891166</v>
+        <v>473896.1227246863</v>
       </c>
       <c r="G3">
         <v>1989</v>
       </c>
       <c r="H3">
-        <v>0.3474690486441447</v>
+        <v>0.3474734176259139</v>
       </c>
       <c r="I3">
         <v>401.9526816101074</v>
       </c>
       <c r="J3">
-        <v>0.08644526197767438</v>
+        <v>0.08644634891700057</v>
       </c>
       <c r="K3" t="s">
         <v>43</v>
@@ -683,31 +683,31 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>33.9259451318414</v>
+        <v>33.92606420981944</v>
       </c>
       <c r="C4">
-        <v>7.427943393196257</v>
+        <v>7.427917321663913</v>
       </c>
       <c r="D4">
-        <v>1.061134770456608</v>
+        <v>1.061131045951988</v>
       </c>
       <c r="E4">
-        <v>1429.40589897577</v>
+        <v>1429.414193576256</v>
       </c>
       <c r="F4">
-        <v>765511.5777179936</v>
+        <v>765518.7067661907</v>
       </c>
       <c r="G4">
         <v>1989</v>
       </c>
       <c r="H4">
-        <v>0.339259451318414</v>
+        <v>0.3392606420981945</v>
       </c>
       <c r="I4">
         <v>245.2347645568738</v>
       </c>
       <c r="J4">
-        <v>0.1383406842547132</v>
+        <v>0.138341169821995</v>
       </c>
       <c r="K4" t="s">
         <v>43</v>
@@ -721,31 +721,31 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>32.78771739399839</v>
+        <v>32.78814507822536</v>
       </c>
       <c r="C5">
-        <v>7.685804930297685</v>
+        <v>7.685704677674904</v>
       </c>
       <c r="D5">
-        <v>1.097972132899669</v>
+        <v>1.097957811096415</v>
       </c>
       <c r="E5">
-        <v>961.3348606746271</v>
+        <v>961.341682120413</v>
       </c>
       <c r="F5">
-        <v>497565.3312106048</v>
+        <v>497575.352144797</v>
       </c>
       <c r="G5">
         <v>1989</v>
       </c>
       <c r="H5">
-        <v>0.3278771739399839</v>
+        <v>0.3278814507822536</v>
       </c>
       <c r="I5">
         <v>106.2224682617187</v>
       </c>
       <c r="J5">
-        <v>0.308670264686503</v>
+        <v>0.3086742909931212</v>
       </c>
       <c r="K5" t="s">
         <v>43</v>
@@ -759,31 +759,31 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>32.37954735576731</v>
+        <v>32.38011844623587</v>
       </c>
       <c r="C6">
-        <v>7.78269063588731</v>
+        <v>7.78255337201506</v>
       </c>
       <c r="D6">
-        <v>1.111812947983901</v>
+        <v>1.111793338859294</v>
       </c>
       <c r="E6">
-        <v>1363.594079057384</v>
+        <v>1363.606189768687</v>
       </c>
       <c r="F6">
-        <v>641964.1920016565</v>
+        <v>641981.2162520178</v>
       </c>
       <c r="G6">
         <v>1832</v>
       </c>
       <c r="H6">
-        <v>0.3237954735576731</v>
+        <v>0.3238011844623587</v>
       </c>
       <c r="I6">
         <v>214.404259765625</v>
       </c>
       <c r="J6">
-        <v>0.151021007657044</v>
+        <v>0.1510236712723527</v>
       </c>
       <c r="K6" t="s">
         <v>43</v>
@@ -797,31 +797,31 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>31.78169146795513</v>
+        <v>31.78198761119699</v>
       </c>
       <c r="C7">
-        <v>7.929093398131021</v>
+        <v>7.929019515167732</v>
       </c>
       <c r="D7">
-        <v>1.132727628304431</v>
+        <v>1.13271707359539</v>
       </c>
       <c r="E7">
-        <v>7389.10853344669</v>
+        <v>7389.124595693119</v>
       </c>
       <c r="F7">
-        <v>3707091.374781814</v>
+        <v>3707133.976078431</v>
       </c>
       <c r="G7">
         <v>1989</v>
       </c>
       <c r="H7">
-        <v>0.3178169146795513</v>
+        <v>0.3178198761119699</v>
       </c>
       <c r="I7">
         <v>-13.821</v>
       </c>
       <c r="J7">
-        <v>2.29952184848818</v>
+        <v>2.299543275537008</v>
       </c>
       <c r="K7" t="s">
         <v>43</v>
@@ -835,31 +835,31 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>31.44654654213385</v>
+        <v>31.44673844578386</v>
       </c>
       <c r="C8">
-        <v>8.013598557232866</v>
+        <v>8.013549654265853</v>
       </c>
       <c r="D8">
-        <v>1.14479979389041</v>
+        <v>1.144792807752265</v>
       </c>
       <c r="E8">
-        <v>5305.564665988628</v>
+        <v>5305.590389526624</v>
       </c>
       <c r="F8">
-        <v>2633715.189320714</v>
+        <v>2633744.03106141</v>
       </c>
       <c r="G8">
         <v>1989</v>
       </c>
       <c r="H8">
-        <v>0.3144654654213385</v>
+        <v>0.3144673844578387</v>
       </c>
       <c r="I8">
         <v>-77.23868273925781</v>
       </c>
       <c r="J8">
-        <v>0.4071346820904629</v>
+        <v>0.4071371666440985</v>
       </c>
       <c r="K8" t="s">
         <v>43</v>
@@ -873,31 +873,31 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>31.18931185426068</v>
+        <v>31.18966740816405</v>
       </c>
       <c r="C9">
-        <v>8.079690926735692</v>
+        <v>8.079598820410562</v>
       </c>
       <c r="D9">
-        <v>1.154241560962242</v>
+        <v>1.154228402915795</v>
       </c>
       <c r="E9">
-        <v>320.6075848334035</v>
+        <v>320.6080973787314</v>
       </c>
       <c r="F9">
-        <v>157849.7227223206</v>
+        <v>157851.7745399376</v>
       </c>
       <c r="G9">
         <v>1989</v>
       </c>
       <c r="H9">
-        <v>0.3118931185426068</v>
+        <v>0.3118966740816405</v>
       </c>
       <c r="I9">
         <v>-19.38998184204144</v>
       </c>
       <c r="J9">
-        <v>1.60852713057399</v>
+        <v>1.608545467564002</v>
       </c>
       <c r="K9" t="s">
         <v>43</v>
@@ -911,31 +911,31 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>30.71965126342241</v>
+        <v>30.71999165275505</v>
       </c>
       <c r="C10">
-        <v>8.203218123769977</v>
+        <v>8.203127228955481</v>
       </c>
       <c r="D10">
-        <v>1.171888303395711</v>
+        <v>1.171875318422211</v>
       </c>
       <c r="E10">
-        <v>370.8858484260435</v>
+        <v>370.888473654779</v>
       </c>
       <c r="F10">
-        <v>179854.2819145171</v>
+        <v>179857.5478618507</v>
       </c>
       <c r="G10">
         <v>1989</v>
       </c>
       <c r="H10">
-        <v>0.3071965126342242</v>
+        <v>0.3071999165275505</v>
       </c>
       <c r="I10">
         <v>88.70015106201171</v>
       </c>
       <c r="J10">
-        <v>0.3463314424565727</v>
+        <v>0.3463352799847906</v>
       </c>
       <c r="K10" t="s">
         <v>43</v>
@@ -949,31 +949,31 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>30.64016474060952</v>
+        <v>30.64078406676243</v>
       </c>
       <c r="C11">
-        <v>8.224498860673783</v>
+        <v>8.224332623177121</v>
       </c>
       <c r="D11">
-        <v>1.174928408667683</v>
+        <v>1.174904660453874</v>
       </c>
       <c r="E11">
-        <v>6904.944411892532</v>
+        <v>6904.676360753147</v>
       </c>
       <c r="F11">
-        <v>3339762.012959683</v>
+        <v>3339699.866427021</v>
       </c>
       <c r="G11">
         <v>1989</v>
       </c>
       <c r="H11">
-        <v>0.3064016474060952</v>
+        <v>0.3064078406676243</v>
       </c>
       <c r="I11">
         <v>61.13944287107135</v>
       </c>
       <c r="J11">
-        <v>0.5011521744681643</v>
+        <v>0.50116230419987</v>
       </c>
       <c r="K11" t="s">
         <v>43</v>
@@ -987,31 +987,31 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.13623579359739</v>
+        <v>30.13693617866853</v>
       </c>
       <c r="C12">
-        <v>8.36202642313871</v>
+        <v>8.361832088902593</v>
       </c>
       <c r="D12">
-        <v>1.19457520330553</v>
+        <v>1.194547441271799</v>
       </c>
       <c r="E12">
-        <v>1787.52291772588</v>
+        <v>1787.529417676874</v>
       </c>
       <c r="F12">
-        <v>850363.9915603739</v>
+        <v>850386.8467958946</v>
       </c>
       <c r="G12">
         <v>1989</v>
       </c>
       <c r="H12">
-        <v>0.3013623579359739</v>
+        <v>0.3013693617866853</v>
       </c>
       <c r="I12">
         <v>1609.20613861084</v>
       </c>
       <c r="J12">
-        <v>0.01872739301107361</v>
+        <v>0.01872782824746399</v>
       </c>
       <c r="K12" t="s">
         <v>43</v>
@@ -1025,31 +1025,31 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.12615794086164</v>
+        <v>30.12633269952031</v>
       </c>
       <c r="C13">
-        <v>8.364823702201985</v>
+        <v>8.364775179025109</v>
       </c>
       <c r="D13">
-        <v>1.194974814600284</v>
+        <v>1.194967882717873</v>
       </c>
       <c r="E13">
-        <v>1701.633073447972</v>
+        <v>1701.627360868465</v>
       </c>
       <c r="F13">
-        <v>809233.5962076656</v>
+        <v>809235.5737794822</v>
       </c>
       <c r="G13">
         <v>1989</v>
       </c>
       <c r="H13">
-        <v>0.3012615794086164</v>
+        <v>0.3012633269952031</v>
       </c>
       <c r="I13">
         <v>-65.74945568847656</v>
       </c>
       <c r="J13">
-        <v>0.4581963093900052</v>
+        <v>0.4581989673383767</v>
       </c>
       <c r="K13" t="s">
         <v>43</v>
@@ -1063,31 +1063,31 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.9263870009361</v>
+        <v>29.92654172458437</v>
       </c>
       <c r="C14">
-        <v>8.420662340299129</v>
+        <v>8.420618804510392</v>
       </c>
       <c r="D14">
-        <v>1.202951762899876</v>
+        <v>1.202945543501485</v>
       </c>
       <c r="E14">
-        <v>427.7724841566396</v>
+        <v>427.7761280426009</v>
       </c>
       <c r="F14">
-        <v>202083.7403527408</v>
+        <v>202086.506569087</v>
       </c>
       <c r="G14">
         <v>1989</v>
       </c>
       <c r="H14">
-        <v>0.2992638700093609</v>
+        <v>0.2992654172458437</v>
       </c>
       <c r="I14">
         <v>32.81060238647461</v>
       </c>
       <c r="J14">
-        <v>0.91209501881235</v>
+        <v>0.9120997344724423</v>
       </c>
       <c r="K14" t="s">
         <v>43</v>
@@ -1101,31 +1101,31 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.75340933964809</v>
+        <v>29.75407563733193</v>
       </c>
       <c r="C15">
-        <v>8.469617620061976</v>
+        <v>8.469427955739278</v>
       </c>
       <c r="D15">
-        <v>1.209945374294568</v>
+        <v>1.209918279391325</v>
       </c>
       <c r="E15">
-        <v>758.0791458059637</v>
+        <v>758.0830011321223</v>
       </c>
       <c r="F15">
-        <v>356053.7178057463</v>
+        <v>356063.5020763162</v>
       </c>
       <c r="G15">
         <v>1989</v>
       </c>
       <c r="H15">
-        <v>0.2975340933964809</v>
+        <v>0.2975407563733193</v>
       </c>
       <c r="I15">
         <v>285.4496398010254</v>
       </c>
       <c r="J15">
-        <v>0.1042334800646023</v>
+        <v>0.1042358142685771</v>
       </c>
       <c r="K15" t="s">
         <v>43</v>
@@ -1139,31 +1139,31 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.36780912356847</v>
+        <v>28.36810925585355</v>
       </c>
       <c r="C16">
-        <v>8.883308503039594</v>
+        <v>8.883214518359262</v>
       </c>
       <c r="D16">
-        <v>1.269044071862799</v>
+        <v>1.269030645479895</v>
       </c>
       <c r="E16">
-        <v>354.0185952983485</v>
+        <v>354.0207313755438</v>
       </c>
       <c r="F16">
-        <v>158531.6970152459</v>
+        <v>158534.3308440137</v>
       </c>
       <c r="G16">
         <v>1989</v>
       </c>
       <c r="H16">
-        <v>0.2836780912356848</v>
+        <v>0.2836810925585355</v>
       </c>
       <c r="I16">
         <v>13.96031951904297</v>
       </c>
       <c r="J16">
-        <v>2.032031507937377</v>
+        <v>2.032053006892659</v>
       </c>
       <c r="K16" t="s">
         <v>43</v>
@@ -1177,31 +1177,31 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.99073492158428</v>
+        <v>27.99084571535667</v>
       </c>
       <c r="C17">
-        <v>9.002979046672946</v>
+        <v>9.002943410950413</v>
       </c>
       <c r="D17">
-        <v>1.286139863810421</v>
+        <v>1.286134772992916</v>
       </c>
       <c r="E17">
-        <v>1334.65123620699</v>
+        <v>1334.654976139376</v>
       </c>
       <c r="F17">
-        <v>589720.6458115036</v>
+        <v>589724.6325712443</v>
       </c>
       <c r="G17">
         <v>1989</v>
       </c>
       <c r="H17">
-        <v>0.2799073492158428</v>
+        <v>0.2799084571535668</v>
       </c>
       <c r="I17">
         <v>-161.1098327636719</v>
       </c>
       <c r="J17">
-        <v>0.1737369745932467</v>
+        <v>0.173737662284187</v>
       </c>
       <c r="K17" t="s">
         <v>43</v>
@@ -1215,31 +1215,31 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>27.86734463674831</v>
+        <v>27.86762591941144</v>
       </c>
       <c r="C18">
-        <v>9.042842197016892</v>
+        <v>9.042750922835776</v>
       </c>
       <c r="D18">
-        <v>1.291834599573842</v>
+        <v>1.291821560405111</v>
       </c>
       <c r="E18">
-        <v>1548.506461507993</v>
+        <v>1548.515176694957</v>
       </c>
       <c r="F18">
-        <v>681197.1910679678</v>
+        <v>681207.900721519</v>
       </c>
       <c r="G18">
         <v>1989</v>
       </c>
       <c r="H18">
-        <v>0.2786734463674831</v>
+        <v>0.2786762591941144</v>
       </c>
       <c r="I18">
         <v>-153.2633368530196</v>
       </c>
       <c r="J18">
-        <v>0.1818265555804337</v>
+        <v>0.1818283908703922</v>
       </c>
       <c r="K18" t="s">
         <v>43</v>
@@ -1253,31 +1253,31 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>27.86341678813201</v>
+        <v>27.86331388074051</v>
       </c>
       <c r="C19">
-        <v>9.044116947901934</v>
+        <v>9.044150350478796</v>
       </c>
       <c r="D19">
-        <v>1.292016706843133</v>
+        <v>1.292021478639828</v>
       </c>
       <c r="E19">
-        <v>10280.66305484551</v>
+        <v>10280.793428877</v>
       </c>
       <c r="F19">
-        <v>4521887.307269136</v>
+        <v>4521927.950689988</v>
       </c>
       <c r="G19">
         <v>1989</v>
       </c>
       <c r="H19">
-        <v>0.2786341678813201</v>
+        <v>0.2786331388074051</v>
       </c>
       <c r="I19">
         <v>256.4348703612825</v>
       </c>
       <c r="J19">
-        <v>0.1086568950192935</v>
+        <v>0.1086564937189892</v>
       </c>
       <c r="K19" t="s">
         <v>43</v>
@@ -1291,31 +1291,31 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>26.89127375582474</v>
+        <v>26.89193792180146</v>
       </c>
       <c r="C20">
-        <v>9.37106967442983</v>
+        <v>9.370838231621159</v>
       </c>
       <c r="D20">
-        <v>1.338724239204261</v>
+        <v>1.33869117594588</v>
       </c>
       <c r="E20">
-        <v>2175.075453597677</v>
+        <v>2175.084489611659</v>
       </c>
       <c r="F20">
-        <v>923315.1022258305</v>
+        <v>923341.7423083929</v>
       </c>
       <c r="G20">
         <v>1989</v>
       </c>
       <c r="H20">
-        <v>0.2689127375582474</v>
+        <v>0.2689193792180146</v>
       </c>
       <c r="I20">
         <v>530.7916837158203</v>
       </c>
       <c r="J20">
-        <v>0.05066257550904286</v>
+        <v>0.05066382678331315</v>
       </c>
       <c r="K20" t="s">
         <v>43</v>
@@ -1329,31 +1329,31 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>26.58290038321374</v>
+        <v>26.58309521360215</v>
       </c>
       <c r="C21">
-        <v>9.479778217095152</v>
+        <v>9.479708738772283</v>
       </c>
       <c r="D21">
-        <v>1.354254031013593</v>
+        <v>1.354244105538898</v>
       </c>
       <c r="E21">
-        <v>1030.994687356777</v>
+        <v>1030.993445959051</v>
       </c>
       <c r="F21">
-        <v>432636.3731705531</v>
+        <v>432639.0231010686</v>
       </c>
       <c r="G21">
         <v>1989</v>
       </c>
       <c r="H21">
-        <v>0.2658290038321374</v>
+        <v>0.2658309521360215</v>
       </c>
       <c r="I21">
         <v>-19.27043487548828</v>
       </c>
       <c r="J21">
-        <v>1.379465515696629</v>
+        <v>1.37947562602313</v>
       </c>
       <c r="K21" t="s">
         <v>43</v>
@@ -1367,31 +1367,31 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>25.64371883857743</v>
+        <v>25.64418419898893</v>
       </c>
       <c r="C22">
-        <v>9.826967827337928</v>
+        <v>9.826789499115185</v>
       </c>
       <c r="D22">
-        <v>1.403852546762561</v>
+        <v>1.403827071302169</v>
       </c>
       <c r="E22">
-        <v>639.694927808536</v>
+        <v>639.7006510838095</v>
       </c>
       <c r="F22">
-        <v>258951.333466582</v>
+        <v>258958.349544429</v>
       </c>
       <c r="G22">
         <v>1989</v>
       </c>
       <c r="H22">
-        <v>0.2564371883857743</v>
+        <v>0.2564418419898893</v>
       </c>
       <c r="I22">
         <v>-0.414</v>
       </c>
       <c r="J22">
-        <v>61.9413498516363</v>
+        <v>61.94247391060128</v>
       </c>
       <c r="K22" t="s">
         <v>43</v>
@@ -1405,31 +1405,31 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>25.43585740375006</v>
+        <v>25.43645733242202</v>
       </c>
       <c r="C23">
-        <v>9.907273657024323</v>
+        <v>9.907039990148068</v>
       </c>
       <c r="D23">
-        <v>1.415324808146332</v>
+        <v>1.41529142716401</v>
       </c>
       <c r="E23">
-        <v>3711.10209343682</v>
+        <v>3711.115713771949</v>
       </c>
       <c r="F23">
-        <v>1490093.504909373</v>
+        <v>1490134.119178434</v>
       </c>
       <c r="G23">
         <v>1989</v>
       </c>
       <c r="H23">
-        <v>0.2543585740375006</v>
+        <v>0.2543645733242202</v>
       </c>
       <c r="I23">
         <v>80.23801611326658</v>
       </c>
       <c r="J23">
-        <v>0.3170050636327296</v>
+        <v>0.3170125404959551</v>
       </c>
       <c r="K23" t="s">
         <v>43</v>
@@ -1443,31 +1443,31 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>25.02641650667483</v>
+        <v>25.02698299990121</v>
       </c>
       <c r="C24">
-        <v>10.06936010726061</v>
+        <v>10.06913218429064</v>
       </c>
       <c r="D24">
-        <v>1.438480015322944</v>
+        <v>1.438447454898663</v>
       </c>
       <c r="E24">
-        <v>875.8442398051288</v>
+        <v>875.8385690285694</v>
       </c>
       <c r="F24">
-        <v>346010.9032581476</v>
+        <v>346016.4951485439</v>
       </c>
       <c r="G24">
         <v>1989</v>
       </c>
       <c r="H24">
-        <v>0.2502641650667483</v>
+        <v>0.2502698299990121</v>
       </c>
       <c r="I24">
         <v>-35.22479742431022</v>
       </c>
       <c r="J24">
-        <v>0.7104772301515914</v>
+        <v>0.7104933123796749</v>
       </c>
       <c r="K24" t="s">
         <v>43</v>
@@ -1481,31 +1481,31 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>24.92259108613786</v>
+        <v>24.92314088746575</v>
       </c>
       <c r="C25">
-        <v>10.11130821546739</v>
+        <v>10.1110851612902</v>
       </c>
       <c r="D25">
-        <v>1.444472602209627</v>
+        <v>1.444440737327172</v>
       </c>
       <c r="E25">
-        <v>196.2664625466855</v>
+        <v>196.2673501909645</v>
       </c>
       <c r="F25">
-        <v>77215.32875601551</v>
+        <v>77217.38137947115</v>
       </c>
       <c r="G25">
         <v>1989</v>
       </c>
       <c r="H25">
-        <v>0.2492259108613786</v>
+        <v>0.2492314088746575</v>
       </c>
       <c r="I25">
         <v>-61.650341796875</v>
       </c>
       <c r="J25">
-        <v>0.4042571437519778</v>
+        <v>0.404266061810043</v>
       </c>
       <c r="K25" t="s">
         <v>43</v>
@@ -1519,31 +1519,31 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>24.70927993073185</v>
+        <v>24.70927720225878</v>
       </c>
       <c r="C26">
-        <v>10.19859747861686</v>
+        <v>10.19859860477682</v>
       </c>
       <c r="D26">
-        <v>1.456942496945265</v>
+        <v>1.456942657825259</v>
       </c>
       <c r="E26">
-        <v>4432.410688160371</v>
+        <v>4432.379412066235</v>
       </c>
       <c r="F26">
-        <v>1728877.89271719</v>
+        <v>1728865.502456486</v>
       </c>
       <c r="G26">
         <v>1989</v>
       </c>
       <c r="H26">
-        <v>0.2470927993073185</v>
+        <v>0.2470927720225878</v>
       </c>
       <c r="I26">
         <v>47.55514326477051</v>
       </c>
       <c r="J26">
-        <v>0.5195921667853921</v>
+        <v>0.519592109410461</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -1557,31 +1557,31 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>24.29880101543948</v>
+        <v>24.29921019445444</v>
       </c>
       <c r="C27">
-        <v>10.37088207932066</v>
+        <v>10.37070744206786</v>
       </c>
       <c r="D27">
-        <v>1.481554582760095</v>
+        <v>1.481529634581124</v>
       </c>
       <c r="E27">
-        <v>1151.275118243466</v>
+        <v>1151.268106096806</v>
       </c>
       <c r="F27">
-        <v>441599.1219786872</v>
+        <v>441603.8685534377</v>
       </c>
       <c r="G27">
         <v>1989</v>
       </c>
       <c r="H27">
-        <v>0.2429880101543948</v>
+        <v>0.2429921019445444</v>
       </c>
       <c r="I27">
         <v>-208.0047607421875</v>
       </c>
       <c r="J27">
-        <v>0.1168184849651434</v>
+        <v>0.1168204521269214</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -1595,31 +1595,31 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>24.1887757609856</v>
+        <v>24.18921788875688</v>
       </c>
       <c r="C28">
-        <v>10.41805515459175</v>
+        <v>10.41786473456545</v>
       </c>
       <c r="D28">
-        <v>1.488293593513107</v>
+        <v>1.488266390652207</v>
       </c>
       <c r="E28">
-        <v>1005.38259205839</v>
+        <v>1005.385486676372</v>
       </c>
       <c r="F28">
-        <v>383892.376442789</v>
+        <v>383900.4986049507</v>
       </c>
       <c r="G28">
         <v>1989</v>
       </c>
       <c r="H28">
-        <v>0.241887757609856</v>
+        <v>0.2418921788875688</v>
       </c>
       <c r="I28">
         <v>12.41065533446382</v>
       </c>
       <c r="J28">
-        <v>1.94903291640164</v>
+        <v>1.949068541254589</v>
       </c>
       <c r="K28" t="s">
         <v>43</v>
@@ -1633,31 +1633,31 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>23.84761048073232</v>
+        <v>23.84808825153807</v>
       </c>
       <c r="C29">
-        <v>10.56709644782245</v>
+        <v>10.56688474740727</v>
       </c>
       <c r="D29">
-        <v>1.509585206831779</v>
+        <v>1.509554963915324</v>
       </c>
       <c r="E29">
-        <v>1396.958348183458</v>
+        <v>1396.959663770117</v>
       </c>
       <c r="F29">
-        <v>525887.1570363058</v>
+        <v>525898.1880956958</v>
       </c>
       <c r="G29">
         <v>1989</v>
       </c>
       <c r="H29">
-        <v>0.2384761048073232</v>
+        <v>0.2384808825153807</v>
       </c>
       <c r="I29">
         <v>-283.9264984130859</v>
       </c>
       <c r="J29">
-        <v>0.0839921973257893</v>
+        <v>0.08399388005286275</v>
       </c>
       <c r="K29" t="s">
         <v>43</v>
@@ -1671,31 +1671,31 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>22.27320123866313</v>
+        <v>22.27358432658891</v>
       </c>
       <c r="C30">
-        <v>11.31404495024108</v>
+        <v>11.31385035767131</v>
       </c>
       <c r="D30">
-        <v>1.616292135748726</v>
+        <v>1.616264336810187</v>
       </c>
       <c r="E30">
-        <v>120.4841164011092</v>
+        <v>120.4847838188603</v>
       </c>
       <c r="F30">
-        <v>42362.02146548832</v>
+        <v>42362.98473812205</v>
       </c>
       <c r="G30">
         <v>1989</v>
       </c>
       <c r="H30">
-        <v>0.2227320123866313</v>
+        <v>0.2227358432658891</v>
       </c>
       <c r="I30">
         <v>46.23067474365234</v>
       </c>
       <c r="J30">
-        <v>0.4817840397564462</v>
+        <v>0.4817923262010612</v>
       </c>
       <c r="K30" t="s">
         <v>43</v>
@@ -1709,31 +1709,31 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>21.84782342798901</v>
+        <v>21.8484880608005</v>
       </c>
       <c r="C31">
-        <v>11.53432976198286</v>
+        <v>11.53397888671877</v>
       </c>
       <c r="D31">
-        <v>1.64776139456898</v>
+        <v>1.647711269531252</v>
       </c>
       <c r="E31">
-        <v>492.9679489466685</v>
+        <v>492.9602259944429</v>
       </c>
       <c r="F31">
-        <v>170016.5108312916</v>
+        <v>170019.0193051208</v>
       </c>
       <c r="G31">
         <v>1989</v>
       </c>
       <c r="H31">
-        <v>0.2184782342798901</v>
+        <v>0.218484880608005</v>
       </c>
       <c r="I31">
         <v>-44.9818754272461</v>
       </c>
       <c r="J31">
-        <v>0.4857028129768797</v>
+        <v>0.4857175885460434</v>
       </c>
       <c r="K31" t="s">
         <v>43</v>
@@ -1747,31 +1747,31 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.37297547796422</v>
+        <v>17.37343004598634</v>
       </c>
       <c r="C32">
-        <v>14.50528726755157</v>
+        <v>14.50490774320168</v>
       </c>
       <c r="D32">
-        <v>2.07218389536451</v>
+        <v>2.07212967760024</v>
       </c>
       <c r="E32">
-        <v>297.7613105732244</v>
+        <v>297.7632741667148</v>
       </c>
       <c r="F32">
-        <v>81659.49916138576</v>
+        <v>81662.1743209885</v>
       </c>
       <c r="G32">
         <v>1989</v>
       </c>
       <c r="H32">
-        <v>1.389838038237137</v>
+        <v>1.389874403678907</v>
       </c>
       <c r="I32">
         <v>-480.3542290039063</v>
       </c>
       <c r="J32">
-        <v>0.28933606790955</v>
+        <v>0.2893436384563619</v>
       </c>
       <c r="K32" t="s">
         <v>44</v>
@@ -1785,31 +1785,31 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>16.87583236079463</v>
+        <v>16.87598697732854</v>
       </c>
       <c r="C33">
-        <v>14.93259678174086</v>
+        <v>14.93245997040295</v>
       </c>
       <c r="D33">
-        <v>2.133228111677265</v>
+        <v>2.133208567200422</v>
       </c>
       <c r="E33">
-        <v>466.5545903109585</v>
+        <v>466.5584520543513</v>
       </c>
       <c r="F33">
-        <v>124288.7749119698</v>
+        <v>124290.9424134305</v>
       </c>
       <c r="G33">
         <v>1989</v>
       </c>
       <c r="H33">
-        <v>0.1687583236079463</v>
+        <v>0.1687598697732854</v>
       </c>
       <c r="I33">
         <v>2.178061798095703</v>
       </c>
       <c r="J33">
-        <v>7.748096209000729</v>
+        <v>7.748167197130658</v>
       </c>
       <c r="K33" t="s">
         <v>44</v>
@@ -1869,10 +1869,10 @@
         <v>1.00604063701263</v>
       </c>
       <c r="F2">
-        <v>2536.3252852842</v>
+        <v>2536.402331147744</v>
       </c>
       <c r="G2">
-        <v>352.5338780898718</v>
+        <v>352.5432269368576</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1892,10 +1892,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F3">
-        <v>17578.13890013053</v>
+        <v>17577.93014825169</v>
       </c>
       <c r="G3">
-        <v>1876.058388047477</v>
+        <v>1876.079947408113</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1915,10 +1915,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F4">
-        <v>905.8277320879109</v>
+        <v>905.8515284167265</v>
       </c>
       <c r="G4">
-        <v>102.2690993687959</v>
+        <v>102.2704992758537</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1938,10 +1938,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F5">
-        <v>2100.659255908095</v>
+        <v>2100.636693742586</v>
       </c>
       <c r="G5">
-        <v>266.1372252208025</v>
+        <v>266.1428077407368</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1961,10 +1961,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F6">
-        <v>2743.93922526841</v>
+        <v>2743.806653336388</v>
       </c>
       <c r="G6">
-        <v>298.4416223742428</v>
+        <v>298.4436399652046</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1984,10 +1984,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F7">
-        <v>3091.094400408224</v>
+        <v>3091.125249863479</v>
       </c>
       <c r="G7">
-        <v>387.4046445941264</v>
+        <v>387.4082524120398</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -2007,10 +2007,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F8">
-        <v>595.89963506841</v>
+        <v>595.9026650965263</v>
       </c>
       <c r="G8">
-        <v>91.01937343852077</v>
+        <v>91.02102624587585</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2030,10 +2030,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F9">
-        <v>231.6647731693357</v>
+        <v>231.6685050337896</v>
       </c>
       <c r="G9">
-        <v>37.40766518017791</v>
+        <v>37.40863388248627</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2053,10 +2053,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F10">
-        <v>2102.209875198344</v>
+        <v>2102.290715553645</v>
       </c>
       <c r="G10">
-        <v>194.277518442707</v>
+        <v>194.2816288486593</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2076,10 +2076,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F11">
-        <v>3000.123140814967</v>
+        <v>3000.210299538441</v>
       </c>
       <c r="G11">
-        <v>430.346149575088</v>
+        <v>430.3577159898251</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2099,10 +2099,10 @@
         <v>1.35675306957708</v>
       </c>
       <c r="F12">
-        <v>840.4597962792304</v>
+        <v>840.4374244025792</v>
       </c>
       <c r="G12">
-        <v>84.78088329602305</v>
+        <v>84.78236180997986</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2122,10 +2122,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F13">
-        <v>1268.785533698076</v>
+        <v>1268.858083394993</v>
       </c>
       <c r="G13">
-        <v>131.0482456814686</v>
+        <v>131.0517963281523</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2145,10 +2145,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F14">
-        <v>7459.24938905485</v>
+        <v>7459.329300344932</v>
       </c>
       <c r="G14">
-        <v>754.0959032942169</v>
+        <v>754.1164570741065</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2168,10 +2168,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F15">
-        <v>235.6321441883392</v>
+        <v>235.6303681044118</v>
       </c>
       <c r="G15">
-        <v>21.43826997241312</v>
+        <v>21.4387574585638</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2191,10 +2191,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F16">
-        <v>1413.223811445337</v>
+        <v>1413.240477161831</v>
       </c>
       <c r="G16">
-        <v>180.1891284442036</v>
+        <v>180.1940799981357</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -2214,10 +2214,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F17">
-        <v>19503.985233106</v>
+        <v>19504.57117026958</v>
       </c>
       <c r="G17">
-        <v>2288.404507727296</v>
+        <v>2288.425076260115</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2237,10 +2237,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F18">
-        <v>1887.674489773472</v>
+        <v>1887.718274991777</v>
       </c>
       <c r="G18">
-        <v>239.8211585977311</v>
+        <v>239.8259730388089</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2260,10 +2260,10 @@
         <v>1.35675306957708</v>
       </c>
       <c r="F19">
-        <v>582.3430045612386</v>
+        <v>582.367056532051</v>
       </c>
       <c r="G19">
-        <v>55.70225045114989</v>
+        <v>55.70407525306173</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2283,10 +2283,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F20">
-        <v>719.5490401151328</v>
+        <v>719.5612838118457</v>
       </c>
       <c r="G20">
-        <v>80.22859160690582</v>
+        <v>80.22992451620128</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2306,10 +2306,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F21">
-        <v>10716.16304696409</v>
+        <v>10716.36477989801</v>
       </c>
       <c r="G21">
-        <v>1332.851816457851</v>
+        <v>1332.866412480471</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2329,10 +2329,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F22">
-        <v>19322.98451931082</v>
+        <v>19335.63265102158</v>
       </c>
       <c r="G22">
-        <v>1690.162962024131</v>
+        <v>1690.131511349707</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2352,10 +2352,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F23">
-        <v>2775.579566284877</v>
+        <v>2775.678166388506</v>
       </c>
       <c r="G23">
-        <v>344.7354205809553</v>
+        <v>344.7408404461129</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2375,10 +2375,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F24">
-        <v>4167.414539511426</v>
+        <v>4167.405415933916</v>
       </c>
       <c r="G24">
-        <v>409.5311721698713</v>
+        <v>409.532172965325</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2398,10 +2398,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F25">
-        <v>1983.271493201893</v>
+        <v>1983.383411294083</v>
       </c>
       <c r="G25">
-        <v>218.9455329810492</v>
+        <v>218.9468740390023</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2421,10 +2421,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F26">
-        <v>8030.714677376631</v>
+        <v>8031.287264077861</v>
       </c>
       <c r="G26">
-        <v>874.9382048163915</v>
+        <v>874.9319344415413</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2444,10 +2444,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F27">
-        <v>687.5183892232208</v>
+        <v>687.5271699426687</v>
       </c>
       <c r="G27">
-        <v>79.88346291615417</v>
+        <v>79.88450128539351</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2467,10 +2467,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F28">
-        <v>679.7745287204093</v>
+        <v>679.8426262179684</v>
       </c>
       <c r="G28">
-        <v>86.04074434781961</v>
+        <v>86.04201381838101</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2490,10 +2490,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F29">
-        <v>310.2423300543782</v>
+        <v>310.2470027402736</v>
       </c>
       <c r="G29">
-        <v>39.07658337855036</v>
+        <v>39.0776221556028</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2513,10 +2513,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F30">
-        <v>3004.969998653595</v>
+        <v>3005.007979421407</v>
       </c>
       <c r="G30">
-        <v>467.2647278470802</v>
+        <v>467.2782096702394</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2536,10 +2536,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F31">
-        <v>1975.293542450192</v>
+        <v>1975.267915966568</v>
       </c>
       <c r="G31">
-        <v>175.1067324180909</v>
+        <v>175.1095623221376</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2559,10 +2559,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F32">
-        <v>2059.427694914544</v>
+        <v>2059.470881619161</v>
       </c>
       <c r="G32">
-        <v>223.4813370337486</v>
+        <v>223.4837391464766</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2582,10 +2582,10 @@
         <v>1.006578947368421</v>
       </c>
       <c r="F33">
-        <v>1963.267245896327</v>
+        <v>1963.33720007824</v>
       </c>
       <c r="G33">
-        <v>251.8043174142737</v>
+        <v>251.8093887372454</v>
       </c>
     </row>
   </sheetData>
@@ -2621,13 +2621,13 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>35.42572289384545</v>
+        <v>35.4262885326072</v>
       </c>
       <c r="C2">
-        <v>0.3542572289384545</v>
+        <v>0.354262885326072</v>
       </c>
       <c r="D2">
-        <v>5.367410921508171</v>
+        <v>5.367496622389322</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
@@ -2638,13 +2638,13 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>34.74690486441447</v>
+        <v>34.74734176259139</v>
       </c>
       <c r="C3">
-        <v>0.3474690486441447</v>
+        <v>0.3474734176259139</v>
       </c>
       <c r="D3">
-        <v>0.08644526197767438</v>
+        <v>0.08644634891700057</v>
       </c>
       <c r="E3" t="s">
         <v>53</v>
@@ -2655,13 +2655,13 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>33.9259451318414</v>
+        <v>33.92606420981944</v>
       </c>
       <c r="C4">
-        <v>0.339259451318414</v>
+        <v>0.3392606420981945</v>
       </c>
       <c r="D4">
-        <v>0.1383406842547132</v>
+        <v>0.138341169821995</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -2672,13 +2672,13 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>32.78771739399839</v>
+        <v>32.78814507822536</v>
       </c>
       <c r="C5">
-        <v>0.3278771739399839</v>
+        <v>0.3278814507822536</v>
       </c>
       <c r="D5">
-        <v>0.308670264686503</v>
+        <v>0.3086742909931212</v>
       </c>
       <c r="E5" t="s">
         <v>53</v>
@@ -2689,13 +2689,13 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>32.37954735576731</v>
+        <v>32.38011844623587</v>
       </c>
       <c r="C6">
-        <v>0.3237954735576731</v>
+        <v>0.3238011844623587</v>
       </c>
       <c r="D6">
-        <v>0.151021007657044</v>
+        <v>0.1510236712723527</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
@@ -2706,13 +2706,13 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>31.78169146795513</v>
+        <v>31.78198761119699</v>
       </c>
       <c r="C7">
-        <v>0.3178169146795513</v>
+        <v>0.3178198761119699</v>
       </c>
       <c r="D7">
-        <v>2.29952184848818</v>
+        <v>2.299543275537008</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
@@ -2723,13 +2723,13 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>31.44654654213385</v>
+        <v>31.44673844578386</v>
       </c>
       <c r="C8">
-        <v>0.3144654654213385</v>
+        <v>0.3144673844578387</v>
       </c>
       <c r="D8">
-        <v>0.4071346820904629</v>
+        <v>0.4071371666440985</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>31.18931185426068</v>
+        <v>31.18966740816405</v>
       </c>
       <c r="C9">
-        <v>0.3118931185426068</v>
+        <v>0.3118966740816405</v>
       </c>
       <c r="D9">
-        <v>1.60852713057399</v>
+        <v>1.608545467564002</v>
       </c>
       <c r="E9" t="s">
         <v>53</v>
@@ -2757,13 +2757,13 @@
         <v>19</v>
       </c>
       <c r="B10">
-        <v>30.71965126342241</v>
+        <v>30.71999165275505</v>
       </c>
       <c r="C10">
-        <v>0.3071965126342242</v>
+        <v>0.3071999165275505</v>
       </c>
       <c r="D10">
-        <v>0.3463314424565727</v>
+        <v>0.3463352799847906</v>
       </c>
       <c r="E10" t="s">
         <v>53</v>
@@ -2774,13 +2774,13 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>30.64016474060952</v>
+        <v>30.64078406676243</v>
       </c>
       <c r="C11">
-        <v>0.3064016474060952</v>
+        <v>0.3064078406676243</v>
       </c>
       <c r="D11">
-        <v>0.5011521744681643</v>
+        <v>0.50116230419987</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
@@ -2791,13 +2791,13 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>30.13623579359739</v>
+        <v>30.13693617866853</v>
       </c>
       <c r="C12">
-        <v>0.3013623579359739</v>
+        <v>0.3013693617866853</v>
       </c>
       <c r="D12">
-        <v>0.01872739301107361</v>
+        <v>0.01872782824746399</v>
       </c>
       <c r="E12" t="s">
         <v>53</v>
@@ -2808,13 +2808,13 @@
         <v>22</v>
       </c>
       <c r="B13">
-        <v>30.12615794086164</v>
+        <v>30.12633269952031</v>
       </c>
       <c r="C13">
-        <v>0.3012615794086164</v>
+        <v>0.3012633269952031</v>
       </c>
       <c r="D13">
-        <v>0.4581963093900052</v>
+        <v>0.4581989673383767</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -2825,13 +2825,13 @@
         <v>23</v>
       </c>
       <c r="B14">
-        <v>29.9263870009361</v>
+        <v>29.92654172458437</v>
       </c>
       <c r="C14">
-        <v>0.2992638700093609</v>
+        <v>0.2992654172458437</v>
       </c>
       <c r="D14">
-        <v>0.91209501881235</v>
+        <v>0.9120997344724423</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
@@ -2842,13 +2842,13 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <v>29.75340933964809</v>
+        <v>29.75407563733193</v>
       </c>
       <c r="C15">
-        <v>0.2975340933964809</v>
+        <v>0.2975407563733193</v>
       </c>
       <c r="D15">
-        <v>0.1042334800646023</v>
+        <v>0.1042358142685771</v>
       </c>
       <c r="E15" t="s">
         <v>53</v>
@@ -2859,13 +2859,13 @@
         <v>25</v>
       </c>
       <c r="B16">
-        <v>28.36780912356847</v>
+        <v>28.36810925585355</v>
       </c>
       <c r="C16">
-        <v>0.2836780912356848</v>
+        <v>0.2836810925585355</v>
       </c>
       <c r="D16">
-        <v>2.032031507937377</v>
+        <v>2.032053006892659</v>
       </c>
       <c r="E16" t="s">
         <v>53</v>
@@ -2876,13 +2876,13 @@
         <v>26</v>
       </c>
       <c r="B17">
-        <v>27.99073492158428</v>
+        <v>27.99084571535667</v>
       </c>
       <c r="C17">
-        <v>0.2799073492158428</v>
+        <v>0.2799084571535668</v>
       </c>
       <c r="D17">
-        <v>0.1737369745932467</v>
+        <v>0.173737662284187</v>
       </c>
       <c r="E17" t="s">
         <v>53</v>
@@ -2893,13 +2893,13 @@
         <v>27</v>
       </c>
       <c r="B18">
-        <v>27.86734463674831</v>
+        <v>27.86762591941144</v>
       </c>
       <c r="C18">
-        <v>0.2786734463674831</v>
+        <v>0.2786762591941144</v>
       </c>
       <c r="D18">
-        <v>0.1818265555804337</v>
+        <v>0.1818283908703922</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
@@ -2910,13 +2910,13 @@
         <v>28</v>
       </c>
       <c r="B19">
-        <v>27.86341678813201</v>
+        <v>27.86331388074051</v>
       </c>
       <c r="C19">
-        <v>0.2786341678813201</v>
+        <v>0.2786331388074051</v>
       </c>
       <c r="D19">
-        <v>0.1086568950192935</v>
+        <v>0.1086564937189892</v>
       </c>
       <c r="E19" t="s">
         <v>53</v>
@@ -2927,13 +2927,13 @@
         <v>29</v>
       </c>
       <c r="B20">
-        <v>26.89127375582474</v>
+        <v>26.89193792180146</v>
       </c>
       <c r="C20">
-        <v>0.2689127375582474</v>
+        <v>0.2689193792180146</v>
       </c>
       <c r="D20">
-        <v>0.05066257550904286</v>
+        <v>0.05066382678331315</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
@@ -2944,13 +2944,13 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>26.58290038321374</v>
+        <v>26.58309521360215</v>
       </c>
       <c r="C21">
-        <v>0.2658290038321374</v>
+        <v>0.2658309521360215</v>
       </c>
       <c r="D21">
-        <v>1.379465515696629</v>
+        <v>1.37947562602313</v>
       </c>
       <c r="E21" t="s">
         <v>53</v>
@@ -2961,13 +2961,13 @@
         <v>31</v>
       </c>
       <c r="B22">
-        <v>25.64371883857743</v>
+        <v>25.64418419898893</v>
       </c>
       <c r="C22">
-        <v>0.2564371883857743</v>
+        <v>0.2564418419898893</v>
       </c>
       <c r="D22">
-        <v>61.9413498516363</v>
+        <v>61.94247391060128</v>
       </c>
       <c r="E22" t="s">
         <v>53</v>
@@ -2978,13 +2978,13 @@
         <v>32</v>
       </c>
       <c r="B23">
-        <v>25.43585740375006</v>
+        <v>25.43645733242202</v>
       </c>
       <c r="C23">
-        <v>0.2543585740375006</v>
+        <v>0.2543645733242202</v>
       </c>
       <c r="D23">
-        <v>0.3170050636327296</v>
+        <v>0.3170125404959551</v>
       </c>
       <c r="E23" t="s">
         <v>53</v>
@@ -2995,13 +2995,13 @@
         <v>33</v>
       </c>
       <c r="B24">
-        <v>25.02641650667483</v>
+        <v>25.02698299990121</v>
       </c>
       <c r="C24">
-        <v>0.2502641650667483</v>
+        <v>0.2502698299990121</v>
       </c>
       <c r="D24">
-        <v>0.7104772301515914</v>
+        <v>0.7104933123796749</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
@@ -3012,13 +3012,13 @@
         <v>34</v>
       </c>
       <c r="B25">
-        <v>24.92259108613786</v>
+        <v>24.92314088746575</v>
       </c>
       <c r="C25">
-        <v>0.2492259108613786</v>
+        <v>0.2492314088746575</v>
       </c>
       <c r="D25">
-        <v>0.4042571437519778</v>
+        <v>0.404266061810043</v>
       </c>
       <c r="E25" t="s">
         <v>53</v>
@@ -3029,13 +3029,13 @@
         <v>35</v>
       </c>
       <c r="B26">
-        <v>24.70927993073185</v>
+        <v>24.70927720225878</v>
       </c>
       <c r="C26">
-        <v>0.2470927993073185</v>
+        <v>0.2470927720225878</v>
       </c>
       <c r="D26">
-        <v>0.5195921667853921</v>
+        <v>0.519592109410461</v>
       </c>
       <c r="E26" t="s">
         <v>53</v>
@@ -3046,13 +3046,13 @@
         <v>36</v>
       </c>
       <c r="B27">
-        <v>24.29880101543948</v>
+        <v>24.29921019445444</v>
       </c>
       <c r="C27">
-        <v>0.2429880101543948</v>
+        <v>0.2429921019445444</v>
       </c>
       <c r="D27">
-        <v>0.1168184849651434</v>
+        <v>0.1168204521269214</v>
       </c>
       <c r="E27" t="s">
         <v>53</v>
@@ -3063,13 +3063,13 @@
         <v>37</v>
       </c>
       <c r="B28">
-        <v>24.1887757609856</v>
+        <v>24.18921788875688</v>
       </c>
       <c r="C28">
-        <v>0.241887757609856</v>
+        <v>0.2418921788875688</v>
       </c>
       <c r="D28">
-        <v>1.94903291640164</v>
+        <v>1.949068541254589</v>
       </c>
       <c r="E28" t="s">
         <v>53</v>
@@ -3080,13 +3080,13 @@
         <v>38</v>
       </c>
       <c r="B29">
-        <v>23.84761048073232</v>
+        <v>23.84808825153807</v>
       </c>
       <c r="C29">
-        <v>0.2384761048073232</v>
+        <v>0.2384808825153807</v>
       </c>
       <c r="D29">
-        <v>0.0839921973257893</v>
+        <v>0.08399388005286275</v>
       </c>
       <c r="E29" t="s">
         <v>53</v>
@@ -3097,13 +3097,13 @@
         <v>39</v>
       </c>
       <c r="B30">
-        <v>22.27320123866313</v>
+        <v>22.27358432658891</v>
       </c>
       <c r="C30">
-        <v>0.2227320123866313</v>
+        <v>0.2227358432658891</v>
       </c>
       <c r="D30">
-        <v>0.4817840397564462</v>
+        <v>0.4817923262010612</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -3114,13 +3114,13 @@
         <v>40</v>
       </c>
       <c r="B31">
-        <v>21.84782342798901</v>
+        <v>21.8484880608005</v>
       </c>
       <c r="C31">
-        <v>0.2184782342798901</v>
+        <v>0.218484880608005</v>
       </c>
       <c r="D31">
-        <v>0.4857028129768797</v>
+        <v>0.4857175885460434</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
@@ -3131,13 +3131,13 @@
         <v>41</v>
       </c>
       <c r="B32">
-        <v>17.37297547796422</v>
+        <v>17.37343004598634</v>
       </c>
       <c r="C32">
-        <v>1.389838038237137</v>
+        <v>1.389874403678907</v>
       </c>
       <c r="D32">
-        <v>0.28933606790955</v>
+        <v>0.2893436384563619</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
@@ -3148,13 +3148,13 @@
         <v>42</v>
       </c>
       <c r="B33">
-        <v>16.87583236079463</v>
+        <v>16.87598697732854</v>
       </c>
       <c r="C33">
-        <v>0.1687583236079463</v>
+        <v>0.1687598697732854</v>
       </c>
       <c r="D33">
-        <v>7.748096209000729</v>
+        <v>7.748167197130658</v>
       </c>
       <c r="E33" t="s">
         <v>53</v>
@@ -3217,16 +3217,16 @@
         <v>7.696506550218341</v>
       </c>
       <c r="F2">
-        <v>1585.009293976932</v>
+        <v>1585.025799931751</v>
       </c>
       <c r="G2">
-        <v>5647.092381292968</v>
+        <v>5647.136898567488</v>
       </c>
       <c r="H2">
-        <v>-3561.013608007631</v>
+        <v>-3561.065207074943</v>
       </c>
       <c r="I2">
-        <v>9208.105989300599</v>
+        <v>9208.202105642431</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -3246,16 +3246,16 @@
         <v>-1.206636500754148</v>
       </c>
       <c r="F3">
-        <v>8778.177991933831</v>
+        <v>8778.200189233081</v>
       </c>
       <c r="G3">
-        <v>22104.53632504945</v>
+        <v>22104.83779177294</v>
       </c>
       <c r="H3">
-        <v>-22303.62506864941</v>
+        <v>-22303.67235990087</v>
       </c>
       <c r="I3">
-        <v>44408.16139369886</v>
+        <v>44408.51015167381</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3275,16 +3275,16 @@
         <v>3.418803418803419</v>
       </c>
       <c r="F4">
-        <v>489.2715518923671</v>
+        <v>489.2762586484038</v>
       </c>
       <c r="G4">
-        <v>1270.118216005645</v>
+        <v>1270.180361546758</v>
       </c>
       <c r="H4">
-        <v>-1225.901388765083</v>
+        <v>-1225.883814584021</v>
       </c>
       <c r="I4">
-        <v>2496.019604770727</v>
+        <v>2496.064176130779</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3292,28 +3292,28 @@
         <v>38</v>
       </c>
       <c r="B5">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="C5">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="D5">
         <v>13</v>
       </c>
       <c r="E5">
-        <v>8.949220713926596</v>
+        <v>8.848667672197084</v>
       </c>
       <c r="F5">
-        <v>1613.233263281603</v>
+        <v>1613.229822907522</v>
       </c>
       <c r="G5">
-        <v>6330.998957244219</v>
+        <v>6330.898128545586</v>
       </c>
       <c r="H5">
-        <v>-3576.945365825717</v>
+        <v>-3577.041396179164</v>
       </c>
       <c r="I5">
-        <v>9907.944323069936</v>
+        <v>9907.939524724748</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -3333,16 +3333,16 @@
         <v>10.25641025641026</v>
       </c>
       <c r="F6">
-        <v>1552.29101435198</v>
+        <v>1552.291726891378</v>
       </c>
       <c r="G6">
-        <v>5874.361641401896</v>
+        <v>5874.286450271725</v>
       </c>
       <c r="H6">
-        <v>-3637.012817908294</v>
+        <v>-3636.957445509937</v>
       </c>
       <c r="I6">
-        <v>9511.374459310191</v>
+        <v>9511.243895781661</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3362,16 +3362,16 @@
         <v>3.418803418803419</v>
       </c>
       <c r="F7">
-        <v>1717.031286571692</v>
+        <v>1717.041584941885</v>
       </c>
       <c r="G7">
-        <v>4632.636963088779</v>
+        <v>4632.688156659575</v>
       </c>
       <c r="H7">
-        <v>-4241.471664834472</v>
+        <v>-4241.509598365773</v>
       </c>
       <c r="I7">
-        <v>8874.108627923251</v>
+        <v>8874.197755025347</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3391,16 +3391,16 @@
         <v>2.61437908496732</v>
       </c>
       <c r="F8">
-        <v>452.2598470245931</v>
+        <v>452.2632627296833</v>
       </c>
       <c r="G8">
-        <v>1367.273490200258</v>
+        <v>1367.278418319077</v>
       </c>
       <c r="H8">
-        <v>-1094.147509371898</v>
+        <v>-1094.164469151355</v>
       </c>
       <c r="I8">
-        <v>2461.420999572157</v>
+        <v>2461.442887470433</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3420,16 +3420,16 @@
         <v>2.413273001508296</v>
       </c>
       <c r="F9">
-        <v>161.2664368512376</v>
+        <v>161.2680468440302</v>
       </c>
       <c r="G9">
-        <v>469.4436033030745</v>
+        <v>469.4503204731368</v>
       </c>
       <c r="H9">
-        <v>-389.769584041486</v>
+        <v>-389.7725146378894</v>
       </c>
       <c r="I9">
-        <v>859.2131873445605</v>
+        <v>859.2228351110261</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3449,16 +3449,16 @@
         <v>13.27300150829563</v>
       </c>
       <c r="F10">
-        <v>1155.693789803296</v>
+        <v>1155.697887117685</v>
       </c>
       <c r="G10">
-        <v>6260.359337443201</v>
+        <v>6260.36419717347</v>
       </c>
       <c r="H10">
-        <v>-1710.401176537438</v>
+        <v>-1710.402576191186</v>
       </c>
       <c r="I10">
-        <v>7970.760513980638</v>
+        <v>7970.766773364656</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3478,16 +3478,16 @@
         <v>7.239819004524888</v>
       </c>
       <c r="F11">
-        <v>2160.661860351579</v>
+        <v>2160.670086176731</v>
       </c>
       <c r="G11">
-        <v>7985.426603950807</v>
+        <v>7985.496193346811</v>
       </c>
       <c r="H11">
-        <v>-4162.32250779399</v>
+        <v>-4162.372228579294</v>
       </c>
       <c r="I11">
-        <v>12147.7491117448</v>
+        <v>12147.8684219261</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3507,16 +3507,16 @@
         <v>11.16138763197587</v>
       </c>
       <c r="F12">
-        <v>565.7810746915433</v>
+        <v>565.7850821825238</v>
       </c>
       <c r="G12">
-        <v>1482.194988097972</v>
+        <v>1482.182457854824</v>
       </c>
       <c r="H12">
-        <v>-1209.557057933266</v>
+        <v>-1209.543769988299</v>
       </c>
       <c r="I12">
-        <v>2691.752046031238</v>
+        <v>2691.726227843123</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3536,16 +3536,16 @@
         <v>12.56913021618904</v>
       </c>
       <c r="F13">
-        <v>687.5088571755219</v>
+        <v>687.5211870764737</v>
       </c>
       <c r="G13">
-        <v>2785.462298799501</v>
+        <v>2785.603949950623</v>
       </c>
       <c r="H13">
-        <v>-1305.248720480039</v>
+        <v>-1305.261156522097</v>
       </c>
       <c r="I13">
-        <v>4090.71101927954</v>
+        <v>4090.86510647272</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -3565,16 +3565,16 @@
         <v>6.334841628959276</v>
       </c>
       <c r="F14">
-        <v>4363.65315664418</v>
+        <v>4363.672016463152</v>
       </c>
       <c r="G14">
-        <v>14065.5896457944</v>
+        <v>14065.62729302499</v>
       </c>
       <c r="H14">
-        <v>-11448.92569371443</v>
+        <v>-11448.93927226972</v>
       </c>
       <c r="I14">
-        <v>25514.51533950883</v>
+        <v>25514.56656529471</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -3594,16 +3594,16 @@
         <v>13.77576671694319</v>
       </c>
       <c r="F15">
-        <v>137.438110803502</v>
+        <v>137.4389760106025</v>
       </c>
       <c r="G15">
-        <v>655.8597916156754</v>
+        <v>655.8708037574447</v>
       </c>
       <c r="H15">
-        <v>-248.0128773374849</v>
+        <v>-248.0109062764381</v>
       </c>
       <c r="I15">
-        <v>903.8726689531602</v>
+        <v>903.8817100338829</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -3623,16 +3623,16 @@
         <v>5.530417295123177</v>
       </c>
       <c r="F16">
-        <v>926.827847227338</v>
+        <v>926.8328146771922</v>
       </c>
       <c r="G16">
-        <v>2951.36214092612</v>
+        <v>2951.384986255012</v>
       </c>
       <c r="H16">
-        <v>-2006.211329380025</v>
+        <v>-2006.249049444046</v>
       </c>
       <c r="I16">
-        <v>4957.573470306144</v>
+        <v>4957.634035699059</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -3652,16 +3652,16 @@
         <v>7.642031171442937</v>
       </c>
       <c r="F17">
-        <v>12406.43304259666</v>
+        <v>12406.62334235131</v>
       </c>
       <c r="G17">
-        <v>49348.67379146895</v>
+        <v>49348.94280141697</v>
       </c>
       <c r="H17">
-        <v>-26081.95127362661</v>
+        <v>-26082.07072699111</v>
       </c>
       <c r="I17">
-        <v>75430.62506509556</v>
+        <v>75431.01352840808</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3681,16 +3681,16 @@
         <v>4.323780794369029</v>
       </c>
       <c r="F18">
-        <v>1066.107729250353</v>
+        <v>1066.115304949652</v>
       </c>
       <c r="G18">
-        <v>2740.147639785808</v>
+        <v>2740.186193641149</v>
       </c>
       <c r="H18">
-        <v>-2876.596390259504</v>
+        <v>-2876.622427607036</v>
       </c>
       <c r="I18">
-        <v>5616.744030045312</v>
+        <v>5616.808621248185</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3710,16 +3710,16 @@
         <v>12.36802413273002</v>
       </c>
       <c r="F19">
-        <v>286.7246322488215</v>
+        <v>286.7279738576349</v>
       </c>
       <c r="G19">
-        <v>913.1242359262289</v>
+        <v>913.1446517792563</v>
       </c>
       <c r="H19">
-        <v>-365.9213364631102</v>
+        <v>-365.9250648218328</v>
       </c>
       <c r="I19">
-        <v>1279.045572389339</v>
+        <v>1279.069716601089</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -3739,16 +3739,16 @@
         <v>4.927099044746104</v>
       </c>
       <c r="F20">
-        <v>410.1719105721406</v>
+        <v>410.1745745186069</v>
       </c>
       <c r="G20">
-        <v>1183.026220440097</v>
+        <v>1183.038385926147</v>
       </c>
       <c r="H20">
-        <v>-798.6481471121839</v>
+        <v>-798.647477561165</v>
       </c>
       <c r="I20">
-        <v>1981.674367552281</v>
+        <v>1981.685863487312</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -3768,16 +3768,16 @@
         <v>4.122674710910005</v>
       </c>
       <c r="F21">
-        <v>6352.937380486177</v>
+        <v>6352.983400664354</v>
       </c>
       <c r="G21">
-        <v>17096.5200419668</v>
+        <v>17097.2047107423</v>
       </c>
       <c r="H21">
-        <v>-15706.48856670671</v>
+        <v>-15706.52945310314</v>
       </c>
       <c r="I21">
-        <v>32803.00860867351</v>
+        <v>32803.73416384545</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -3797,16 +3797,16 @@
         <v>5.832076420311714</v>
       </c>
       <c r="F22">
-        <v>7846.13566433406</v>
+        <v>7845.788790281837</v>
       </c>
       <c r="G22">
-        <v>27843.83666164801</v>
+        <v>27844.23444956758</v>
       </c>
       <c r="H22">
-        <v>-24637.97202697679</v>
+        <v>-24638.44247219026</v>
       </c>
       <c r="I22">
-        <v>52481.8086886248</v>
+        <v>52482.67692175784</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -3826,16 +3826,16 @@
         <v>5.329311211664153</v>
       </c>
       <c r="F23">
-        <v>1740.782286402502</v>
+        <v>1740.801085607834</v>
       </c>
       <c r="G23">
-        <v>5998.138664117503</v>
+        <v>5998.142018885897</v>
       </c>
       <c r="H23">
-        <v>-4074.417671189571</v>
+        <v>-4074.48668880604</v>
       </c>
       <c r="I23">
-        <v>10072.55633530707</v>
+        <v>10072.62870769194</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -3855,16 +3855,16 @@
         <v>2.61437908496732</v>
       </c>
       <c r="F24">
-        <v>2006.636464335872</v>
+        <v>2006.637178857844</v>
       </c>
       <c r="G24">
-        <v>6423.42976944728</v>
+        <v>6423.536492173555</v>
       </c>
       <c r="H24">
-        <v>-7169.941195106214</v>
+        <v>-7169.882054025652</v>
       </c>
       <c r="I24">
-        <v>13593.37096455349</v>
+        <v>13593.41854619921</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -3884,16 +3884,16 @@
         <v>9.854198089492208</v>
       </c>
       <c r="F25">
-        <v>1142.582012013234</v>
+        <v>1142.580909994277</v>
       </c>
       <c r="G25">
-        <v>4707.481513579053</v>
+        <v>4707.417489024808</v>
       </c>
       <c r="H25">
-        <v>-2076.174657615929</v>
+        <v>-2076.180322922512</v>
       </c>
       <c r="I25">
-        <v>6783.656171194983</v>
+        <v>6783.597811947319</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -3913,16 +3913,16 @@
         <v>12.16691804927099</v>
       </c>
       <c r="F26">
-        <v>4419.687736443002</v>
+        <v>4419.56955575861</v>
       </c>
       <c r="G26">
-        <v>15255.18736558071</v>
+        <v>15254.4191036076</v>
       </c>
       <c r="H26">
-        <v>-9917.756211744476</v>
+        <v>-9916.649032251413</v>
       </c>
       <c r="I26">
-        <v>25172.94357732519</v>
+        <v>25171.06813585901</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -3942,16 +3942,16 @@
         <v>0.5027652086475616</v>
       </c>
       <c r="F27">
-        <v>377.5852281798587</v>
+        <v>377.5856651064173</v>
       </c>
       <c r="G27">
-        <v>891.5954418183245</v>
+        <v>891.5905995477046</v>
       </c>
       <c r="H27">
-        <v>-941.1139484531096</v>
+        <v>-941.1080256073105</v>
       </c>
       <c r="I27">
-        <v>1832.709390271434</v>
+        <v>1832.698625155015</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3971,16 +3971,16 @@
         <v>8.848667672197084</v>
       </c>
       <c r="F28">
-        <v>554.8874634674929</v>
+        <v>554.8787862868569</v>
       </c>
       <c r="G28">
-        <v>1926.177013913394</v>
+        <v>1926.151721809492</v>
       </c>
       <c r="H28">
-        <v>-998.5254631997432</v>
+        <v>-998.4060836942111</v>
       </c>
       <c r="I28">
-        <v>2924.702477113137</v>
+        <v>2924.557805503703</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -4000,16 +4000,16 @@
         <v>5.932629462041226</v>
       </c>
       <c r="F29">
-        <v>233.8591731048626</v>
+        <v>233.8599902061802</v>
       </c>
       <c r="G29">
-        <v>841.6696479396144</v>
+        <v>841.6727524128535</v>
       </c>
       <c r="H29">
-        <v>-512.8142704891862</v>
+        <v>-512.8348065028458</v>
       </c>
       <c r="I29">
-        <v>1354.483918428801</v>
+        <v>1354.507558915699</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -4029,16 +4029,16 @@
         <v>11.36249371543489</v>
       </c>
       <c r="F30">
-        <v>2494.472949303092</v>
+        <v>2494.484020307435</v>
       </c>
       <c r="G30">
-        <v>9347.542840980799</v>
+        <v>9347.559418315544</v>
       </c>
       <c r="H30">
-        <v>-4110.045844454616</v>
+        <v>-4110.055687214123</v>
       </c>
       <c r="I30">
-        <v>13457.58868543541</v>
+        <v>13457.61510552967</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -4058,16 +4058,16 @@
         <v>7.440925087983912</v>
       </c>
       <c r="F31">
-        <v>1109.858721229039</v>
+        <v>1109.852201152301</v>
       </c>
       <c r="G31">
-        <v>4654.141362070584</v>
+        <v>4653.798090849013</v>
       </c>
       <c r="H31">
-        <v>-2959.446948303254</v>
+        <v>-2959.756542688187</v>
       </c>
       <c r="I31">
-        <v>7613.588310373838</v>
+        <v>7613.554633537199</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -4087,16 +4087,16 @@
         <v>11.76470588235294</v>
       </c>
       <c r="F32">
-        <v>1319.260478011091</v>
+        <v>1319.257387824551</v>
       </c>
       <c r="G32">
-        <v>5108.877694986662</v>
+        <v>5109.006818882287</v>
       </c>
       <c r="H32">
-        <v>-2727.577603954907</v>
+        <v>-2727.589782363752</v>
       </c>
       <c r="I32">
-        <v>7836.45529894157</v>
+        <v>7836.596601246039</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -4104,28 +4104,28 @@
         <v>14</v>
       </c>
       <c r="B33">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="C33">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="D33">
         <v>13</v>
       </c>
       <c r="E33">
-        <v>2.61437908496732</v>
+        <v>2.513826043237808</v>
       </c>
       <c r="F33">
-        <v>1174.727185976258</v>
+        <v>1174.737714418364</v>
       </c>
       <c r="G33">
-        <v>3493.573101921227</v>
+        <v>3493.591262761759</v>
       </c>
       <c r="H33">
-        <v>-2663.491714014139</v>
+        <v>-2663.541733323611</v>
       </c>
       <c r="I33">
-        <v>6157.064815935366</v>
+        <v>6157.132996085369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>